<commit_message>
Registra la revision AIC completa y aplica el criterio de aptitud a MET y CMA
- AIC: revision manual de los 508 candidatos con el criterio de estructura
  observable (228 principal, 124 secundario, 156 descartados); los workbooks
  conservan el motivo original del revisor y lo enriquecen con el analisis de
  imagen.
- MET y CMA: la validacion ciega de 40 imagenes dio kappa 0,56 (< 0,6), por lo
  que no se aplican las sugerencias del modelo. Solo se aplican las reglas
  aprobadas (49 cambios: fotografia monocroma, plumaria, periodo, resolucion e
  imagen inexistente) y las 9 decisiones de la validacion; MET:307683 queda en
  revisar porque su anotacion contradice su motivo.
- config/corpus.toml registra cada cambio con su fecha y motivo.
</commit_message>
<xml_diff>
--- a/data/metadata/cma_revision_manual_v2.xlsx
+++ b/data/metadata/cma_revision_manual_v2.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resumen" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="revision_cma_v2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="listas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="resumen" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="revision_cma_v2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="listas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'revision_cma_v2'!$A$1:$Z$147</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'revision_cma_v2'!$A$1:$AD$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -48,7 +48,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +65,11 @@
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007F6000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -79,7 +84,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -91,6 +96,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -552,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z147"/>
+  <dimension ref="A1:AD147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -581,6 +589,10 @@
     <col width="36" customWidth="1" min="24" max="24"/>
     <col width="34" customWidth="1" min="25" max="25"/>
     <col width="24" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="70" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -712,6 +724,26 @@
       <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>origen_curacion</t>
+        </is>
+      </c>
+      <c r="AA1" s="7" t="inlineStr">
+        <is>
+          <t>puntaje_aptitud</t>
+        </is>
+      </c>
+      <c r="AB1" s="7" t="inlineStr">
+        <is>
+          <t>banda_sugerida</t>
+        </is>
+      </c>
+      <c r="AC1" s="7" t="inlineStr">
+        <is>
+          <t>motivo_banda</t>
+        </is>
+      </c>
+      <c r="AD1" s="7" t="inlineStr">
+        <is>
+          <t>justificacion_aptitud</t>
         </is>
       </c>
     </row>
@@ -802,6 +834,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA2" s="4" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="AB2" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC2" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD2" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,22; textil de 1576 px de lado); colores identificables (probabilidad 0,73; 3 colores claramente distintos, 2 tonos, colorido 25); formas visibles (probabilidad 0,72; bordes cromáticos en el 30 % del textil); textil incompleto (probabilidad 0,33; compacidad 0,67, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 56.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -890,6 +940,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA3" s="4" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="AB3" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC3" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD3" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,79; textil de 2752 px de lado); colores identificables (probabilidad 0,79; 1 color claramente distinto, 0 tonos, colorido 18); formas visibles (probabilidad 0,89; bordes cromáticos en el 23 % del textil); completitud incierta (probabilidad 0,64; compacidad 0,95, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 61.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -978,6 +1046,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA4" s="4" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="AB4" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC4" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD4" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,60; textil de 2024 px de lado); colores parcialmente identificables (probabilidad 0,59; 2 colores claramente distintos, 1 tono, colorido 15); formas parcialmente visibles (probabilidad 0,63; bordes cromáticos en el 13 % del textil); textil incompleto (probabilidad 0,29; compacidad 0,54, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 45.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1066,6 +1152,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA5" s="4" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="AB5" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC5" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD5" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,40; textil de 2152 px de lado); colores identificables (probabilidad 0,81; 1 color claramente distinto, 1 tono, colorido 17); formas visibles (probabilidad 0,87; bordes cromáticos en el 5 % del textil); textil completo (probabilidad 0,71; compacidad 0,92, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 61.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1154,6 +1258,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA6" s="4" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="AB6" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC6" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD6" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,60; textil de 1360 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 38); formas visibles (probabilidad 0,99; bordes cromáticos en el 49 % del textil); textil completo (probabilidad 0,97; compacidad 0,90, lagunas 0,0 %); estructura repetitiva. Puntaje 88 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1242,6 +1364,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA7" s="4" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="AB7" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC7" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD7" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,17; textil de 2199 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 35); formas visibles (probabilidad 0,99; bordes cromáticos en el 52 % del textil); textil completo (probabilidad 0,84; compacidad 0,76, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 85 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1330,6 +1470,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA8" s="4" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="AB8" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC8" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD8" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,14; textil de 1404 px de lado); colores identificables (probabilidad 0,96; 3 colores claramente distintos, 3 tonos, colorido 36); formas visibles (probabilidad 0,93; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,82; compacidad 0,76, lagunas 0,0 %); estructura repetitiva. Puntaje 82 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1418,6 +1576,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA9" s="4" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="AB9" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC9" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD9" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,15; textil de 1375 px de lado); colores identificables (probabilidad 0,94; 3 colores claramente distintos, 2 tonos, colorido 36); formas visibles (probabilidad 0,89; bordes cromáticos en el 45 % del textil); textil completo (probabilidad 0,79; compacidad 0,78, lagunas 0,0 %); estructura repetitiva. Puntaje 78 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1506,6 +1682,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA10" s="4" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="AB10" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC10" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD10" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,10; textil de 1325 px de lado); colores identificables (probabilidad 0,94; 2 colores claramente distintos, 3 tonos, colorido 34); formas visibles (probabilidad 0,91; bordes cromáticos en el 49 % del textil); textil completo (probabilidad 0,78; compacidad 0,73, lagunas 0,2 %); estructura repetitiva. Puntaje 81 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1594,6 +1788,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA11" s="4" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="AB11" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC11" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD11" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,13; textil de 1297 px de lado); colores identificables (probabilidad 0,95; 3 colores claramente distintos, 3 tonos, colorido 37); formas visibles (probabilidad 0,92; bordes cromáticos en el 52 % del textil); textil completo (probabilidad 0,80; compacidad 0,72, lagunas 0,0 %); estructura repetitiva. Puntaje 83 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1682,6 +1894,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA12" s="4" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="AB12" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC12" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD12" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,27; textil de 2350 px de lado); colores identificables (probabilidad 0,97; 3 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,98; bordes cromáticos en el 41 % del textil); completitud incierta (probabilidad 0,58; compacidad 0,93, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 72.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1770,6 +2000,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA13" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="AB13" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC13" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD13" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,27; textil de 1544 px de lado); colores identificables (probabilidad 0,95; 3 colores claramente distintos, 3 tonos, colorido 41); formas visibles (probabilidad 0,94; bordes cromáticos en el 40 % del textil); completitud incierta (probabilidad 0,69; compacidad 0,92, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 75.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1858,6 +2106,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA14" s="4" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="AB14" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC14" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD14" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,24; textil de 1551 px de lado); colores identificables (probabilidad 0,88; 3 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,86; bordes cromáticos en el 40 % del textil); completitud incierta (probabilidad 0,56; compacidad 0,86, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 67.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1946,6 +2212,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA15" s="4" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="AB15" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC15" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD15" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,31; textil de 1549 px de lado); colores identificables (probabilidad 0,84; 3 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,83; bordes cromáticos en el 38 % del textil); completitud incierta (probabilidad 0,48; compacidad 0,85, lagunas 0,1 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -2034,6 +2318,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA16" s="4" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="AB16" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC16" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD16" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,88; textil de 1702 px de lado); colores identificables (probabilidad 0,87; 2 colores claramente distintos, 2 tonos, colorido 29); formas visibles (probabilidad 0,91; bordes cromáticos en el 26 % del textil); textil incompleto (probabilidad 0,26; compacidad 0,74, lagunas 2,2 %, el título dice «fragment»); estructura repetitiva. Puntaje 63.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -2122,6 +2424,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA17" s="4" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="AB17" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC17" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD17" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,97; textil de 2643 px de lado); colores identificables (probabilidad 0,90; 1 color claramente distinto, 3 tonos, colorido 27); formas visibles (probabilidad 0,94; bordes cromáticos en el 18 % del textil); textil completo (probabilidad 0,72; compacidad 0,87, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 67.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -2210,6 +2530,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA18" s="4" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="AB18" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC18" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD18" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,81; textil de 2462 px de lado); colores identificables (probabilidad 0,91; 2 colores claramente distintos, 3 tonos, colorido 26); formas visibles (probabilidad 0,92; bordes cromáticos en el 33 % del textil); textil completo (probabilidad 0,77; compacidad 0,74, lagunas 0,2 %); estructura no evidente. Puntaje 72.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -2298,6 +2636,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA19" s="4" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="AB19" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC19" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD19" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,84; textil de 2697 px de lado); colores identificables (probabilidad 0,85; 2 colores claramente distintos, 1 tono, colorido 15); formas visibles (probabilidad 0,90; bordes cromáticos en el 19 % del textil); textil completo (probabilidad 0,72; compacidad 0,90, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 64.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -2386,6 +2742,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA20" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="AB20" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC20" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD20" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,45; textil de 1607 px de lado); colores identificables (probabilidad 0,99; 1 color claramente distinto, 2 tonos, colorido 19); formas visibles (probabilidad 0,99; bordes cromáticos en el 21 % del textil); textil completo (probabilidad 0,97; compacidad 0,95, lagunas 0,0 %); estructura repetitiva. Puntaje 76.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2474,6 +2848,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA21" s="4" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="AB21" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC21" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD21" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,16; textil de 2151 px de lado); colores parcialmente identificables (probabilidad 0,68; 2 colores claramente distintos, 3 tonos, colorido 38); formas visibles (probabilidad 0,70; bordes cromáticos en el 22 % del textil); textil incompleto (probabilidad 0,28; compacidad 0,67, lagunas 0,2 %, el título dice «fragment»); estructura no evidente. Puntaje 50.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2562,6 +2954,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA22" s="4" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="AB22" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC22" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD22" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 0,96; textil de 2262 px de lado); colores identificables (probabilidad 0,96; 3 colores claramente distintos, 3 tonos, colorido 51); formas visibles (probabilidad 0,95; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,85; compacidad 0,89, lagunas 3,9 %); estructura no evidente. Puntaje 78 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2650,6 +3060,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA23" s="4" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="AB23" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC23" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD23" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,34; textil de 2152 px de lado); colores parcialmente identificables (probabilidad 0,66; 3 colores claramente distintos, 3 tonos, colorido 21); formas visibles (probabilidad 0,89; bordes cromáticos en el 40 % del textil); textil incompleto (probabilidad 0,19; compacidad 0,90, lagunas 35,4 %); estructura no evidente. Puntaje 77 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2738,6 +3166,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA24" s="4" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="AB24" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC24" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD24" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,49; textil de 1786 px de lado); colores identificables (probabilidad 0,84; 1 color claramente distinto, 2 tonos, colorido 36); formas visibles (probabilidad 0,83; bordes cromáticos en el 21 % del textil); textil completo (probabilidad 0,83; compacidad 0,67, lagunas 0,5 %); estructura repetitiva. Puntaje 65.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2826,6 +3272,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA25" s="4" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="AB25" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC25" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD25" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 0,94; textil de 2036 px de lado); colores identificables (probabilidad 0,74; 3 colores claramente distintos, 2 tonos, colorido 34); formas visibles (probabilidad 0,77; bordes cromáticos en el 23 % del textil); textil incompleto (probabilidad 0,37; compacidad 0,88, lagunas 1,7 %, el título dice «fragment»); estructura no evidente. Puntaje 56.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2914,6 +3378,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA26" s="4" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="AB26" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC26" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD26" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,46; textil de 1769 px de lado); colores identificables (probabilidad 0,98; 1 color claramente distinto, 1 tono, colorido 19); formas visibles (probabilidad 0,98; bordes cromáticos en el 44 % del textil); textil completo (probabilidad 0,98; compacidad 0,95, lagunas 0,0 %); estructura no evidente. Puntaje 79 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -3002,6 +3484,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA27" s="4" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="AB27" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC27" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD27" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,01; textil de 2301 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 2 tonos, colorido 19); formas visibles (probabilidad 0,97; bordes cromáticos en el 20 % del textil); textil completo (probabilidad 0,88; toma cerrada, el contorno de la pieza no se ve); estructura repetitiva y simétrica. Puntaje 80 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -3090,6 +3590,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA28" s="4" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="AB28" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC28" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD28" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,18; textil de 3112 px de lado); colores identificables (probabilidad 0,97; 2 colores claramente distintos, 3 tonos, colorido 23); formas visibles (probabilidad 0,98; bordes cromáticos en el 15 % del textil); textil completo (probabilidad 0,91; compacidad 0,97, lagunas 0,0 %); estructura repetitiva. Puntaje 72.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -3178,6 +3696,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA29" s="4" t="n">
+        <v>79.7</v>
+      </c>
+      <c r="AB29" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC29" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD29" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 1,00; textil de 1289 px de lado); colores identificables (probabilidad 0,98; 5 colores claramente distintos, 3 tonos, colorido 65); formas visibles (probabilidad 0,96; bordes cromáticos en el 39 % del textil); textil completo (probabilidad 0,80; compacidad 0,87, lagunas 0,0 %); estructura simétrica. Puntaje 80 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -3266,6 +3802,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA30" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="AB30" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC30" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD30" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,04; textil de 1962 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 0 tonos, colorido 11); formas visibles (probabilidad 0,97; bordes cromáticos en el 6 % del textil); textil completo (probabilidad 0,92; compacidad 0,98, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 71.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -3354,6 +3908,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA31" s="4" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="AB31" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC31" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD31" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,48; textil de 1083 px de lado); colores identificables (probabilidad 0,73; 2 colores claramente distintos, 1 tono, colorido 53); formas parcialmente visibles (probabilidad 0,54; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,71; compacidad 0,51, lagunas 0,0 %); estructura no evidente. Puntaje 52.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -3442,6 +4014,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA32" s="4" t="n">
+        <v>55.9</v>
+      </c>
+      <c r="AB32" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC32" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD32" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,81; textil de 1352 px de lado); colores identificables (probabilidad 0,79; 2 colores claramente distintos, 1 tono, colorido 56); formas parcialmente visibles (probabilidad 0,66; bordes cromáticos en el 15 % del textil); textil completo (probabilidad 0,81; compacidad 0,63, lagunas 0,0 %); estructura no evidente. Puntaje 56.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -3530,6 +4120,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA33" s="4" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="AB33" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC33" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD33" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,62; textil de 2287 px de lado); colores identificables (probabilidad 0,89; 1 color claramente distinto, 2 tonos, colorido 28); formas visibles (probabilidad 0,92; bordes cromáticos en el 22 % del textil); textil completo (probabilidad 0,83; compacidad 0,82, lagunas 4,9 %); estructura no evidente. Puntaje 69.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -3618,6 +4226,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA34" s="4" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="AB34" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC34" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD34" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,35; textil de 1651 px de lado); colores identificables (probabilidad 0,86; 1 color claramente distinto, 2 tonos, colorido 25); formas visibles (probabilidad 0,90; bordes cromáticos en el 26 % del textil); textil completo (probabilidad 0,76; compacidad 0,80, lagunas 11,0 %); estructura no evidente. Puntaje 72.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -3706,6 +4332,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA35" s="4" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="AB35" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC35" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD35" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,87; textil de 1596 px de lado); colores identificables (probabilidad 0,78; 2 colores claramente distintos, 2 tonos, colorido 36); formas visibles (probabilidad 0,76; bordes cromáticos en el 24 % del textil); completitud incierta (probabilidad 0,62; compacidad 0,63, lagunas 6,2 %); estructura no evidente. Puntaje 63.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -3794,6 +4438,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA36" s="4" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="AB36" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC36" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD36" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,48; textil de 2034 px de lado); colores identificables (probabilidad 0,85; 3 colores claramente distintos, 2 tonos, colorido 46); formas visibles (probabilidad 0,85; bordes cromáticos en el 22 % del textil); textil completo (probabilidad 0,71; compacidad 0,80, lagunas 7,7 %); estructura no evidente. Puntaje 69.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -3882,6 +4544,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA37" s="4" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="AB37" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC37" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD37" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,71; textil de 1980 px de lado); colores identificables (probabilidad 0,87; 2 colores claramente distintos, 1 tono, colorido 25); formas visibles (probabilidad 0,87; bordes cromáticos en el 26 % del textil); textil completo (probabilidad 0,81; compacidad 0,74, lagunas 1,8 %); estructura no evidente. Puntaje 67.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -3970,6 +4650,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA38" s="4" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="AB38" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC38" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD38" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,92; textil de 1928 px de lado); colores identificables (probabilidad 0,77; 2 colores claramente distintos, 2 tonos, colorido 34); formas visibles (probabilidad 0,81; bordes cromáticos en el 19 % del textil); completitud incierta (probabilidad 0,62; compacidad 0,76, lagunas 8,5 %); estructura no evidente. Puntaje 64.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -4058,6 +4756,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA39" s="4" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="AB39" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC39" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD39" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,99; textil de 1810 px de lado); colores identificables (probabilidad 0,89; 2 colores claramente distintos, 2 tonos, colorido 39); formas visibles (probabilidad 0,86; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,82; compacidad 0,69, lagunas 1,1 %); estructura no evidente. Puntaje 69.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -4146,6 +4862,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA40" s="4" t="n">
+        <v>65.3</v>
+      </c>
+      <c r="AB40" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC40" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD40" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,28; textil de 1821 px de lado); colores identificables (probabilidad 0,72; 2 colores claramente distintos, 1 tono, colorido 27); formas visibles (probabilidad 0,84; bordes cromáticos en el 10 % del textil); completitud incierta (probabilidad 0,60; compacidad 0,81, lagunas 23,2 %); estructura no evidente. Puntaje 65.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -4234,6 +4968,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA41" s="4" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="AB41" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC41" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD41" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,62; textil de 2116 px de lado); colores identificables (probabilidad 0,92; 1 color claramente distinto, 2 tonos, colorido 20); formas visibles (probabilidad 0,93; bordes cromáticos en el 34 % del textil); textil completo (probabilidad 0,85; compacidad 0,74, lagunas 0,0 %); estructura no evidente. Puntaje 73.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -4322,6 +5074,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA42" s="4" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="AB42" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC42" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD42" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,97; textil de 1846 px de lado); colores identificables (probabilidad 0,77; 2 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,84; bordes cromáticos en el 23 % del textil); completitud incierta (probabilidad 0,63; compacidad 0,84, lagunas 14,0 %); estructura no evidente. Puntaje 69.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -4410,6 +5180,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA43" s="4" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="AB43" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC43" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD43" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,78; textil de 2126 px de lado); colores parcialmente identificables (probabilidad 0,53; 1 color claramente distinto, 2 tonos, colorido 25); formas parcialmente visibles (probabilidad 0,69; bordes cromáticos en el 21 % del textil); textil incompleto (probabilidad 0,29; compacidad 0,54, lagunas 10,4 %, el título dice «fragment»); estructura no evidente. Puntaje 49.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -4498,6 +5286,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA44" s="4" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="AB44" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC44" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD44" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,70; textil de 1301 px de lado); colores identificables (probabilidad 0,87; 2 colores claramente distintos, 2 tonos, colorido 36); formas visibles (probabilidad 0,84; bordes cromáticos en el 45 % del textil); textil completo (probabilidad 0,72; compacidad 0,64, lagunas 7,4 %); estructura no evidente. Puntaje 75.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -4586,6 +5392,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA45" s="4" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="AB45" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC45" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD45" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,83; textil de 3136 px de lado); colores identificables (probabilidad 0,94; 2 colores claramente distintos, 3 tonos, colorido 34); formas visibles (probabilidad 0,96; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,76; compacidad 0,88, lagunas 0,3 %, el título dice «fragment»); estructura no evidente. Puntaje 71.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -4674,6 +5498,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA46" s="4" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="AB46" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC46" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD46" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,98; textil de 2443 px de lado); colores identificables (probabilidad 0,96; 3 colores claramente distintos, 2 tonos, colorido 51); formas visibles (probabilidad 0,95; bordes cromáticos en el 25 % del textil); textil completo (probabilidad 0,85; compacidad 0,96, lagunas 0,0 %); estructura repetitiva. Puntaje 69.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -4762,6 +5604,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA47" s="4" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="AB47" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC47" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD47" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,56; textil de 2877 px de lado); colores identificables (probabilidad 0,97; 4 colores claramente distintos, 3 tonos, colorido 48); formas visibles (probabilidad 0,96; bordes cromáticos en el 44 % del textil); textil completo (probabilidad 0,85; compacidad 0,92, lagunas 0,0 %); estructura no evidente. Puntaje 75.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -4850,6 +5710,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA48" s="4" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="AB48" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC48" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD48" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,17; textil de 1495 px de lado); colores identificables (probabilidad 0,77; 2 colores claramente distintos, 3 tonos, colorido 32); formas visibles (probabilidad 0,72; bordes cromáticos en el 37 % del textil); completitud incierta (probabilidad 0,48; compacidad 0,50, lagunas 0,0 %); estructura repetitiva. Puntaje 63.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -4938,6 +5816,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA49" s="4" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="AB49" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC49" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD49" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,76; textil de 3094 px de lado); colores identificables (probabilidad 0,93; 2 colores claramente distintos, 3 tonos, colorido 36); formas visibles (probabilidad 0,95; bordes cromáticos en el 47 % del textil); completitud incierta (probabilidad 0,67; compacidad 0,86, lagunas 0,1 %, el título dice «fragment»); estructura no evidente. Puntaje 69.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -5026,6 +5922,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA50" s="4" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="AB50" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC50" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD50" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,87; textil de 3193 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 3 tonos, colorido 33); formas visibles (probabilidad 0,99; bordes cromáticos en el 36 % del textil); textil completo (probabilidad 0,93; compacidad 0,97, lagunas 0,0 %); estructura no evidente. Puntaje 74.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -5114,6 +6028,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA51" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="AB51" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC51" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD51" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,32; textil de 2721 px de lado); colores identificables (probabilidad 0,98; 3 colores claramente distintos, 3 tonos, colorido 43); formas visibles (probabilidad 0,98; bordes cromáticos en el 24 % del textil); textil completo (probabilidad 0,93; compacidad 0,95, lagunas 0,0 %); estructura repetitiva. Puntaje 75.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -5202,6 +6134,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA52" s="4" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="AB52" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC52" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD52" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,41; textil de 2116 px de lado); colores identificables (probabilidad 0,83; 2 colores claramente distintos, 3 tonos, colorido 30); formas visibles (probabilidad 0,90; bordes cromáticos en el 28 % del textil); completitud incierta (probabilidad 0,64; compacidad 0,83, lagunas 13,6 %); estructura no evidente. Puntaje 72.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -5290,6 +6240,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA53" s="4" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="AB53" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC53" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD53" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,51; textil de 3149 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 42); formas visibles (probabilidad 0,98; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,92; compacidad 0,96, lagunas 0,0 %); estructura no evidente. Puntaje 74.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -5378,6 +6346,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA54" s="4" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="AB54" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC54" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD54" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,63; textil de 2925 px de lado); colores identificables (probabilidad 0,97; 1 color claramente distinto, 3 tonos, colorido 39); formas visibles (probabilidad 0,98; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,94; compacidad 0,93, lagunas 0,0 %); estructura repetitiva. Puntaje 74.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -5466,6 +6452,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA55" s="4" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="AB55" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC55" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD55" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 0,90; textil de 1874 px de lado); colores parcialmente identificables (probabilidad 0,57; 3 colores claramente distintos, 2 tonos, colorido 37); formas parcialmente visibles (probabilidad 0,59; bordes cromáticos en el 34 % del textil); textil incompleto (probabilidad 0,25; compacidad 0,66, lagunas 2,9 %, el título dice «fragment»); estructura no evidente. Puntaje 47.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -5554,6 +6558,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA56" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB56" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC56" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD56" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,50; textil de 2790 px de lado); colores identificables (probabilidad 0,91; 2 colores claramente distintos, 3 tonos, colorido 39); formas visibles (probabilidad 0,96; bordes cromáticos en el 37 % del textil); completitud incierta (probabilidad 0,69; compacidad 0,92, lagunas 22,7 %); estructura no evidente. Puntaje 80 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -5642,6 +6664,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA57" s="4" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="AB57" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC57" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD57" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,91; textil de 2911 px de lado); colores identificables (probabilidad 0,91; 2 colores claramente distintos, 1 tono, colorido 18); formas visibles (probabilidad 0,94; bordes cromáticos en el 6 % del textil); textil completo (probabilidad 0,83; compacidad 0,90, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 66.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -5730,6 +6770,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA58" s="4" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="AB58" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC58" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD58" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,87; textil de 2204 px de lado); colores identificables (probabilidad 0,74; 1 color claramente distinto, 3 tonos, colorido 25); formas visibles (probabilidad 0,82; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,48; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 57.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -5818,6 +6876,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA59" s="4" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="AB59" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC59" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD59" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,15; textil de 2409 px de lado); colores identificables (probabilidad 0,85; 1 color claramente distinto, 2 tonos, colorido 32); formas visibles (probabilidad 0,90; bordes cromáticos en el 19 % del textil); completitud incierta (probabilidad 0,67; compacidad 0,94, lagunas 0,3 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -5906,6 +6982,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA60" s="4" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="AB60" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC60" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD60" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 1,00; textil de 1225 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 2 tonos, colorido 37); formas visibles (probabilidad 0,97; bordes cromáticos en el 31 % del textil); textil completo (probabilidad 0,86; compacidad 0,93, lagunas 0,0 %, el título dice «fragment»); estructura simétrica. Puntaje 77 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -5994,6 +7088,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA61" s="4" t="n">
+        <v>74.7</v>
+      </c>
+      <c r="AB61" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC61" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD61" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,51; textil de 2454 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 59); formas visibles (probabilidad 0,99; bordes cromáticos en el 60 % del textil); textil completo (probabilidad 0,91; compacidad 0,96, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 75.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -6082,6 +7194,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA62" s="4" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="AB62" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC62" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD62" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,35; textil de 2897 px de lado); colores identificables (probabilidad 0,93; 3 colores claramente distintos, 3 tonos, colorido 46); formas visibles (probabilidad 0,93; bordes cromáticos en el 21 % del textil); completitud incierta (probabilidad 0,63; compacidad 0,90, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 68.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -6170,6 +7300,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA63" s="4" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="AB63" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC63" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD63" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,63; textil de 2088 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 45); formas visibles (probabilidad 1,00; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,97; compacidad 0,97, lagunas 0,0 %, el título dice «fragment»); estructura simétrica. Puntaje 81 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -6258,6 +7406,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA64" s="4" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="AB64" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC64" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD64" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 0,87; textil de 2456 px de lado); colores identificables (probabilidad 0,92; 3 colores claramente distintos, 2 tonos, colorido 52); formas visibles (probabilidad 0,83; bordes cromáticos en el 35 % del textil); completitud incierta (probabilidad 0,62; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 67.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -6346,6 +7512,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA65" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="AB65" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC65" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD65" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,96; textil de 814 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 3 tonos, colorido 38); formas visibles (probabilidad 0,96; bordes cromáticos en el 40 % del textil); textil completo (probabilidad 0,72; compacidad 0,82, lagunas 0,4 %); estructura no evidente. Puntaje 78 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -6434,6 +7618,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA66" s="4" t="n">
+        <v>80.2</v>
+      </c>
+      <c r="AB66" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC66" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD66" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,15; textil de 704 px de lado); colores identificables (probabilidad 0,97; 3 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,95; bordes cromáticos en el 40 % del textil); textil completo (probabilidad 0,80; compacidad 0,83, lagunas 0,0 %); estructura no evidente. Puntaje 80 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -6522,6 +7724,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA67" s="4" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="AB67" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC67" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD67" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,89; textil de 1207 px de lado); colores identificables (probabilidad 0,93; 2 colores claramente distintos, 2 tonos, colorido 37); formas visibles (probabilidad 0,90; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,76; compacidad 0,62, lagunas 0,0 %); estructura no evidente. Puntaje 73.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -6610,6 +7830,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA68" s="4" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="AB68" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC68" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD68" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,13; textil de 1077 px de lado); colores identificables (probabilidad 0,97; 3 colores claramente distintos, 3 tonos, colorido 49); formas visibles (probabilidad 0,95; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,73; compacidad 0,64, lagunas 3,1 %); estructura repetitiva. Puntaje 78 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -6698,6 +7936,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA69" s="4" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="AB69" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC69" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD69" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,02; textil de 1558 px de lado); colores identificables (probabilidad 0,93; 2 colores claramente distintos, 3 tonos, colorido 24); formas visibles (probabilidad 0,92; bordes cromáticos en el 24 % del textil); completitud incierta (probabilidad 0,56; compacidad 0,90, lagunas 0,1 %, el título dice «fragment»); estructura no evidente. Puntaje 67.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -6786,6 +8042,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA70" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="AB70" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC70" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD70" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,00; textil de 1666 px de lado); colores identificables (probabilidad 0,90; 2 colores claramente distintos, 3 tonos, colorido 23); formas visibles (probabilidad 0,91; bordes cromáticos en el 19 % del textil); completitud incierta (probabilidad 0,54; compacidad 0,90, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 66.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -6874,6 +8148,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA71" s="4" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="AB71" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC71" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD71" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,61; textil de 2077 px de lado); colores identificables (probabilidad 0,94; 2 colores claramente distintos, 3 tonos, colorido 30); formas visibles (probabilidad 0,95; bordes cromáticos en el 29 % del textil); completitud incierta (probabilidad 0,61; compacidad 0,91, lagunas 2,4 %, el título dice «fragment»); estructura no evidente. Puntaje 70.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -6962,6 +8254,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA72" s="4" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="AB72" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC72" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD72" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,36; textil de 2716 px de lado); colores identificables (probabilidad 0,97; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,97; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,95; compacidad 0,95, lagunas 0,0 %); estructura simétrica. Puntaje 74.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -7050,6 +8360,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA73" s="4" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="AB73" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC73" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD73" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 3,19; textil de 2988 px de lado); colores identificables (probabilidad 0,94; 1 color claramente distinto, 1 tono, colorido 35); formas visibles (probabilidad 0,96; bordes cromáticos en el 18 % del textil); textil completo (probabilidad 0,95; compacidad 0,95, lagunas 0,0 %); estructura no evidente. Puntaje 69.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -7138,6 +8466,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA74" s="4" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="AB74" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC74" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD74" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,17; textil de 2477 px de lado); colores identificables (probabilidad 0,93; 2 colores claramente distintos, 2 tonos, colorido 22); formas visibles (probabilidad 0,94; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,79; compacidad 0,92, lagunas 3,8 %); estructura no evidente. Puntaje 70.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -7226,6 +8572,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA75" s="4" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="AB75" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC75" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD75" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,92; textil de 2430 px de lado); colores identificables (probabilidad 0,72; 2 colores claramente distintos, 2 tonos, colorido 31); formas visibles (probabilidad 0,85; bordes cromáticos en el 25 % del textil); textil incompleto (probabilidad 0,38; compacidad 0,86, lagunas 15,1 %, el título dice «fragment»); estructura no evidente. Puntaje 61.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -7314,6 +8678,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA76" s="4" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="AB76" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC76" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD76" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,39; textil de 2469 px de lado); colores identificables (probabilidad 0,96; 1 color claramente distinto, 2 tonos, colorido 18); formas visibles (probabilidad 0,97; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,91; compacidad 0,90, lagunas 0,0 %); estructura repetitiva. Puntaje 71.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -7402,6 +8784,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA77" s="4" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="AB77" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC77" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD77" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 0,98; textil de 2858 px de lado); colores identificables (probabilidad 0,92; 1 color claramente distinto, 1 tono, colorido 15); formas visibles (probabilidad 0,94; bordes cromáticos en el 10 % del textil); textil completo (probabilidad 0,84; compacidad 0,91, lagunas 0,9 %); estructura repetitiva y simétrica. Puntaje 68.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -7490,6 +8890,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA78" s="4" t="n">
+        <v>79.40000000000001</v>
+      </c>
+      <c r="AB78" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC78" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD78" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,05; textil de 2968 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 4 tonos, colorido 44); formas visibles (probabilidad 1,00; bordes cromáticos en el 56 % del textil); textil completo (probabilidad 0,96; compacidad 0,98, lagunas 1,0 %, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 79 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -7578,6 +8996,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA79" s="4" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="AB79" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC79" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD79" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,88; textil de 2489 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 45); formas visibles (probabilidad 0,99; bordes cromáticos en el 56 % del textil); textil completo (probabilidad 0,96; compacidad 0,95, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 79 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -7666,6 +9102,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA80" s="4" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="AB80" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC80" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD80" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,87; textil de 2535 px de lado); colores identificables (probabilidad 1,00; 5 colores claramente distintos, 4 tonos, colorido 45); formas visibles (probabilidad 1,00; bordes cromáticos en el 54 % del textil); textil completo (probabilidad 0,94; compacidad 0,98, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 80 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -7754,6 +9208,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA81" s="4" t="n">
+        <v>79.40000000000001</v>
+      </c>
+      <c r="AB81" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC81" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD81" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,45; textil de 3178 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 57); formas visibles (probabilidad 1,00; bordes cromáticos en el 40 % del textil); textil completo (probabilidad 0,98; compacidad 0,93, lagunas 0,1 %); estructura repetitiva y simétrica. Puntaje 79 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -7842,6 +9314,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA82" s="4" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="AB82" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC82" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD82" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,18; textil de 2399 px de lado); colores identificables (probabilidad 0,88; 1 color claramente distinto, 2 tonos, colorido 29); formas visibles (probabilidad 0,92; bordes cromáticos en el 11 % del textil); textil completo (probabilidad 0,80; compacidad 0,85, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 66.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -7930,6 +9420,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA83" s="4" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="AB83" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC83" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD83" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,18; textil de 2399 px de lado); colores identificables (probabilidad 0,88; 1 color claramente distinto, 2 tonos, colorido 29); formas visibles (probabilidad 0,92; bordes cromáticos en el 11 % del textil); textil completo (probabilidad 0,80; compacidad 0,85, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 66.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -8018,6 +9526,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA84" s="4" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="AB84" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC84" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD84" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,29; textil de 2283 px de lado); colores identificables (probabilidad 0,84; 1 color claramente distinto, 2 tonos, colorido 28); formas visibles (probabilidad 0,90; bordes cromáticos en el 12 % del textil); completitud incierta (probabilidad 0,69; compacidad 0,80, lagunas 1,3 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -8106,6 +9632,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA85" s="4" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="AB85" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC85" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD85" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,23; textil de 2605 px de lado); colores identificables (probabilidad 0,82; 1 color claramente distinto, 2 tonos, colorido 30); formas visibles (probabilidad 0,89; bordes cromáticos en el 14 % del textil); textil completo (probabilidad 0,74; compacidad 0,82, lagunas 0,7 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -8194,6 +9738,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA86" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="AB86" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC86" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD86" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,12; textil de 2809 px de lado); colores identificables (probabilidad 0,86; 1 color claramente distinto, 2 tonos, colorido 18); formas visibles (probabilidad 0,89; bordes cromáticos en el 3 % del textil); textil completo (probabilidad 0,83; compacidad 0,85, lagunas 0,0 %); estructura no evidente. Puntaje 64.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -8282,6 +9844,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA87" s="4" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="AB87" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC87" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD87" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,04; textil de 1679 px de lado); colores identificables (probabilidad 0,82; 1 color claramente distinto, 1 tono, colorido 22); formas visibles (probabilidad 0,82; bordes cromáticos en el 16 % del textil); textil completo (probabilidad 0,85; compacidad 0,70, lagunas 0,0 %); estructura repetitiva. Puntaje 66.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -8370,6 +9950,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA88" s="4" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="AB88" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC88" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD88" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,24; textil de 2757 px de lado); colores identificables (probabilidad 0,92; 4 colores claramente distintos, 2 tonos, colorido 48); formas visibles (probabilidad 0,86; bordes cromáticos en el 30 % del textil); textil completo (probabilidad 0,72; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 69.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -8458,6 +10056,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA89" s="4" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="AB89" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC89" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD89" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,56; textil de 1657 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 3 tonos, colorido 45); formas visibles (probabilidad 0,98; bordes cromáticos en el 36 % del textil); textil completo (probabilidad 0,95; compacidad 0,85, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 80 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -8546,6 +10162,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA90" s="4" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="AB90" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC90" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD90" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,60; textil de 2088 px de lado); colores identificables (probabilidad 0,96; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,97; bordes cromáticos en el 27 % del textil); completitud incierta (probabilidad 0,59; compacidad 0,83, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 71.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -8634,6 +10268,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA91" s="4" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="AB91" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC91" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD91" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,65; textil de 1378 px de lado); colores identificables (probabilidad 0,85; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,84; bordes cromáticos en el 27 % del textil); completitud incierta (probabilidad 0,57; compacidad 0,82, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -8722,6 +10374,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA92" s="4" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="AB92" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC92" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD92" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,56; textil de 1445 px de lado); colores identificables (probabilidad 0,84; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,84; bordes cromáticos en el 24 % del textil); completitud incierta (probabilidad 0,60; compacidad 0,87, lagunas 0,2 %, el título dice «fragment»); estructura no evidente. Puntaje 64.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -8810,6 +10480,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA93" s="4" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="AB93" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC93" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD93" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,76; textil de 1528 px de lado); colores identificables (probabilidad 0,93; 3 colores claramente distintos, 3 tonos, colorido 36); formas visibles (probabilidad 0,92; bordes cromáticos en el 30 % del textil); completitud incierta (probabilidad 0,64; compacidad 0,81, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 72.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -8898,6 +10586,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA94" s="4" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="AB94" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC94" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD94" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 3,33; textil de 1348 px de lado); colores identificables (probabilidad 0,79; 2 colores claramente distintos, 1 tono, colorido 20); formas visibles (probabilidad 0,75; bordes cromáticos en el 38 % del textil); textil completo (probabilidad 0,70; compacidad 0,38, lagunas 5,4 %); estructura no evidente. Puntaje 68.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -8912,18 +10618,34 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>descartados</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr"/>
-      <c r="F95" s="4" t="inlineStr"/>
-      <c r="G95" s="4" t="inlineStr"/>
-      <c r="H95" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>plumaria</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>Asignacion automatica (puntaje de aptitud). Textil con plumaria: fuera del estudio. Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía buena (nitidez 1,85; textil de 1849 px de lado); colores identificables (probabilidad 0,94; 1 color claramente distinto, 2 tonos, colorido 36); formas visibles (probabilidad 0,94; bordes cromáticos en el 9 % del textil); textil completo (probabilidad 0,93; compacidad 0,91, lagunas 0,4 %); estructura no evidente. Puntaje 69. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
           <t>Feathered Panel</t>
@@ -8983,7 +10705,25 @@
       <c r="Y95" s="4" t="inlineStr"/>
       <c r="Z95" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>aptitud_automatica</t>
+        </is>
+      </c>
+      <c r="AA95" s="4" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="AB95" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC95" s="4" t="inlineStr">
+        <is>
+          <t>plumaria</t>
+        </is>
+      </c>
+      <c r="AD95" s="4" t="inlineStr">
+        <is>
+          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía buena (nitidez 1,85; textil de 1849 px de lado); colores identificables (probabilidad 0,94; 1 color claramente distinto, 2 tonos, colorido 36); formas visibles (probabilidad 0,94; bordes cromáticos en el 9 % del textil); textil completo (probabilidad 0,93; compacidad 0,91, lagunas 0,4 %); estructura no evidente. Puntaje 69.</t>
         </is>
       </c>
     </row>
@@ -9074,6 +10814,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA96" s="4" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="AB96" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC96" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD96" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,24; textil de 1536 px de lado); colores identificables (probabilidad 0,85; 2 colores claramente distintos, 1 tono, colorido 16); formas visibles (probabilidad 0,80; bordes cromáticos en el 49 % del textil); textil completo (probabilidad 0,77; compacidad 0,52, lagunas 0,0 %); estructura no evidente. Puntaje 71.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -9088,18 +10846,34 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E97" s="4" t="inlineStr"/>
-      <c r="F97" s="4" t="inlineStr"/>
-      <c r="G97" s="4" t="inlineStr"/>
-      <c r="H97" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>textil completo con colores y formas visibles. La mejor imagen para el estudio</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>Anotación de la validación ciega del 2026-10-19 (data/metadata/validacion_met_cma_v2.xlsx, orden 12): principal. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
           <t>Four-Cornered Hat</t>
@@ -9159,7 +10933,25 @@
       <c r="Y97" s="4" t="inlineStr"/>
       <c r="Z97" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>validacion_ciega_v2</t>
+        </is>
+      </c>
+      <c r="AA97" s="4" t="n">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="AB97" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC97" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD97" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,02; textil de 2238 px de lado); colores identificables (probabilidad 0,94; 5 colores claramente distintos, 4 tonos, colorido 61); formas visibles (probabilidad 0,84; bordes cromáticos en el 38 % del textil); completitud incierta (probabilidad 0,45; compacidad 0,69, lagunas 0,1 %); estructura no evidente. Puntaje 71.</t>
         </is>
       </c>
     </row>
@@ -9250,6 +11042,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA98" s="4" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="AB98" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC98" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD98" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 0,69; textil de 3140 px de lado); colores identificables (probabilidad 0,89; 5 colores claramente distintos, 3 tonos, colorido 54); formas visibles (probabilidad 0,80; bordes cromáticos en el 22 % del textil); completitud incierta (probabilidad 0,59; toma cerrada, el contorno de la pieza no se ve); estructura simétrica. Puntaje 66.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -9338,6 +11148,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA99" s="4" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="AB99" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC99" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD99" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,49; textil de 2055 px de lado); colores identificables (probabilidad 0,93; 3 colores claramente distintos, 3 tonos, colorido 59); formas visibles (probabilidad 0,90; bordes cromáticos en el 47 % del textil); completitud incierta (probabilidad 0,55; compacidad 0,81, lagunas 0,0 %); estructura no evidente. Puntaje 68.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -9426,6 +11254,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA100" s="4" t="n">
+        <v>73.3</v>
+      </c>
+      <c r="AB100" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC100" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD100" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,50; textil de 2177 px de lado); colores identificables (probabilidad 0,96; 4 colores claramente distintos, 3 tonos, colorido 50); formas visibles (probabilidad 0,93; bordes cromáticos en el 42 % del textil); completitud incierta (probabilidad 0,62; compacidad 0,80, lagunas 0,0 %); estructura no evidente. Puntaje 73.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -9440,18 +11286,34 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>descartados</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E101" s="4" t="inlineStr"/>
-      <c r="F101" s="4" t="inlineStr"/>
-      <c r="G101" s="4" t="inlineStr"/>
-      <c r="H101" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>plumaria</t>
+        </is>
+      </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>Asignacion automatica (puntaje de aptitud). Textil con plumaria: fuera del estudio. Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía buena (nitidez 1,58; textil de 3053 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 3 tonos, colorido 51); formas visibles (probabilidad 0,97; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,90; compacidad 0,86, lagunas 0,8 %); estructura repetitiva y simétrica. Puntaje 73. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
           <t>Feathered Tabard or Tunic</t>
@@ -9511,7 +11373,25 @@
       <c r="Y101" s="4" t="inlineStr"/>
       <c r="Z101" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>aptitud_automatica</t>
+        </is>
+      </c>
+      <c r="AA101" s="4" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="AB101" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC101" s="4" t="inlineStr">
+        <is>
+          <t>plumaria</t>
+        </is>
+      </c>
+      <c r="AD101" s="4" t="inlineStr">
+        <is>
+          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía buena (nitidez 1,58; textil de 3053 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 3 tonos, colorido 51); formas visibles (probabilidad 0,97; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,90; compacidad 0,86, lagunas 0,8 %); estructura repetitiva y simétrica. Puntaje 73.</t>
         </is>
       </c>
     </row>
@@ -9602,6 +11482,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA102" s="4" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="AB102" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC102" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD102" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,37; textil de 1774 px de lado); colores identificables (probabilidad 0,90; 4 colores claramente distintos, 3 tonos, colorido 63); formas visibles (probabilidad 0,80; bordes cromáticos en el 35 % del textil); completitud incierta (probabilidad 0,57; compacidad 0,65, lagunas 0,4 %); estructura no evidente. Puntaje 68.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -9616,18 +11514,34 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>descartados</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E103" s="4" t="inlineStr"/>
-      <c r="F103" s="4" t="inlineStr"/>
-      <c r="G103" s="4" t="inlineStr"/>
-      <c r="H103" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>plumaria</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
+          <t>Asignacion automatica (puntaje de aptitud). Textil con plumaria: fuera del estudio. Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía deficiente (nitidez 0,71; textil de 2797 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 28); formas visibles (probabilidad 0,99; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,90; toma cerrada, el contorno de la pieza no se ve); estructura simétrica. Puntaje 82. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="I103" s="4" t="inlineStr">
         <is>
           <t>Feathered Tabard or Tunic</t>
@@ -9687,7 +11601,25 @@
       <c r="Y103" s="4" t="inlineStr"/>
       <c r="Z103" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>aptitud_automatica</t>
+        </is>
+      </c>
+      <c r="AA103" s="4" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="AB103" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC103" s="4" t="inlineStr">
+        <is>
+          <t>plumaria</t>
+        </is>
+      </c>
+      <c r="AD103" s="4" t="inlineStr">
+        <is>
+          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía deficiente (nitidez 0,71; textil de 2797 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 28); formas visibles (probabilidad 0,99; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,90; toma cerrada, el contorno de la pieza no se ve); estructura simétrica. Puntaje 82.</t>
         </is>
       </c>
     </row>
@@ -9704,18 +11636,34 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>descartados</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E104" s="4" t="inlineStr"/>
-      <c r="F104" s="4" t="inlineStr"/>
-      <c r="G104" s="4" t="inlineStr"/>
-      <c r="H104" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>plumaria</t>
+        </is>
+      </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>Asignacion automatica (puntaje de aptitud). Textil con plumaria: fuera del estudio. Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía regular (nitidez 1,09; textil de 2509 px de lado); colores identificables (probabilidad 0,99; 4 colores claramente distintos, 3 tonos, colorido 100); formas visibles (probabilidad 0,96; bordes cromáticos en el 45 % del textil); textil completo (probabilidad 0,89; toma cerrada, el contorno de la pieza no se ve); estructura repetitiva y simétrica. Puntaje 78. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="H104" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="I104" s="4" t="inlineStr">
         <is>
           <t>Feathered Tabard or Tunic</t>
@@ -9775,7 +11723,25 @@
       <c r="Y104" s="4" t="inlineStr"/>
       <c r="Z104" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>aptitud_automatica</t>
+        </is>
+      </c>
+      <c r="AA104" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="AB104" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC104" s="4" t="inlineStr">
+        <is>
+          <t>plumaria</t>
+        </is>
+      </c>
+      <c r="AD104" s="4" t="inlineStr">
+        <is>
+          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía regular (nitidez 1,09; textil de 2509 px de lado); colores identificables (probabilidad 0,99; 4 colores claramente distintos, 3 tonos, colorido 100); formas visibles (probabilidad 0,96; bordes cromáticos en el 45 % del textil); textil completo (probabilidad 0,89; toma cerrada, el contorno de la pieza no se ve); estructura repetitiva y simétrica. Puntaje 78.</t>
         </is>
       </c>
     </row>
@@ -9866,6 +11832,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA105" s="4" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="AB105" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC105" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD105" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 0,73; textil de 3203 px de lado); colores identificables (probabilidad 0,80; 3 colores claramente distintos, 2 tonos, colorido 22); formas visibles (probabilidad 0,77; bordes cromáticos en el 11 % del textil); completitud incierta (probabilidad 0,53; toma cerrada, el contorno de la pieza no se ve); estructura simétrica. Puntaje 59.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -9880,18 +11864,34 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>descartados</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E106" s="4" t="inlineStr"/>
-      <c r="F106" s="4" t="inlineStr"/>
-      <c r="G106" s="4" t="inlineStr"/>
-      <c r="H106" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr">
+        <is>
+          <t>plumaria</t>
+        </is>
+      </c>
+      <c r="F106" s="4" t="inlineStr">
+        <is>
+          <t>Asignacion automatica (puntaje de aptitud). Textil con plumaria: fuera del estudio. Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía deficiente (nitidez 0,77; textil de 2078 px de lado); colores no identificables (probabilidad 0,21; 4 colores claramente distintos, 4 tonos, colorido 127); formas no visibles (probabilidad 0,21; bordes cromáticos en el 20 % del textil); textil incompleto (probabilidad 0,10; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 18. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="H106" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="I106" s="4" t="inlineStr">
         <is>
           <t>Feathered Panel</t>
@@ -9951,7 +11951,25 @@
       <c r="Y106" s="4" t="inlineStr"/>
       <c r="Z106" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>aptitud_automatica</t>
+        </is>
+      </c>
+      <c r="AA106" s="4" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="AB106" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC106" s="4" t="inlineStr">
+        <is>
+          <t>plumaria</t>
+        </is>
+      </c>
+      <c r="AD106" s="4" t="inlineStr">
+        <is>
+          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía deficiente (nitidez 0,77; textil de 2078 px de lado); colores no identificables (probabilidad 0,21; 4 colores claramente distintos, 4 tonos, colorido 127); formas no visibles (probabilidad 0,21; bordes cromáticos en el 20 % del textil); textil incompleto (probabilidad 0,10; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 18.</t>
         </is>
       </c>
     </row>
@@ -10042,6 +12060,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA107" s="4" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="AB107" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC107" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD107" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 0,99; textil de 1749 px de lado); colores identificables (probabilidad 0,86; 3 colores claramente distintos, 1 tono, colorido 15); formas visibles (probabilidad 0,81; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,66; compacidad 0,77, lagunas 1,3 %); estructura simétrica. Puntaje 65.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -10130,6 +12166,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA108" s="4" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="AB108" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC108" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD108" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 0,60; textil de 1139 px de lado); colores no identificables (probabilidad 0,29; 3 colores claramente distintos, 1 tono, colorido 21); formas no visibles (probabilidad 0,20; bordes cromáticos en el 15 % del textil); textil incompleto (probabilidad 0,09; compacidad 0,44, lagunas 0,1 %); estructura no evidente. Puntaje 21.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -10218,6 +12272,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA109" s="4" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="AB109" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC109" s="4" t="inlineStr">
+        <is>
+          <t>posterior_inca</t>
+        </is>
+      </c>
+      <c r="AD109" s="4" t="inlineStr">
+        <is>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,06; textil de 3273 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 2 tonos, colorido 63); formas visibles (probabilidad 0,99; bordes cromáticos en el 30 % del textil); textil completo (probabilidad 0,98; compacidad 0,97, lagunas 0,0 %); estructura repetitiva. Puntaje 73.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -10306,6 +12378,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA110" s="4" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="AB110" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC110" s="4" t="inlineStr">
+        <is>
+          <t>posterior_inca</t>
+        </is>
+      </c>
+      <c r="AD110" s="4" t="inlineStr">
+        <is>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,92; textil de 2142 px de lado); colores identificables (probabilidad 0,97; 2 colores claramente distintos, 1 tono, colorido 30); formas visibles (probabilidad 0,97; bordes cromáticos en el 31 % del textil); textil completo (probabilidad 0,95; compacidad 0,96, lagunas 0,0 %); estructura no evidente. Puntaje 74.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -10394,6 +12484,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA111" s="4" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="AB111" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC111" s="4" t="inlineStr">
+        <is>
+          <t>posterior_inca</t>
+        </is>
+      </c>
+      <c r="AD111" s="4" t="inlineStr">
+        <is>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,73; textil de 1410 px de lado); colores identificables (probabilidad 0,96; 2 colores claramente distintos, 0 tonos, colorido 11); formas visibles (probabilidad 0,95; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,93; compacidad 0,88, lagunas 0,0 %); estructura no evidente. Puntaje 76.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
@@ -10482,6 +12590,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA112" s="4" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="AB112" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC112" s="4" t="inlineStr">
+        <is>
+          <t>resolucion_insuficiente</t>
+        </is>
+      </c>
+      <c r="AD112" s="4" t="inlineStr">
+        <is>
+          <t>El textil mide 288 px de lado en la imagen institucional (mínimo 300). Fotografía buena (nitidez 2,99; textil de 288 px de lado); colores identificables (probabilidad 0,98; 1 color claramente distinto, 2 tonos, colorido 17); formas visibles (probabilidad 0,97; bordes cromáticos en el 3 % del textil); textil completo (probabilidad 0,89; compacidad 0,51, lagunas 0,0 %); estructura no evidente. Puntaje 76.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -10570,6 +12696,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA113" s="4" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="AB113" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC113" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD113" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 0,64; textil de 1599 px de lado); colores identificables (probabilidad 0,94; 4 colores claramente distintos, 5 tonos, colorido 38); formas visibles (probabilidad 0,92; bordes cromáticos en el 17 % del textil); completitud incierta (probabilidad 0,42; compacidad 0,76, lagunas 0,2 %); estructura no evidente. Puntaje 75.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
@@ -10658,6 +12802,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA114" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="AB114" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC114" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD114" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,08; textil de 2550 px de lado); colores parcialmente identificables (probabilidad 0,52; 2 colores claramente distintos, 1 tono, colorido 18); formas parcialmente visibles (probabilidad 0,61; bordes cromáticos en el 19 % del textil); textil incompleto (probabilidad 0,18; compacidad 0,79, lagunas 0,3 %, el título dice «fragment»); estructura no evidente. Puntaje 41.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -10672,18 +12834,34 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>secundario</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E115" s="4" t="inlineStr"/>
-      <c r="F115" s="4" t="inlineStr"/>
-      <c r="G115" s="4" t="inlineStr"/>
-      <c r="H115" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="inlineStr">
+        <is>
+          <t>textil con colores visibles</t>
+        </is>
+      </c>
+      <c r="F115" s="4" t="inlineStr">
+        <is>
+          <t>Anotación de la validación ciega del 2026-10-19 (data/metadata/validacion_met_cma_v2.xlsx, orden 29): secundario. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G115" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H115" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="I115" s="4" t="inlineStr">
         <is>
           <t>Border Fragment with Birds and Flowers</t>
@@ -10743,7 +12921,25 @@
       <c r="Y115" s="4" t="inlineStr"/>
       <c r="Z115" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>validacion_ciega_v2</t>
+        </is>
+      </c>
+      <c r="AA115" s="4" t="n">
+        <v>70.40000000000001</v>
+      </c>
+      <c r="AB115" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC115" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD115" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,28; textil de 920 px de lado); colores identificables (probabilidad 0,90; 3 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,80; bordes cromáticos en el 57 % del textil); textil incompleto (probabilidad 0,39; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 70.</t>
         </is>
       </c>
     </row>
@@ -10834,6 +13030,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA116" s="4" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="AB116" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC116" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD116" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,26; textil de 922 px de lado); colores identificables (probabilidad 0,91; 3 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,81; bordes cromáticos en el 57 % del textil); completitud incierta (probabilidad 0,45; compacidad 0,68, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 72.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -10922,6 +13136,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA117" s="4" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="AB117" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC117" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD117" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,28; textil de 918 px de lado); colores identificables (probabilidad 0,91; 3 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,82; bordes cromáticos en el 57 % del textil); completitud incierta (probabilidad 0,43; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 72.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
@@ -11010,6 +13242,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA118" s="4" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="AB118" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC118" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD118" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,28; textil de 925 px de lado); colores identificables (probabilidad 0,88; 2 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,80; bordes cromáticos en el 57 % del textil); completitud incierta (probabilidad 0,43; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 70.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -11098,6 +13348,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA119" s="4" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="AB119" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC119" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD119" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,54; textil de 2608 px de lado); colores identificables (probabilidad 0,72; 1 color claramente distinto, 2 tonos, colorido 22); formas visibles (probabilidad 0,75; bordes cromáticos en el 11 % del textil); completitud incierta (probabilidad 0,56; compacidad 0,73, lagunas 0,5 %); estructura no evidente. Puntaje 53.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
@@ -11186,6 +13454,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA120" s="4" t="n">
+        <v>85.8</v>
+      </c>
+      <c r="AB120" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC120" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD120" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,18; textil de 1118 px de lado); colores identificables (probabilidad 0,99; 4 colores claramente distintos, 3 tonos, colorido 46); formas visibles (probabilidad 0,97; bordes cromáticos en el 68 % del textil); textil completo (probabilidad 0,87; compacidad 0,89, lagunas 0,0 %); estructura no evidente. Puntaje 86 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -11274,6 +13560,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA121" s="4" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="AB121" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC121" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD121" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,30; textil de 842 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 2 tonos, colorido 37); formas visibles (probabilidad 0,96; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,95; compacidad 0,79, lagunas 0,0 %); estructura no evidente. Puntaje 82 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
@@ -11362,6 +13666,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA122" s="4" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="AB122" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC122" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD122" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,23; textil de 1167 px de lado); colores identificables (probabilidad 0,91; 3 colores claramente distintos, 3 tonos, colorido 40); formas visibles (probabilidad 0,84; bordes cromáticos en el 42 % del textil); completitud incierta (probabilidad 0,49; compacidad 0,71, lagunas 0,0 %); estructura no evidente. Puntaje 72.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -11450,6 +13772,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA123" s="4" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="AB123" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC123" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD123" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,84; textil de 1632 px de lado); colores parcialmente identificables (probabilidad 0,64; 2 colores claramente distintos, 1 tono, colorido 20); formas parcialmente visibles (probabilidad 0,61; bordes cromáticos en el 16 % del textil); completitud incierta (probabilidad 0,53; compacidad 0,61, lagunas 0,0 %); estructura no evidente. Puntaje 48.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
@@ -11538,6 +13878,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA124" s="4" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="AB124" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC124" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD124" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 0,27; textil de 1975 px de lado); colores identificables (probabilidad 0,87; 2 colores claramente distintos, 2 tonos, colorido 16); formas visibles (probabilidad 0,85; bordes cromáticos en el 8 % del textil); completitud incierta (probabilidad 0,49; toma cerrada, el contorno de la pieza no se ve, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 67.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -11626,6 +13984,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA125" s="4" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="AB125" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC125" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD125" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 1,00; textil de 737 px de lado); colores identificables (probabilidad 0,89; 2 colores claramente distintos, 2 tonos, colorido 27); formas visibles (probabilidad 0,89; bordes cromáticos en el 33 % del textil); completitud incierta (probabilidad 0,64; compacidad 0,87, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 72.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -11714,6 +14090,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA126" s="4" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="AB126" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC126" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD126" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía deficiente (nitidez 0,96; textil de 815 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 2 tonos, colorido 27); formas visibles (probabilidad 0,95; bordes cromáticos en el 25 % del textil); textil completo (probabilidad 0,82; compacidad 0,88, lagunas 0,0 %, el título dice «fragment»); estructura simétrica. Puntaje 79 (imagen de referencia sugerida).</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -11802,6 +14196,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA127" s="4" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="AB127" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC127" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD127" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,39; textil de 2469 px de lado); colores identificables (probabilidad 0,96; 1 color claramente distinto, 2 tonos, colorido 18); formas visibles (probabilidad 0,97; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,91; compacidad 0,90, lagunas 0,0 %); estructura repetitiva. Puntaje 71.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
@@ -11890,6 +14302,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA128" s="4" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="AB128" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC128" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD128" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,20; textil de 1289 px de lado); colores no identificables (probabilidad 0,27; 2 colores claramente distintos, 1 tono, colorido 16); formas no visibles (probabilidad 0,27; bordes cromáticos en el 19 % del textil); textil incompleto (probabilidad 0,20; compacidad 0,37, lagunas 7,2 %); estructura no evidente. Puntaje 31.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -11904,18 +14334,34 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>secundario</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E129" s="4" t="inlineStr"/>
-      <c r="F129" s="4" t="inlineStr"/>
-      <c r="G129" s="4" t="inlineStr"/>
-      <c r="H129" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E129" s="4" t="inlineStr">
+        <is>
+          <t>Textil incompleto con colores visibles</t>
+        </is>
+      </c>
+      <c r="F129" s="4" t="inlineStr">
+        <is>
+          <t>Anotación de la validación ciega del 2026-10-19 (data/metadata/validacion_met_cma_v2.xlsx, orden 18): secundario. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G129" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H129" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="I129" s="4" t="inlineStr">
         <is>
           <t>Textile Fragment</t>
@@ -11975,7 +14421,25 @@
       <c r="Y129" s="4" t="inlineStr"/>
       <c r="Z129" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>validacion_ciega_v2</t>
+        </is>
+      </c>
+      <c r="AA129" s="4" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="AB129" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC129" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD129" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,56; textil de 2124 px de lado); colores parcialmente identificables (probabilidad 0,56; 1 color claramente distinto, 2 tonos, colorido 27); formas parcialmente visibles (probabilidad 0,69; bordes cromáticos en el 13 % del textil); textil incompleto (probabilidad 0,37; compacidad 0,55, lagunas 8,1 %, el título dice «fragment»); estructura no evidente. Puntaje 48.</t>
         </is>
       </c>
     </row>
@@ -12066,6 +14530,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA130" s="4" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="AB130" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC130" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD130" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,43; textil de 2361 px de lado); colores identificables (probabilidad 0,74; 1 color claramente distinto, 2 tonos, colorido 29); formas visibles (probabilidad 0,85; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,62; compacidad 0,76, lagunas 4,3 %, el título dice «fragment»); estructura no evidente. Puntaje 59.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -12154,6 +14636,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA131" s="4" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="AB131" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC131" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD131" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,91; textil de 2166 px de lado); colores parcialmente identificables (probabilidad 0,64; 1 color claramente distinto, 2 tonos, colorido 30); formas visibles (probabilidad 0,76; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,43; compacidad 0,66, lagunas 8,9 %, el título dice «fragment»); estructura no evidente. Puntaje 54.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
@@ -12242,6 +14742,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA132" s="4" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="AB132" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC132" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD132" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,20; textil de 2285 px de lado); colores no identificables (probabilidad 0,18; 2 colores claramente distintos, 2 tonos, colorido 42); formas no visibles (probabilidad 0,15; bordes cromáticos en el 31 % del textil); textil incompleto (probabilidad 0,01; compacidad 0,07, lagunas 2,0 %, el título dice «fragment»); estructura no evidente. Puntaje 14.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -12330,6 +14848,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA133" s="4" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="AB133" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC133" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD133" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,04; textil de 1825 px de lado); colores identificables (probabilidad 0,78; 2 colores claramente distintos, 1 tono, colorido 23); formas visibles (probabilidad 0,79; bordes cromáticos en el 17 % del textil); completitud incierta (probabilidad 0,62; compacidad 0,70, lagunas 0,0 %); estructura repetitiva. Puntaje 61.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
@@ -12418,6 +14954,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA134" s="4" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="AB134" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC134" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD134" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,22; textil de 1284 px de lado); colores no identificables (probabilidad 0,28; 2 colores claramente distintos, 1 tono, colorido 16); formas no visibles (probabilidad 0,27; bordes cromáticos en el 17 % del textil); textil incompleto (probabilidad 0,21; compacidad 0,35, lagunas 3,9 %); estructura repetitiva. Puntaje 29.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -12506,6 +15060,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA135" s="4" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="AB135" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC135" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD135" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 1,77; textil de 1155 px de lado); colores identificables (probabilidad 0,81; 2 colores claramente distintos, 3 tonos, colorido 43); formas parcialmente visibles (probabilidad 0,67; bordes cromáticos en el 50 % del textil); completitud incierta (probabilidad 0,49; compacidad 0,35, lagunas 0,0 %); estructura no evidente. Puntaje 65.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
@@ -12520,18 +15092,34 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E136" s="4" t="inlineStr"/>
-      <c r="F136" s="4" t="inlineStr"/>
-      <c r="G136" s="4" t="inlineStr"/>
-      <c r="H136" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E136" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto con figuras visibles</t>
+        </is>
+      </c>
+      <c r="F136" s="4" t="inlineStr">
+        <is>
+          <t>Anotación de la validación ciega del 2026-10-19 (data/metadata/validacion_met_cma_v2.xlsx, orden 22): principal. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G136" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H136" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="I136" s="4" t="inlineStr">
         <is>
           <t>Textile Fragment with Cotton Goddess</t>
@@ -12591,7 +15179,25 @@
       <c r="Y136" s="4" t="inlineStr"/>
       <c r="Z136" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>validacion_ciega_v2</t>
+        </is>
+      </c>
+      <c r="AA136" s="4" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="AB136" s="4" t="inlineStr">
+        <is>
+          <t>revisar</t>
+        </is>
+      </c>
+      <c r="AC136" s="4" t="inlineStr">
+        <is>
+          <t>zona_intermedia</t>
+        </is>
+      </c>
+      <c r="AD136" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía buena (nitidez 2,03; textil de 2930 px de lado); colores identificables (probabilidad 0,78; 1 color claramente distinto, 1 tono, colorido 30); formas visibles (probabilidad 0,87; bordes cromáticos en el 4 % del textil); textil completo (probabilidad 0,78; compacidad 0,88, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 59.</t>
         </is>
       </c>
     </row>
@@ -12608,18 +15214,34 @@
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E137" s="4" t="inlineStr"/>
-      <c r="F137" s="4" t="inlineStr"/>
-      <c r="G137" s="4" t="inlineStr"/>
-      <c r="H137" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="inlineStr">
+        <is>
+          <t>textil completo con colores y formas visibles. La mejor imagen para el estudio</t>
+        </is>
+      </c>
+      <c r="F137" s="4" t="inlineStr">
+        <is>
+          <t>Anotación de la validación ciega del 2026-10-19 (data/metadata/validacion_met_cma_v2.xlsx, orden 25): principal. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G137" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H137" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
       <c r="I137" s="4" t="inlineStr">
         <is>
           <t>Head Cloth</t>
@@ -12679,7 +15301,25 @@
       <c r="Y137" s="4" t="inlineStr"/>
       <c r="Z137" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>validacion_ciega_v2</t>
+        </is>
+      </c>
+      <c r="AA137" s="4" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="AB137" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC137" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD137" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,28; textil de 2912 px de lado); colores identificables (probabilidad 0,79; 2 colores claramente distintos, 2 tonos, colorido 48); formas visibles (probabilidad 0,83; bordes cromáticos en el 12 % del textil); completitud incierta (probabilidad 0,69; compacidad 0,84, lagunas 0,0 %); estructura repetitiva. Puntaje 60.</t>
         </is>
       </c>
     </row>
@@ -12770,6 +15410,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA138" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="AB138" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC138" s="4" t="inlineStr">
+        <is>
+          <t>posterior_inca</t>
+        </is>
+      </c>
+      <c r="AD138" s="4" t="inlineStr">
+        <is>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,01; textil de 2470 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 33); formas visibles (probabilidad 0,99; bordes cromáticos en el 36 % del textil); textil completo (probabilidad 0,95; compacidad 0,97, lagunas 0,0 %); estructura no evidente. Puntaje 78.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -12858,6 +15516,24 @@
           <t>revision_manual_cma</t>
         </is>
       </c>
+      <c r="AA139" s="4" t="n">
+        <v>78.09999999999999</v>
+      </c>
+      <c r="AB139" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC139" s="4" t="inlineStr">
+        <is>
+          <t>posterior_inca</t>
+        </is>
+      </c>
+      <c r="AD139" s="4" t="inlineStr">
+        <is>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 1,86; textil de 2462 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 2 tonos, colorido 33); formas visibles (probabilidad 0,99; bordes cromáticos en el 33 % del textil); textil completo (probabilidad 0,96; compacidad 0,98, lagunas 0,0 %); estructura no evidente. Puntaje 78.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
@@ -12962,6 +15638,24 @@
           <t>descarte_automatico_cma</t>
         </is>
       </c>
+      <c r="AA140" s="4" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="AB140" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC140" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD140" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,55; textil de 530 px de lado); colores identificables (probabilidad 0,76; 2 colores claramente distintos, 1 tono, colorido 24); formas parcialmente visibles (probabilidad 0,52; bordes cromáticos en el 44 % del textil); textil completo (probabilidad 0,70; compacidad 0,44, lagunas 0,0 %); estructura no evidente. Puntaje 63.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -13066,6 +15760,24 @@
           <t>descarte_automatico_cma</t>
         </is>
       </c>
+      <c r="AA141" s="4" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="AB141" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC141" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD141" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,54; textil de 500 px de lado); colores identificables (probabilidad 0,77; 2 colores claramente distintos, 0 tonos, colorido 12); formas parcialmente visibles (probabilidad 0,54; bordes cromáticos en el 60 % del textil); completitud incierta (probabilidad 0,65; compacidad 0,52, lagunas 0,0 %); estructura no evidente. Puntaje 65.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
@@ -13170,6 +15882,24 @@
           <t>descarte_automatico_cma</t>
         </is>
       </c>
+      <c r="AA142" s="4" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="AB142" s="4" t="inlineStr">
+        <is>
+          <t>principal</t>
+        </is>
+      </c>
+      <c r="AC142" s="4" t="inlineStr">
+        <is>
+          <t>puntaje</t>
+        </is>
+      </c>
+      <c r="AD142" s="4" t="inlineStr">
+        <is>
+          <t>Fotografía regular (nitidez 1,17; textil de 706 px de lado); colores identificables (probabilidad 0,84; 1 color claramente distinto, 2 tonos, colorido 20); formas parcialmente visibles (probabilidad 0,66; bordes cromáticos en el 27 % del textil); completitud incierta (probabilidad 0,48; compacidad 0,35, lagunas 6,9 %); estructura simétrica. Puntaje 69.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -13274,6 +16004,24 @@
           <t>descarte_automatico_cma</t>
         </is>
       </c>
+      <c r="AA143" s="4" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="AB143" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC143" s="4" t="inlineStr">
+        <is>
+          <t>posterior_inca</t>
+        </is>
+      </c>
+      <c r="AD143" s="4" t="inlineStr">
+        <is>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 1,84; textil de 2602 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 2 tonos, colorido 48); formas visibles (probabilidad 0,98; bordes cromáticos en el 39 % del textil); textil completo (probabilidad 0,97; compacidad 0,83, lagunas 0,0 %); estructura simétrica. Puntaje 81.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
@@ -13378,6 +16126,24 @@
           <t>descarte_automatico_cma</t>
         </is>
       </c>
+      <c r="AA144" s="4" t="n">
+        <v>86.59999999999999</v>
+      </c>
+      <c r="AB144" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC144" s="4" t="inlineStr">
+        <is>
+          <t>posterior_inca</t>
+        </is>
+      </c>
+      <c r="AD144" s="4" t="inlineStr">
+        <is>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía regular (nitidez 0,92; textil de 3022 px de lado); colores identificables (probabilidad 1,00; 4 colores claramente distintos, 3 tonos, colorido 64); formas visibles (probabilidad 1,00; bordes cromáticos en el 64 % del textil); textil completo (probabilidad 0,99; compacidad 0,95, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 87.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -13482,6 +16248,24 @@
           <t>descarte_automatico_cma</t>
         </is>
       </c>
+      <c r="AA145" s="4" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="AB145" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC145" s="4" t="inlineStr">
+        <is>
+          <t>posterior_inca</t>
+        </is>
+      </c>
+      <c r="AD145" s="4" t="inlineStr">
+        <is>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía regular (nitidez 0,92; textil de 2405 px de lado); colores identificables (probabilidad 1,00; 4 colores claramente distintos, 3 tonos, colorido 63); formas visibles (probabilidad 1,00; bordes cromáticos en el 60 % del textil); textil completo (probabilidad 0,98; compacidad 0,94, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 84.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -13586,6 +16370,24 @@
           <t>descarte_automatico_cma</t>
         </is>
       </c>
+      <c r="AA146" s="4" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="AB146" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC146" s="4" t="inlineStr">
+        <is>
+          <t>posterior_inca</t>
+        </is>
+      </c>
+      <c r="AD146" s="4" t="inlineStr">
+        <is>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía deficiente (nitidez 0,89; textil de 2270 px de lado); colores identificables (probabilidad 1,00; 4 colores claramente distintos, 3 tonos, colorido 65); formas visibles (probabilidad 0,99; bordes cromáticos en el 62 % del textil); textil completo (probabilidad 0,92; compacidad 0,96, lagunas 0,1 %); estructura repetitiva y simétrica. Puntaje 79.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -13690,9 +16492,27 @@
           <t>descarte_automatico_cma</t>
         </is>
       </c>
+      <c r="AA147" s="4" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="AB147" s="4" t="inlineStr">
+        <is>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="AC147" s="4" t="inlineStr">
+        <is>
+          <t>posterior_inca</t>
+        </is>
+      </c>
+      <c r="AD147" s="4" t="inlineStr">
+        <is>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía deficiente (nitidez 0,89; textil de 3181 px de lado); colores identificables (probabilidad 0,77; 5 colores claramente distintos, 2 tonos, colorido 39); formas parcialmente visibles (probabilidad 0,65; bordes cromáticos en el 21 % del textil); textil incompleto (probabilidad 0,37; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 53.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z147"/>
+  <autoFilter ref="A1:AD147"/>
   <dataValidations count="2">
     <dataValidation sqref="C2:C147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"principal,secundario,descartados,revisar"</formula1>

</xml_diff>

<commit_message>
Aplica la revision de MET y CMA con el criterio v2
El revisor decidio los 94 registros de revision_criterio_v2_met_cma.xlsx; se
trasladaron con src/imagenes/revision_v2.py (54 cambios y 40 confirmaciones con
motivo nuevo, sin contradicciones):

- MET: 25 de secundario y 2 de descartados suben a principal; los 7 pendientes
  se resuelven (6 descartados, 1 secundario). MET queda en 130/25/65/0.
- CMA: 8 de secundario y 5 de descartados suben a principal; 5 de secundario
  pasan a descartados y 2 descartados a secundario. CMA queda en 104/4/38.

Cada fila conserva la decision anterior en la observacion.
</commit_message>
<xml_diff>
--- a/data/metadata/cma_revision_manual_v2.xlsx
+++ b/data/metadata/cma_revision_manual_v2.xlsx
@@ -10088,18 +10088,34 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E90" s="4" t="inlineStr"/>
-      <c r="F90" s="4" t="inlineStr"/>
-      <c r="G90" s="4" t="inlineStr"/>
-      <c r="H90" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto con formas y colores visibles</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 68): principal. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I90" s="4" t="inlineStr">
         <is>
           <t>Three Border Fragments</t>
@@ -10159,7 +10175,7 @@
       <c r="Y90" s="4" t="inlineStr"/>
       <c r="Z90" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA90" s="4" t="n">
@@ -10194,18 +10210,34 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E91" s="4" t="inlineStr"/>
-      <c r="F91" s="4" t="inlineStr"/>
-      <c r="G91" s="4" t="inlineStr"/>
-      <c r="H91" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto con formas y colores visibles</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 67): principal. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
           <t>Three Border Fragments</t>
@@ -10265,7 +10297,7 @@
       <c r="Y91" s="4" t="inlineStr"/>
       <c r="Z91" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA91" s="4" t="n">
@@ -10300,18 +10332,34 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E92" s="4" t="inlineStr"/>
-      <c r="F92" s="4" t="inlineStr"/>
-      <c r="G92" s="4" t="inlineStr"/>
-      <c r="H92" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto con formas y colores visibles</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 66): principal. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I92" s="4" t="inlineStr">
         <is>
           <t>Three Border Fragments</t>
@@ -10371,7 +10419,7 @@
       <c r="Y92" s="4" t="inlineStr"/>
       <c r="Z92" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA92" s="4" t="n">
@@ -10406,18 +10454,34 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E93" s="4" t="inlineStr"/>
-      <c r="F93" s="4" t="inlineStr"/>
-      <c r="G93" s="4" t="inlineStr"/>
-      <c r="H93" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>Textil incompleto con colores y formas visibles</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 63): principal. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I93" s="4" t="inlineStr">
         <is>
           <t>Three Border Fragments</t>
@@ -10477,7 +10541,7 @@
       <c r="Y93" s="4" t="inlineStr"/>
       <c r="Z93" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA93" s="4" t="n">
@@ -10512,18 +10576,34 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>descartados</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E94" s="4" t="inlineStr"/>
-      <c r="F94" s="4" t="inlineStr"/>
-      <c r="G94" s="4" t="inlineStr"/>
-      <c r="H94" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>textil sin formas y colores visibles</t>
+        </is>
+      </c>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 64): descartados. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I94" s="4" t="inlineStr">
         <is>
           <t>Inka Khipu (Fiber Recording Device)</t>
@@ -10583,7 +10663,7 @@
       <c r="Y94" s="4" t="inlineStr"/>
       <c r="Z94" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA94" s="4" t="n">
@@ -10740,18 +10820,34 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>descartados</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E96" s="4" t="inlineStr"/>
-      <c r="F96" s="4" t="inlineStr"/>
-      <c r="G96" s="4" t="inlineStr"/>
-      <c r="H96" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>textil sin colores visibles</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 62): descartados. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I96" s="4" t="inlineStr">
         <is>
           <t>Band</t>
@@ -10811,7 +10907,7 @@
       <c r="Y96" s="4" t="inlineStr"/>
       <c r="Z96" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA96" s="4" t="n">
@@ -10968,18 +11064,34 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E98" s="4" t="inlineStr"/>
-      <c r="F98" s="4" t="inlineStr"/>
-      <c r="G98" s="4" t="inlineStr"/>
-      <c r="H98" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>textil completo con figuras y colores visibles</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 72): principal. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I98" s="4" t="inlineStr">
         <is>
           <t>Four-Cornered Hat</t>
@@ -11039,7 +11151,7 @@
       <c r="Y98" s="4" t="inlineStr"/>
       <c r="Z98" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA98" s="4" t="n">
@@ -11074,18 +11186,34 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E99" s="4" t="inlineStr"/>
-      <c r="F99" s="4" t="inlineStr"/>
-      <c r="G99" s="4" t="inlineStr"/>
-      <c r="H99" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>textil completo con figuras y colores visibles</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 70): principal. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
           <t>Four-Cornered Hat</t>
@@ -11145,7 +11273,7 @@
       <c r="Y99" s="4" t="inlineStr"/>
       <c r="Z99" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA99" s="4" t="n">
@@ -11180,18 +11308,34 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E100" s="4" t="inlineStr"/>
-      <c r="F100" s="4" t="inlineStr"/>
-      <c r="G100" s="4" t="inlineStr"/>
-      <c r="H100" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>Textil completo con formas y colores visibles</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 65): principal. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I100" s="4" t="inlineStr">
         <is>
           <t>Four-Cornered Hat</t>
@@ -11251,7 +11395,7 @@
       <c r="Y100" s="4" t="inlineStr"/>
       <c r="Z100" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA100" s="4" t="n">
@@ -11408,18 +11552,34 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>descartados</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E102" s="4" t="inlineStr"/>
-      <c r="F102" s="4" t="inlineStr"/>
-      <c r="G102" s="4" t="inlineStr"/>
-      <c r="H102" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>es muñeco</t>
+        </is>
+      </c>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 71): descartados. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I102" s="4" t="inlineStr">
         <is>
           <t>Male Figure with Modern Additions</t>
@@ -11479,7 +11639,7 @@
       <c r="Y102" s="4" t="inlineStr"/>
       <c r="Z102" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA102" s="4" t="n">
@@ -11758,18 +11918,34 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E105" s="4" t="inlineStr"/>
-      <c r="F105" s="4" t="inlineStr"/>
-      <c r="G105" s="4" t="inlineStr"/>
-      <c r="H105" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>textil completo con figuras y colores visibles</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 73): principal. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
           <t>Four-Cornered Hat</t>
@@ -11829,7 +12005,7 @@
       <c r="Y105" s="4" t="inlineStr"/>
       <c r="Z105" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA105" s="4" t="n">
@@ -11986,18 +12162,34 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>descartados</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E107" s="4" t="inlineStr"/>
-      <c r="F107" s="4" t="inlineStr"/>
-      <c r="G107" s="4" t="inlineStr"/>
-      <c r="H107" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr">
+        <is>
+          <t>textil sin figuras visibles</t>
+        </is>
+      </c>
+      <c r="F107" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 69): descartados. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G107" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H107" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
           <t>Turban</t>
@@ -12057,7 +12249,7 @@
       <c r="Y107" s="4" t="inlineStr"/>
       <c r="Z107" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA107" s="4" t="n">
@@ -12092,18 +12284,34 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>secundario</t>
+          <t>descartados</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E108" s="4" t="inlineStr"/>
-      <c r="F108" s="4" t="inlineStr"/>
-      <c r="G108" s="4" t="inlineStr"/>
-      <c r="H108" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="inlineStr">
+        <is>
+          <t>textil sin figuras visibles</t>
+        </is>
+      </c>
+      <c r="F108" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 74): descartados. Decisión anterior: secundario (aceptar_secundario).</t>
+        </is>
+      </c>
+      <c r="G108" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H108" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I108" s="4" t="inlineStr">
         <is>
           <t>Padded Hat</t>
@@ -12163,7 +12371,7 @@
       <c r="Y108" s="4" t="inlineStr"/>
       <c r="Z108" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA108" s="4" t="n">
@@ -12203,13 +12411,29 @@
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E109" s="4" t="inlineStr"/>
-      <c r="F109" s="4" t="inlineStr"/>
-      <c r="G109" s="4" t="inlineStr"/>
-      <c r="H109" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>No es textil andino</t>
+        </is>
+      </c>
+      <c r="F109" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 75): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G109" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
           <t>Head Cloth</t>
@@ -12269,7 +12493,7 @@
       <c r="Y109" s="4" t="inlineStr"/>
       <c r="Z109" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA109" s="4" t="n">
@@ -12521,13 +12745,29 @@
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E112" s="4" t="inlineStr"/>
-      <c r="F112" s="4" t="inlineStr"/>
-      <c r="G112" s="4" t="inlineStr"/>
-      <c r="H112" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="inlineStr">
+        <is>
+          <t>textil sin formas y colores visibles</t>
+        </is>
+      </c>
+      <c r="F112" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 77): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G112" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H112" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I112" s="4" t="inlineStr">
         <is>
           <t>Headcloth</t>
@@ -12587,7 +12827,7 @@
       <c r="Y112" s="4" t="inlineStr"/>
       <c r="Z112" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA112" s="4" t="n">
@@ -12627,13 +12867,29 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr"/>
-      <c r="F113" s="4" t="inlineStr"/>
-      <c r="G113" s="4" t="inlineStr"/>
-      <c r="H113" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E113" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto</t>
+        </is>
+      </c>
+      <c r="F113" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 90): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G113" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H113" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
           <t>Mummy Bundle Turban</t>
@@ -12693,7 +12949,7 @@
       <c r="Y113" s="4" t="inlineStr"/>
       <c r="Z113" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA113" s="4" t="n">
@@ -12733,13 +12989,29 @@
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E114" s="4" t="inlineStr"/>
-      <c r="F114" s="4" t="inlineStr"/>
-      <c r="G114" s="4" t="inlineStr"/>
-      <c r="H114" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="inlineStr">
+        <is>
+          <t>son muñecos</t>
+        </is>
+      </c>
+      <c r="F114" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 91): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G114" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H114" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I114" s="4" t="inlineStr">
         <is>
           <t>Border Fragment</t>
@@ -12799,7 +13071,7 @@
       <c r="Y114" s="4" t="inlineStr"/>
       <c r="Z114" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA114" s="4" t="n">
@@ -12961,13 +13233,29 @@
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E116" s="4" t="inlineStr"/>
-      <c r="F116" s="4" t="inlineStr"/>
-      <c r="G116" s="4" t="inlineStr"/>
-      <c r="H116" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>textil con colores visibles</t>
+        </is>
+      </c>
+      <c r="F116" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 83): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G116" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H116" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I116" s="4" t="inlineStr">
         <is>
           <t>Border Fragment with Birds and Flowers</t>
@@ -13027,7 +13315,7 @@
       <c r="Y116" s="4" t="inlineStr"/>
       <c r="Z116" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA116" s="4" t="n">
@@ -13067,13 +13355,29 @@
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E117" s="4" t="inlineStr"/>
-      <c r="F117" s="4" t="inlineStr"/>
-      <c r="G117" s="4" t="inlineStr"/>
-      <c r="H117" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr">
+        <is>
+          <t>textil con colores visibles</t>
+        </is>
+      </c>
+      <c r="F117" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 86): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G117" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I117" s="4" t="inlineStr">
         <is>
           <t>Border Fragment with Birds and Flowers</t>
@@ -13133,7 +13437,7 @@
       <c r="Y117" s="4" t="inlineStr"/>
       <c r="Z117" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA117" s="4" t="n">
@@ -13173,13 +13477,29 @@
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E118" s="4" t="inlineStr"/>
-      <c r="F118" s="4" t="inlineStr"/>
-      <c r="G118" s="4" t="inlineStr"/>
-      <c r="H118" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="inlineStr">
+        <is>
+          <t>textil con colores visibles</t>
+        </is>
+      </c>
+      <c r="F118" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 84): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G118" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H118" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I118" s="4" t="inlineStr">
         <is>
           <t>Border Fragment with Birds and Flowers</t>
@@ -13239,7 +13559,7 @@
       <c r="Y118" s="4" t="inlineStr"/>
       <c r="Z118" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA118" s="4" t="n">
@@ -13380,18 +13700,34 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E120" s="4" t="inlineStr"/>
-      <c r="F120" s="4" t="inlineStr"/>
-      <c r="G120" s="4" t="inlineStr"/>
-      <c r="H120" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto con colores y formas visibles</t>
+        </is>
+      </c>
+      <c r="F120" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 78): principal. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G120" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H120" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I120" s="4" t="inlineStr">
         <is>
           <t>Band with Trophy Heads</t>
@@ -13451,7 +13787,7 @@
       <c r="Y120" s="4" t="inlineStr"/>
       <c r="Z120" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA120" s="4" t="n">
@@ -13486,18 +13822,34 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E121" s="4" t="inlineStr"/>
-      <c r="F121" s="4" t="inlineStr"/>
-      <c r="G121" s="4" t="inlineStr"/>
-      <c r="H121" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto con colores y formas visibles</t>
+        </is>
+      </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 76): principal. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G121" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I121" s="4" t="inlineStr">
         <is>
           <t>Lower Border of a Garment</t>
@@ -13557,7 +13909,7 @@
       <c r="Y121" s="4" t="inlineStr"/>
       <c r="Z121" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA121" s="4" t="n">
@@ -13597,13 +13949,29 @@
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E122" s="4" t="inlineStr"/>
-      <c r="F122" s="4" t="inlineStr"/>
-      <c r="G122" s="4" t="inlineStr"/>
-      <c r="H122" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto</t>
+        </is>
+      </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 82): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H122" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I122" s="4" t="inlineStr">
         <is>
           <t>Textile</t>
@@ -13663,7 +14031,7 @@
       <c r="Y122" s="4" t="inlineStr"/>
       <c r="Z122" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA122" s="4" t="n">
@@ -13703,13 +14071,29 @@
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E123" s="4" t="inlineStr"/>
-      <c r="F123" s="4" t="inlineStr"/>
-      <c r="G123" s="4" t="inlineStr"/>
-      <c r="H123" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>textil con colores visibles</t>
+        </is>
+      </c>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 87): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G123" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
           <t>Textile</t>
@@ -13769,7 +14153,7 @@
       <c r="Y123" s="4" t="inlineStr"/>
       <c r="Z123" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA123" s="4" t="n">
@@ -13804,18 +14188,34 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E124" s="4" t="inlineStr"/>
-      <c r="F124" s="4" t="inlineStr"/>
-      <c r="G124" s="4" t="inlineStr"/>
-      <c r="H124" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto con colores y formas visibles</t>
+        </is>
+      </c>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 89): principal. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H124" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I124" s="4" t="inlineStr">
         <is>
           <t>Fragments of a Belt</t>
@@ -13875,7 +14275,7 @@
       <c r="Y124" s="4" t="inlineStr"/>
       <c r="Z124" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA124" s="4" t="n">
@@ -13910,18 +14310,34 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E125" s="4" t="inlineStr"/>
-      <c r="F125" s="4" t="inlineStr"/>
-      <c r="G125" s="4" t="inlineStr"/>
-      <c r="H125" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto con colores y formas visibles</t>
+        </is>
+      </c>
+      <c r="F125" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 81): principal. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G125" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H125" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I125" s="4" t="inlineStr">
         <is>
           <t>Fragment of a Belt</t>
@@ -13981,7 +14397,7 @@
       <c r="Y125" s="4" t="inlineStr"/>
       <c r="Z125" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA125" s="4" t="n">
@@ -14016,18 +14432,34 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E126" s="4" t="inlineStr"/>
-      <c r="F126" s="4" t="inlineStr"/>
-      <c r="G126" s="4" t="inlineStr"/>
-      <c r="H126" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="inlineStr">
+        <is>
+          <t>textil incompleto con colores y formas visibles</t>
+        </is>
+      </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 79): principal. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H126" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I126" s="4" t="inlineStr">
         <is>
           <t>Fragment of a Belt</t>
@@ -14087,7 +14519,7 @@
       <c r="Y126" s="4" t="inlineStr"/>
       <c r="Z126" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA126" s="4" t="n">
@@ -14233,13 +14665,29 @@
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E128" s="4" t="inlineStr"/>
-      <c r="F128" s="4" t="inlineStr"/>
-      <c r="G128" s="4" t="inlineStr"/>
-      <c r="H128" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="inlineStr">
+        <is>
+          <t>textil sin colores visibles</t>
+        </is>
+      </c>
+      <c r="F128" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 93): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G128" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H128" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I128" s="4" t="inlineStr">
         <is>
           <t>Band with Tassels</t>
@@ -14299,7 +14747,7 @@
       <c r="Y128" s="4" t="inlineStr"/>
       <c r="Z128" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA128" s="4" t="n">
@@ -14456,18 +14904,34 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>secundario</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E130" s="4" t="inlineStr"/>
-      <c r="F130" s="4" t="inlineStr"/>
-      <c r="G130" s="4" t="inlineStr"/>
-      <c r="H130" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="inlineStr">
+        <is>
+          <t>textil con colores visibles</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 80): secundario. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G130" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H130" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I130" s="4" t="inlineStr">
         <is>
           <t>Textile Fragment</t>
@@ -14527,7 +14991,7 @@
       <c r="Y130" s="4" t="inlineStr"/>
       <c r="Z130" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA130" s="4" t="n">
@@ -14562,18 +15026,34 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>descartados</t>
+          <t>secundario</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E131" s="4" t="inlineStr"/>
-      <c r="F131" s="4" t="inlineStr"/>
-      <c r="G131" s="4" t="inlineStr"/>
-      <c r="H131" s="4" t="inlineStr"/>
+          <t>mover</t>
+        </is>
+      </c>
+      <c r="E131" s="4" t="inlineStr">
+        <is>
+          <t>textil con colores visibles</t>
+        </is>
+      </c>
+      <c r="F131" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 88): secundario. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G131" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H131" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
           <t>Textile Fragment</t>
@@ -14633,7 +15113,7 @@
       <c r="Y131" s="4" t="inlineStr"/>
       <c r="Z131" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA131" s="4" t="n">
@@ -14673,13 +15153,29 @@
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E132" s="4" t="inlineStr"/>
-      <c r="F132" s="4" t="inlineStr"/>
-      <c r="G132" s="4" t="inlineStr"/>
-      <c r="H132" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="inlineStr">
+        <is>
+          <t>textil sin formas visibles</t>
+        </is>
+      </c>
+      <c r="F132" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 94): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G132" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H132" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I132" s="4" t="inlineStr">
         <is>
           <t>Loose Textile Fragments</t>
@@ -14739,7 +15235,7 @@
       <c r="Y132" s="4" t="inlineStr"/>
       <c r="Z132" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA132" s="4" t="n">
@@ -14885,13 +15381,29 @@
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E134" s="4" t="inlineStr"/>
-      <c r="F134" s="4" t="inlineStr"/>
-      <c r="G134" s="4" t="inlineStr"/>
-      <c r="H134" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="inlineStr">
+        <is>
+          <t>textil sin colores visibles</t>
+        </is>
+      </c>
+      <c r="F134" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 92): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G134" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H134" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I134" s="4" t="inlineStr">
         <is>
           <t>Band</t>
@@ -14951,7 +15463,7 @@
       <c r="Y134" s="4" t="inlineStr"/>
       <c r="Z134" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA134" s="4" t="n">
@@ -14991,13 +15503,29 @@
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>mantener</t>
-        </is>
-      </c>
-      <c r="E135" s="4" t="inlineStr"/>
-      <c r="F135" s="4" t="inlineStr"/>
-      <c r="G135" s="4" t="inlineStr"/>
-      <c r="H135" s="4" t="inlineStr"/>
+          <t>descartar</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>textil con colores visibles</t>
+        </is>
+      </c>
+      <c r="F135" s="4" t="inlineStr">
+        <is>
+          <t>Revisión con el criterio v2 del 2026-10-20 (data/metadata/revision_criterio_v2_met_cma.xlsx, orden 85): descartados. Decisión anterior: descartados (descartar_baja_calidad).</t>
+        </is>
+      </c>
+      <c r="G135" s="4" t="inlineStr">
+        <is>
+          <t>Henry Sánchez</t>
+        </is>
+      </c>
+      <c r="H135" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
       <c r="I135" s="4" t="inlineStr">
         <is>
           <t>Band (Headband?)</t>
@@ -15057,7 +15585,7 @@
       <c r="Y135" s="4" t="inlineStr"/>
       <c r="Z135" s="4" t="inlineStr">
         <is>
-          <t>revision_manual_cma</t>
+          <t>revision_criterio_v2</t>
         </is>
       </c>
       <c r="AA135" s="4" t="n">

</xml_diff>

<commit_message>
Calibra el puntaje con AIC, MET y CMA y marca posibles figurillas
- Calibracion conjunta: el modelo calibrado solo con AIC no generalizaba a MET
  (separacion util/resto 0,49 con las etiquetas del criterio v2). Ahora calibran
  todas las decisiones humanas de AIC y, de MET y CMA, solo las tomadas con el
  criterio v2 (validacion ciega y revision v2): 316 + 51 + 35 registros. Fuera
  de pliegue, util/resto queda en 0,91 (AIC), 0,76 (MET) y 0,83 (CMA). La
  validacion cruzada se estratifica por fuente; el informe pasa a
  outputs/reports/aptitud_calibracion_v2.md, con cifras por fuente.
- Posible figurilla: siete piezas que el revisor descarto como munecos se
  titulan "..., Figure". Por prudencia la regla no descarta: "Figure" en
  singular, sin "with", "of"... delante, solo manda la imagen a revisar, para no
  quitar textiles con figuras representadas.
- La ficha de los workbooks se actualiza con el modelo nuevo sin tocar ninguna
  decision ni motivo del revisor.
</commit_message>
<xml_diff>
--- a/data/metadata/cma_revision_manual_v2.xlsx
+++ b/data/metadata/cma_revision_manual_v2.xlsx
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>55.6</v>
+        <v>63.5</v>
       </c>
       <c r="AB2" s="4" t="inlineStr">
         <is>
@@ -849,7 +849,7 @@
       </c>
       <c r="AD2" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,22; textil de 1576 px de lado); colores identificables (probabilidad 0,73; 3 colores claramente distintos, 2 tonos, colorido 25); formas visibles (probabilidad 0,72; bordes cromáticos en el 30 % del textil); textil incompleto (probabilidad 0,33; compacidad 0,67, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 56.</t>
+          <t>Fotografía regular (nitidez 1,22; textil de 1576 px de lado); colores identificables (probabilidad 0,83; 3 colores claramente distintos, 2 tonos, colorido 25); formas visibles (probabilidad 0,84; bordes cromáticos en el 30 % del textil); completitud incierta (probabilidad 0,41; compacidad 0,67, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 64.</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>60.6</v>
+        <v>74</v>
       </c>
       <c r="AB3" s="4" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
       </c>
       <c r="AD3" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,79; textil de 2752 px de lado); colores identificables (probabilidad 0,79; 1 color claramente distinto, 0 tonos, colorido 18); formas visibles (probabilidad 0,89; bordes cromáticos en el 23 % del textil); completitud incierta (probabilidad 0,64; compacidad 0,95, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 61.</t>
+          <t>Fotografía buena (nitidez 1,79; textil de 2752 px de lado); colores identificables (probabilidad 0,81; 1 color claramente distinto, 0 tonos, colorido 18); formas visibles (probabilidad 0,93; bordes cromáticos en el 23 % del textil); completitud incierta (probabilidad 0,56; compacidad 0,95, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 74.</t>
         </is>
       </c>
     </row>
@@ -1047,21 +1047,21 @@
         </is>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>45.4</v>
+        <v>53.8</v>
       </c>
       <c r="AB4" s="4" t="inlineStr">
         <is>
-          <t>descartar</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC4" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD4" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,60; textil de 2024 px de lado); colores parcialmente identificables (probabilidad 0,59; 2 colores claramente distintos, 1 tono, colorido 15); formas parcialmente visibles (probabilidad 0,63; bordes cromáticos en el 13 % del textil); textil incompleto (probabilidad 0,29; compacidad 0,54, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 45.</t>
+          <t>Fotografía buena (nitidez 1,60; textil de 2024 px de lado); colores parcialmente identificables (probabilidad 0,66; 2 colores claramente distintos, 1 tono, colorido 15); formas visibles (probabilidad 0,70; bordes cromáticos en el 13 % del textil); textil incompleto (probabilidad 0,29; compacidad 0,54, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 54.</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
         </is>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>60.9</v>
+        <v>79</v>
       </c>
       <c r="AB5" s="4" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="AD5" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,40; textil de 2152 px de lado); colores identificables (probabilidad 0,81; 1 color claramente distinto, 1 tono, colorido 17); formas visibles (probabilidad 0,87; bordes cromáticos en el 5 % del textil); textil completo (probabilidad 0,71; compacidad 0,92, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 61.</t>
+          <t>Fotografía regular (nitidez 1,40; textil de 2152 px de lado); colores identificables (probabilidad 0,84; 1 color claramente distinto, 1 tono, colorido 17); formas visibles (probabilidad 0,89; bordes cromáticos en el 5 % del textil); completitud incierta (probabilidad 0,68; compacidad 0,92, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 79.</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
         </is>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>87.8</v>
+        <v>97</v>
       </c>
       <c r="AB6" s="4" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="AD6" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,60; textil de 1360 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 38); formas visibles (probabilidad 0,99; bordes cromáticos en el 49 % del textil); textil completo (probabilidad 0,97; compacidad 0,90, lagunas 0,0 %); estructura repetitiva. Puntaje 88 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 1,60; textil de 1360 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 38); formas visibles (probabilidad 0,99; bordes cromáticos en el 49 % del textil); textil completo (probabilidad 0,97; compacidad 0,90, lagunas 0,0 %); estructura repetitiva. Puntaje 97 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>84.59999999999999</v>
+        <v>83.5</v>
       </c>
       <c r="AB7" s="4" t="inlineStr">
         <is>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="AD7" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,17; textil de 2199 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 35); formas visibles (probabilidad 0,99; bordes cromáticos en el 52 % del textil); textil completo (probabilidad 0,84; compacidad 0,76, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 85 (imagen de referencia sugerida).</t>
+          <t>Fotografía regular (nitidez 1,17; textil de 2199 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 35); formas visibles (probabilidad 1,00; bordes cromáticos en el 52 % del textil); textil completo (probabilidad 0,84; compacidad 0,76, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 83.</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>82.40000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="AB8" s="4" t="inlineStr">
         <is>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="AD8" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,14; textil de 1404 px de lado); colores identificables (probabilidad 0,96; 3 colores claramente distintos, 3 tonos, colorido 36); formas visibles (probabilidad 0,93; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,82; compacidad 0,76, lagunas 0,0 %); estructura repetitiva. Puntaje 82 (imagen de referencia sugerida).</t>
+          <t>Fotografía regular (nitidez 1,14; textil de 1404 px de lado); colores identificables (probabilidad 0,96; 3 colores claramente distintos, 3 tonos, colorido 36); formas visibles (probabilidad 0,95; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,86; compacidad 0,76, lagunas 0,0 %); estructura repetitiva. Puntaje 90 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>77.59999999999999</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="AB9" s="4" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="AD9" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,15; textil de 1375 px de lado); colores identificables (probabilidad 0,94; 3 colores claramente distintos, 2 tonos, colorido 36); formas visibles (probabilidad 0,89; bordes cromáticos en el 45 % del textil); textil completo (probabilidad 0,79; compacidad 0,78, lagunas 0,0 %); estructura repetitiva. Puntaje 78 (imagen de referencia sugerida).</t>
+          <t>Fotografía regular (nitidez 1,15; textil de 1375 px de lado); colores identificables (probabilidad 0,94; 3 colores claramente distintos, 2 tonos, colorido 36); formas visibles (probabilidad 0,92; bordes cromáticos en el 45 % del textil); textil completo (probabilidad 0,84; compacidad 0,78, lagunas 0,0 %); estructura repetitiva. Puntaje 88 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1683,7 @@
         </is>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>80.59999999999999</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="AB10" s="4" t="inlineStr">
         <is>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="AD10" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,10; textil de 1325 px de lado); colores identificables (probabilidad 0,94; 2 colores claramente distintos, 3 tonos, colorido 34); formas visibles (probabilidad 0,91; bordes cromáticos en el 49 % del textil); textil completo (probabilidad 0,78; compacidad 0,73, lagunas 0,2 %); estructura repetitiva. Puntaje 81 (imagen de referencia sugerida).</t>
+          <t>Fotografía regular (nitidez 1,10; textil de 1325 px de lado); colores identificables (probabilidad 0,95; 2 colores claramente distintos, 3 tonos, colorido 34); formas visibles (probabilidad 0,93; bordes cromáticos en el 49 % del textil); textil completo (probabilidad 0,78; compacidad 0,73, lagunas 0,2 %); estructura repetitiva. Puntaje 85 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>83.2</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="AB11" s="4" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="AD11" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,13; textil de 1297 px de lado); colores identificables (probabilidad 0,95; 3 colores claramente distintos, 3 tonos, colorido 37); formas visibles (probabilidad 0,92; bordes cromáticos en el 52 % del textil); textil completo (probabilidad 0,80; compacidad 0,72, lagunas 0,0 %); estructura repetitiva. Puntaje 83 (imagen de referencia sugerida).</t>
+          <t>Fotografía regular (nitidez 1,13; textil de 1297 px de lado); colores identificables (probabilidad 0,96; 3 colores claramente distintos, 3 tonos, colorido 37); formas visibles (probabilidad 0,95; bordes cromáticos en el 52 % del textil); textil completo (probabilidad 0,85; compacidad 0,72, lagunas 0,0 %); estructura repetitiva. Puntaje 89 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -1895,21 +1895,21 @@
         </is>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>71.8</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="AB12" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC12" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD12" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,27; textil de 2350 px de lado); colores identificables (probabilidad 0,97; 3 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,98; bordes cromáticos en el 41 % del textil); completitud incierta (probabilidad 0,58; compacidad 0,93, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 72.</t>
+          <t>Fotografía regular (nitidez 1,27; textil de 2350 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,99; bordes cromáticos en el 41 % del textil); completitud incierta (probabilidad 0,55; compacidad 0,93, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 67.</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
         </is>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>75</v>
+        <v>81.8</v>
       </c>
       <c r="AB13" s="4" t="inlineStr">
         <is>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="AD13" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,27; textil de 1544 px de lado); colores identificables (probabilidad 0,95; 3 colores claramente distintos, 3 tonos, colorido 41); formas visibles (probabilidad 0,94; bordes cromáticos en el 40 % del textil); completitud incierta (probabilidad 0,69; compacidad 0,92, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 75.</t>
+          <t>Fotografía regular (nitidez 1,27; textil de 1544 px de lado); colores identificables (probabilidad 0,97; 3 colores claramente distintos, 3 tonos, colorido 41); formas visibles (probabilidad 0,97; bordes cromáticos en el 40 % del textil); textil completo (probabilidad 0,70; compacidad 0,92, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 82.</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
         </is>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>67.2</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="AB14" s="4" t="inlineStr">
         <is>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="AD14" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,24; textil de 1551 px de lado); colores identificables (probabilidad 0,88; 3 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,86; bordes cromáticos en el 40 % del textil); completitud incierta (probabilidad 0,56; compacidad 0,86, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 67.</t>
+          <t>Fotografía regular (nitidez 1,24; textil de 1551 px de lado); colores identificables (probabilidad 0,92; 3 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,93; bordes cromáticos en el 40 % del textil); completitud incierta (probabilidad 0,58; compacidad 0,86, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva. Puntaje 75.</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2213,7 @@
         </is>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>63.5</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="AB15" s="4" t="inlineStr">
         <is>
@@ -2227,7 +2227,7 @@
       </c>
       <c r="AD15" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,31; textil de 1549 px de lado); colores identificables (probabilidad 0,84; 3 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,83; bordes cromáticos en el 38 % del textil); completitud incierta (probabilidad 0,48; compacidad 0,85, lagunas 0,1 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
+          <t>Fotografía regular (nitidez 1,31; textil de 1549 px de lado); colores identificables (probabilidad 0,91; 3 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,91; bordes cromáticos en el 38 % del textil); completitud incierta (probabilidad 0,52; compacidad 0,85, lagunas 0,1 %, el título dice «fragment»); estructura no evidente. Puntaje 72.</t>
         </is>
       </c>
     </row>
@@ -2319,21 +2319,21 @@
         </is>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>62.9</v>
+        <v>52.9</v>
       </c>
       <c r="AB16" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC16" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD16" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,88; textil de 1702 px de lado); colores identificables (probabilidad 0,87; 2 colores claramente distintos, 2 tonos, colorido 29); formas visibles (probabilidad 0,91; bordes cromáticos en el 26 % del textil); textil incompleto (probabilidad 0,26; compacidad 0,74, lagunas 2,2 %, el título dice «fragment»); estructura repetitiva. Puntaje 63.</t>
+          <t>Fotografía buena (nitidez 1,88; textil de 1702 px de lado); colores identificables (probabilidad 0,92; 2 colores claramente distintos, 2 tonos, colorido 29); formas visibles (probabilidad 0,94; bordes cromáticos en el 26 % del textil); textil incompleto (probabilidad 0,21; compacidad 0,74, lagunas 2,2 %, el título dice «fragment»); estructura repetitiva. Puntaje 53.</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2425,7 @@
         </is>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>66.5</v>
+        <v>84.3</v>
       </c>
       <c r="AB17" s="4" t="inlineStr">
         <is>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="AD17" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,97; textil de 2643 px de lado); colores identificables (probabilidad 0,90; 1 color claramente distinto, 3 tonos, colorido 27); formas visibles (probabilidad 0,94; bordes cromáticos en el 18 % del textil); textil completo (probabilidad 0,72; compacidad 0,87, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 67.</t>
+          <t>Fotografía buena (nitidez 1,97; textil de 2643 px de lado); colores identificables (probabilidad 0,94; 1 color claramente distinto, 3 tonos, colorido 27); formas visibles (probabilidad 0,96; bordes cromáticos en el 18 % del textil); textil completo (probabilidad 0,71; compacidad 0,87, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 84.</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>72.2</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="AB18" s="4" t="inlineStr">
         <is>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="AD18" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,81; textil de 2462 px de lado); colores identificables (probabilidad 0,91; 2 colores claramente distintos, 3 tonos, colorido 26); formas visibles (probabilidad 0,92; bordes cromáticos en el 33 % del textil); textil completo (probabilidad 0,77; compacidad 0,74, lagunas 0,2 %); estructura no evidente. Puntaje 72.</t>
+          <t>Fotografía buena (nitidez 1,81; textil de 2462 px de lado); colores identificables (probabilidad 0,92; 2 colores claramente distintos, 3 tonos, colorido 26); formas visibles (probabilidad 0,95; bordes cromáticos en el 33 % del textil); textil completo (probabilidad 0,82; compacidad 0,74, lagunas 0,2 %); estructura no evidente. Puntaje 89 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>64.40000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="AB19" s="4" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
       </c>
       <c r="AD19" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,84; textil de 2697 px de lado); colores identificables (probabilidad 0,85; 2 colores claramente distintos, 1 tono, colorido 15); formas visibles (probabilidad 0,90; bordes cromáticos en el 19 % del textil); textil completo (probabilidad 0,72; compacidad 0,90, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 64.</t>
+          <t>Fotografía buena (nitidez 1,84; textil de 2697 px de lado); colores identificables (probabilidad 0,86; 2 colores claramente distintos, 1 tono, colorido 15); formas visibles (probabilidad 0,93; bordes cromáticos en el 19 % del textil); textil completo (probabilidad 0,75; compacidad 0,90, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 85.</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
         </is>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>76</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="AB20" s="4" t="inlineStr">
         <is>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="AD20" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,45; textil de 1607 px de lado); colores identificables (probabilidad 0,99; 1 color claramente distinto, 2 tonos, colorido 19); formas visibles (probabilidad 0,99; bordes cromáticos en el 21 % del textil); textil completo (probabilidad 0,97; compacidad 0,95, lagunas 0,0 %); estructura repetitiva. Puntaje 76.</t>
+          <t>Fotografía buena (nitidez 2,45; textil de 1607 px de lado); colores identificables (probabilidad 0,98; 1 color claramente distinto, 2 tonos, colorido 19); formas visibles (probabilidad 0,98; bordes cromáticos en el 21 % del textil); textil completo (probabilidad 0,96; compacidad 0,95, lagunas 0,0 %); estructura repetitiva. Puntaje 96 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2849,7 @@
         </is>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>50.2</v>
+        <v>58</v>
       </c>
       <c r="AB21" s="4" t="inlineStr">
         <is>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="AD21" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,16; textil de 2151 px de lado); colores parcialmente identificables (probabilidad 0,68; 2 colores claramente distintos, 3 tonos, colorido 38); formas visibles (probabilidad 0,70; bordes cromáticos en el 22 % del textil); textil incompleto (probabilidad 0,28; compacidad 0,67, lagunas 0,2 %, el título dice «fragment»); estructura no evidente. Puntaje 50.</t>
+          <t>Fotografía regular (nitidez 1,16; textil de 2151 px de lado); colores identificables (probabilidad 0,81; 2 colores claramente distintos, 3 tonos, colorido 38); formas visibles (probabilidad 0,82; bordes cromáticos en el 22 % del textil); textil incompleto (probabilidad 0,31; compacidad 0,67, lagunas 0,2 %, el título dice «fragment»); estructura no evidente. Puntaje 58.</t>
         </is>
       </c>
     </row>
@@ -2955,7 +2955,7 @@
         </is>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>78.40000000000001</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="AB22" s="4" t="inlineStr">
         <is>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="AD22" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 0,96; textil de 2262 px de lado); colores identificables (probabilidad 0,96; 3 colores claramente distintos, 3 tonos, colorido 51); formas visibles (probabilidad 0,95; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,85; compacidad 0,89, lagunas 3,9 %); estructura no evidente. Puntaje 78 (imagen de referencia sugerida).</t>
+          <t>Fotografía regular (nitidez 0,96; textil de 2262 px de lado); colores identificables (probabilidad 0,98; 3 colores claramente distintos, 3 tonos, colorido 51); formas visibles (probabilidad 0,97; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,93; compacidad 0,89, lagunas 3,9 %); estructura no evidente. Puntaje 94 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -3061,21 +3061,21 @@
         </is>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>77.09999999999999</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="AB23" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC23" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD23" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,34; textil de 2152 px de lado); colores parcialmente identificables (probabilidad 0,66; 3 colores claramente distintos, 3 tonos, colorido 21); formas visibles (probabilidad 0,89; bordes cromáticos en el 40 % del textil); textil incompleto (probabilidad 0,19; compacidad 0,90, lagunas 35,4 %); estructura no evidente. Puntaje 77 (imagen de referencia sugerida).</t>
+          <t>Fotografía regular (nitidez 1,34; textil de 2152 px de lado); colores identificables (probabilidad 0,86; 3 colores claramente distintos, 3 tonos, colorido 21); formas visibles (probabilidad 0,97; bordes cromáticos en el 40 % del textil); completitud incierta (probabilidad 0,48; compacidad 0,90, lagunas 35,4 %); estructura no evidente. Puntaje 65.</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
         </is>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>64.5</v>
+        <v>85.8</v>
       </c>
       <c r="AB24" s="4" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="AD24" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,49; textil de 1786 px de lado); colores identificables (probabilidad 0,84; 1 color claramente distinto, 2 tonos, colorido 36); formas visibles (probabilidad 0,83; bordes cromáticos en el 21 % del textil); textil completo (probabilidad 0,83; compacidad 0,67, lagunas 0,5 %); estructura repetitiva. Puntaje 65.</t>
+          <t>Fotografía buena (nitidez 1,49; textil de 1786 px de lado); colores identificables (probabilidad 0,85; 1 color claramente distinto, 2 tonos, colorido 36); formas visibles (probabilidad 0,83; bordes cromáticos en el 21 % del textil); textil completo (probabilidad 0,84; compacidad 0,67, lagunas 0,5 %); estructura repetitiva. Puntaje 86 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -3273,21 +3273,21 @@
         </is>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>55.7</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="AB25" s="4" t="inlineStr">
         <is>
-          <t>revisar</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="AC25" s="4" t="inlineStr">
         <is>
-          <t>zona_intermedia</t>
+          <t>puntaje</t>
         </is>
       </c>
       <c r="AD25" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 0,94; textil de 2036 px de lado); colores identificables (probabilidad 0,74; 3 colores claramente distintos, 2 tonos, colorido 34); formas visibles (probabilidad 0,77; bordes cromáticos en el 23 % del textil); textil incompleto (probabilidad 0,37; compacidad 0,88, lagunas 1,7 %, el título dice «fragment»); estructura no evidente. Puntaje 56.</t>
+          <t>Fotografía regular (nitidez 0,94; textil de 2036 px de lado); colores identificables (probabilidad 0,86; 3 colores claramente distintos, 2 tonos, colorido 34); formas visibles (probabilidad 0,90; bordes cromáticos en el 23 % del textil); completitud incierta (probabilidad 0,51; compacidad 0,88, lagunas 1,7 %, el título dice «fragment»); estructura no evidente. Puntaje 70.</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3379,7 @@
         </is>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>78.59999999999999</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="AB26" s="4" t="inlineStr">
         <is>
@@ -3393,7 +3393,7 @@
       </c>
       <c r="AD26" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,46; textil de 1769 px de lado); colores identificables (probabilidad 0,98; 1 color claramente distinto, 1 tono, colorido 19); formas visibles (probabilidad 0,98; bordes cromáticos en el 44 % del textil); textil completo (probabilidad 0,98; compacidad 0,95, lagunas 0,0 %); estructura no evidente. Puntaje 79 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 2,46; textil de 1769 px de lado); colores identificables (probabilidad 0,97; 1 color claramente distinto, 1 tono, colorido 19); formas visibles (probabilidad 0,98; bordes cromáticos en el 44 % del textil); textil completo (probabilidad 0,98; compacidad 0,95, lagunas 0,0 %); estructura no evidente. Puntaje 98 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
         </is>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>79.90000000000001</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="AB27" s="4" t="inlineStr">
         <is>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="AD27" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,01; textil de 2301 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 2 tonos, colorido 19); formas visibles (probabilidad 0,97; bordes cromáticos en el 20 % del textil); textil completo (probabilidad 0,88; toma cerrada, el contorno de la pieza no se ve); estructura repetitiva y simétrica. Puntaje 80 (imagen de referencia sugerida).</t>
+          <t>Fotografía regular (nitidez 1,01; textil de 2301 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 2 tonos, colorido 19); formas visibles (probabilidad 0,96; bordes cromáticos en el 20 % del textil); textil completo (probabilidad 0,91; toma cerrada, el contorno de la pieza no se ve); estructura repetitiva y simétrica. Puntaje 92 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>72.09999999999999</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="AB28" s="4" t="inlineStr">
         <is>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="AD28" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,18; textil de 3112 px de lado); colores identificables (probabilidad 0,97; 2 colores claramente distintos, 3 tonos, colorido 23); formas visibles (probabilidad 0,98; bordes cromáticos en el 15 % del textil); textil completo (probabilidad 0,91; compacidad 0,97, lagunas 0,0 %); estructura repetitiva. Puntaje 72.</t>
+          <t>Fotografía regular (nitidez 1,18; textil de 3112 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 3 tonos, colorido 23); formas visibles (probabilidad 0,99; bordes cromáticos en el 15 % del textil); textil completo (probabilidad 0,95; compacidad 0,97, lagunas 0,0 %); estructura repetitiva. Puntaje 95 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>79.7</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="AB29" s="4" t="inlineStr">
         <is>
@@ -3711,7 +3711,7 @@
       </c>
       <c r="AD29" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 1,00; textil de 1289 px de lado); colores identificables (probabilidad 0,98; 5 colores claramente distintos, 3 tonos, colorido 65); formas visibles (probabilidad 0,96; bordes cromáticos en el 39 % del textil); textil completo (probabilidad 0,80; compacidad 0,87, lagunas 0,0 %); estructura simétrica. Puntaje 80 (imagen de referencia sugerida).</t>
+          <t>Fotografía deficiente (nitidez 1,00; textil de 1289 px de lado); colores identificables (probabilidad 0,99; 5 colores claramente distintos, 3 tonos, colorido 65); formas visibles (probabilidad 0,97; bordes cromáticos en el 39 % del textil); textil completo (probabilidad 0,94; compacidad 0,87, lagunas 0,0 %); estructura simétrica. Puntaje 94 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3803,7 @@
         </is>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>71</v>
+        <v>94.7</v>
       </c>
       <c r="AB30" s="4" t="inlineStr">
         <is>
@@ -3817,7 +3817,7 @@
       </c>
       <c r="AD30" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,04; textil de 1962 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 0 tonos, colorido 11); formas visibles (probabilidad 0,97; bordes cromáticos en el 6 % del textil); textil completo (probabilidad 0,92; compacidad 0,98, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 71.</t>
+          <t>Fotografía regular (nitidez 1,04; textil de 1962 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 0 tonos, colorido 11); formas visibles (probabilidad 0,95; bordes cromáticos en el 6 % del textil); textil completo (probabilidad 0,96; compacidad 0,98, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 95 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>52.3</v>
+        <v>68.3</v>
       </c>
       <c r="AB31" s="4" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
       </c>
       <c r="AD31" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,48; textil de 1083 px de lado); colores identificables (probabilidad 0,73; 2 colores claramente distintos, 1 tono, colorido 53); formas parcialmente visibles (probabilidad 0,54; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,71; compacidad 0,51, lagunas 0,0 %); estructura no evidente. Puntaje 52.</t>
+          <t>Fotografía regular (nitidez 1,48; textil de 1083 px de lado); colores parcialmente identificables (probabilidad 0,69; 2 colores claramente distintos, 1 tono, colorido 53); formas parcialmente visibles (probabilidad 0,45; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,73; compacidad 0,51, lagunas 0,0 %); estructura no evidente. Puntaje 68.</t>
         </is>
       </c>
     </row>
@@ -4015,21 +4015,21 @@
         </is>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>55.9</v>
+        <v>78.5</v>
       </c>
       <c r="AB32" s="4" t="inlineStr">
         <is>
-          <t>revisar</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="AC32" s="4" t="inlineStr">
         <is>
-          <t>zona_intermedia</t>
+          <t>puntaje</t>
         </is>
       </c>
       <c r="AD32" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,81; textil de 1352 px de lado); colores identificables (probabilidad 0,79; 2 colores claramente distintos, 1 tono, colorido 56); formas parcialmente visibles (probabilidad 0,66; bordes cromáticos en el 15 % del textil); textil completo (probabilidad 0,81; compacidad 0,63, lagunas 0,0 %); estructura no evidente. Puntaje 56.</t>
+          <t>Fotografía buena (nitidez 1,81; textil de 1352 px de lado); colores identificables (probabilidad 0,76; 2 colores claramente distintos, 1 tono, colorido 56); formas parcialmente visibles (probabilidad 0,58; bordes cromáticos en el 15 % del textil); textil completo (probabilidad 0,85; compacidad 0,63, lagunas 0,0 %); estructura no evidente. Puntaje 79.</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>68.8</v>
+        <v>90</v>
       </c>
       <c r="AB33" s="4" t="inlineStr">
         <is>
@@ -4135,7 +4135,7 @@
       </c>
       <c r="AD33" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,62; textil de 2287 px de lado); colores identificables (probabilidad 0,89; 1 color claramente distinto, 2 tonos, colorido 28); formas visibles (probabilidad 0,92; bordes cromáticos en el 22 % del textil); textil completo (probabilidad 0,83; compacidad 0,82, lagunas 4,9 %); estructura no evidente. Puntaje 69.</t>
+          <t>Fotografía buena (nitidez 2,62; textil de 2287 px de lado); colores identificables (probabilidad 0,89; 1 color claramente distinto, 2 tonos, colorido 28); formas visibles (probabilidad 0,93; bordes cromáticos en el 22 % del textil); textil completo (probabilidad 0,86; compacidad 0,82, lagunas 4,9 %); estructura no evidente. Puntaje 90 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4227,7 @@
         </is>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>72.40000000000001</v>
+        <v>83.5</v>
       </c>
       <c r="AB34" s="4" t="inlineStr">
         <is>
@@ -4241,7 +4241,7 @@
       </c>
       <c r="AD34" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,35; textil de 1651 px de lado); colores identificables (probabilidad 0,86; 1 color claramente distinto, 2 tonos, colorido 25); formas visibles (probabilidad 0,90; bordes cromáticos en el 26 % del textil); textil completo (probabilidad 0,76; compacidad 0,80, lagunas 11,0 %); estructura no evidente. Puntaje 72.</t>
+          <t>Fotografía buena (nitidez 2,35; textil de 1651 px de lado); colores identificables (probabilidad 0,85; 1 color claramente distinto, 2 tonos, colorido 25); formas visibles (probabilidad 0,90; bordes cromáticos en el 26 % del textil); textil completo (probabilidad 0,76; compacidad 0,80, lagunas 11,0 %); estructura no evidente. Puntaje 83.</t>
         </is>
       </c>
     </row>
@@ -4333,7 +4333,7 @@
         </is>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>63.2</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="AB35" s="4" t="inlineStr">
         <is>
@@ -4347,7 +4347,7 @@
       </c>
       <c r="AD35" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,87; textil de 1596 px de lado); colores identificables (probabilidad 0,78; 2 colores claramente distintos, 2 tonos, colorido 36); formas visibles (probabilidad 0,76; bordes cromáticos en el 24 % del textil); completitud incierta (probabilidad 0,62; compacidad 0,63, lagunas 6,2 %); estructura no evidente. Puntaje 63.</t>
+          <t>Fotografía buena (nitidez 1,87; textil de 1596 px de lado); colores identificables (probabilidad 0,80; 2 colores claramente distintos, 2 tonos, colorido 36); formas visibles (probabilidad 0,76; bordes cromáticos en el 24 % del textil); completitud incierta (probabilidad 0,70; compacidad 0,63, lagunas 6,2 %); estructura no evidente. Puntaje 77.</t>
         </is>
       </c>
     </row>
@@ -4439,7 +4439,7 @@
         </is>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>69.40000000000001</v>
+        <v>87.7</v>
       </c>
       <c r="AB36" s="4" t="inlineStr">
         <is>
@@ -4453,7 +4453,7 @@
       </c>
       <c r="AD36" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,48; textil de 2034 px de lado); colores identificables (probabilidad 0,85; 3 colores claramente distintos, 2 tonos, colorido 46); formas visibles (probabilidad 0,85; bordes cromáticos en el 22 % del textil); textil completo (probabilidad 0,71; compacidad 0,80, lagunas 7,7 %); estructura no evidente. Puntaje 69.</t>
+          <t>Fotografía buena (nitidez 1,48; textil de 2034 px de lado); colores identificables (probabilidad 0,90; 3 colores claramente distintos, 2 tonos, colorido 46); formas visibles (probabilidad 0,90; bordes cromáticos en el 22 % del textil); textil completo (probabilidad 0,85; compacidad 0,80, lagunas 7,7 %); estructura no evidente. Puntaje 88 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
         </is>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>66.59999999999999</v>
+        <v>86.8</v>
       </c>
       <c r="AB37" s="4" t="inlineStr">
         <is>
@@ -4559,7 +4559,7 @@
       </c>
       <c r="AD37" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,71; textil de 1980 px de lado); colores identificables (probabilidad 0,87; 2 colores claramente distintos, 1 tono, colorido 25); formas visibles (probabilidad 0,87; bordes cromáticos en el 26 % del textil); textil completo (probabilidad 0,81; compacidad 0,74, lagunas 1,8 %); estructura no evidente. Puntaje 67.</t>
+          <t>Fotografía buena (nitidez 2,71; textil de 1980 px de lado); colores identificables (probabilidad 0,82; 2 colores claramente distintos, 1 tono, colorido 25); formas visibles (probabilidad 0,86; bordes cromáticos en el 26 % del textil); textil completo (probabilidad 0,84; compacidad 0,74, lagunas 1,8 %); estructura no evidente. Puntaje 87 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
         </is>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>64.3</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="AB38" s="4" t="inlineStr">
         <is>
@@ -4665,7 +4665,7 @@
       </c>
       <c r="AD38" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,92; textil de 1928 px de lado); colores identificables (probabilidad 0,77; 2 colores claramente distintos, 2 tonos, colorido 34); formas visibles (probabilidad 0,81; bordes cromáticos en el 19 % del textil); completitud incierta (probabilidad 0,62; compacidad 0,76, lagunas 8,5 %); estructura no evidente. Puntaje 64.</t>
+          <t>Fotografía buena (nitidez 1,92; textil de 1928 px de lado); colores identificables (probabilidad 0,81; 2 colores claramente distintos, 2 tonos, colorido 34); formas visibles (probabilidad 0,84; bordes cromáticos en el 19 % del textil); textil completo (probabilidad 0,72; compacidad 0,76, lagunas 8,5 %); estructura no evidente. Puntaje 80.</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4757,7 @@
         </is>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>68.7</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="AB39" s="4" t="inlineStr">
         <is>
@@ -4771,7 +4771,7 @@
       </c>
       <c r="AD39" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,99; textil de 1810 px de lado); colores identificables (probabilidad 0,89; 2 colores claramente distintos, 2 tonos, colorido 39); formas visibles (probabilidad 0,86; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,82; compacidad 0,69, lagunas 1,1 %); estructura no evidente. Puntaje 69.</t>
+          <t>Fotografía buena (nitidez 1,99; textil de 1810 px de lado); colores identificables (probabilidad 0,89; 2 colores claramente distintos, 2 tonos, colorido 39); formas visibles (probabilidad 0,86; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,86; compacidad 0,69, lagunas 1,1 %); estructura no evidente. Puntaje 88 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -4863,7 +4863,7 @@
         </is>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>65.3</v>
+        <v>80.5</v>
       </c>
       <c r="AB40" s="4" t="inlineStr">
         <is>
@@ -4877,7 +4877,7 @@
       </c>
       <c r="AD40" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,28; textil de 1821 px de lado); colores identificables (probabilidad 0,72; 2 colores claramente distintos, 1 tono, colorido 27); formas visibles (probabilidad 0,84; bordes cromáticos en el 10 % del textil); completitud incierta (probabilidad 0,60; compacidad 0,81, lagunas 23,2 %); estructura no evidente. Puntaje 65.</t>
+          <t>Fotografía buena (nitidez 2,28; textil de 1821 px de lado); colores identificables (probabilidad 0,77; 2 colores claramente distintos, 1 tono, colorido 27); formas visibles (probabilidad 0,86; bordes cromáticos en el 10 % del textil); textil completo (probabilidad 0,76; compacidad 0,81, lagunas 23,2 %); estructura no evidente. Puntaje 80.</t>
         </is>
       </c>
     </row>
@@ -4969,7 +4969,7 @@
         </is>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>72.8</v>
+        <v>88.5</v>
       </c>
       <c r="AB41" s="4" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="AD41" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,62; textil de 2116 px de lado); colores identificables (probabilidad 0,92; 1 color claramente distinto, 2 tonos, colorido 20); formas visibles (probabilidad 0,93; bordes cromáticos en el 34 % del textil); textil completo (probabilidad 0,85; compacidad 0,74, lagunas 0,0 %); estructura no evidente. Puntaje 73.</t>
+          <t>Fotografía buena (nitidez 2,62; textil de 2116 px de lado); colores identificables (probabilidad 0,89; 1 color claramente distinto, 2 tonos, colorido 20); formas visibles (probabilidad 0,93; bordes cromáticos en el 34 % del textil); textil completo (probabilidad 0,82; compacidad 0,74, lagunas 0,0 %); estructura no evidente. Puntaje 89 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -5075,7 +5075,7 @@
         </is>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>68.59999999999999</v>
+        <v>81.7</v>
       </c>
       <c r="AB42" s="4" t="inlineStr">
         <is>
@@ -5089,7 +5089,7 @@
       </c>
       <c r="AD42" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,97; textil de 1846 px de lado); colores identificables (probabilidad 0,77; 2 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,84; bordes cromáticos en el 23 % del textil); completitud incierta (probabilidad 0,63; compacidad 0,84, lagunas 14,0 %); estructura no evidente. Puntaje 69.</t>
+          <t>Fotografía buena (nitidez 1,97; textil de 1846 px de lado); colores identificables (probabilidad 0,83; 2 colores claramente distintos, 2 tonos, colorido 41); formas visibles (probabilidad 0,87; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,74; compacidad 0,84, lagunas 14,0 %); estructura no evidente. Puntaje 82.</t>
         </is>
       </c>
     </row>
@@ -5181,7 +5181,7 @@
         </is>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>48.5</v>
+        <v>55.8</v>
       </c>
       <c r="AB43" s="4" t="inlineStr">
         <is>
@@ -5195,7 +5195,7 @@
       </c>
       <c r="AD43" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,78; textil de 2126 px de lado); colores parcialmente identificables (probabilidad 0,53; 1 color claramente distinto, 2 tonos, colorido 25); formas parcialmente visibles (probabilidad 0,69; bordes cromáticos en el 21 % del textil); textil incompleto (probabilidad 0,29; compacidad 0,54, lagunas 10,4 %, el título dice «fragment»); estructura no evidente. Puntaje 49.</t>
+          <t>Fotografía buena (nitidez 1,78; textil de 2126 px de lado); colores identificables (probabilidad 0,71; 1 color claramente distinto, 2 tonos, colorido 25); formas visibles (probabilidad 0,79; bordes cromáticos en el 21 % del textil); textil incompleto (probabilidad 0,31; compacidad 0,54, lagunas 10,4 %, el título dice «fragment»); estructura no evidente. Puntaje 56.</t>
         </is>
       </c>
     </row>
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>74.59999999999999</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="AB44" s="4" t="inlineStr">
         <is>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="AD44" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,70; textil de 1301 px de lado); colores identificables (probabilidad 0,87; 2 colores claramente distintos, 2 tonos, colorido 36); formas visibles (probabilidad 0,84; bordes cromáticos en el 45 % del textil); textil completo (probabilidad 0,72; compacidad 0,64, lagunas 7,4 %); estructura no evidente. Puntaje 75.</t>
+          <t>Fotografía buena (nitidez 1,70; textil de 1301 px de lado); colores identificables (probabilidad 0,87; 2 colores claramente distintos, 2 tonos, colorido 36); formas visibles (probabilidad 0,85; bordes cromáticos en el 45 % del textil); textil completo (probabilidad 0,73; compacidad 0,64, lagunas 7,4 %); estructura no evidente. Puntaje 80.</t>
         </is>
       </c>
     </row>
@@ -5393,7 +5393,7 @@
         </is>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>70.8</v>
+        <v>88.8</v>
       </c>
       <c r="AB45" s="4" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="AD45" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,83; textil de 3136 px de lado); colores identificables (probabilidad 0,94; 2 colores claramente distintos, 3 tonos, colorido 34); formas visibles (probabilidad 0,96; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,76; compacidad 0,88, lagunas 0,3 %, el título dice «fragment»); estructura no evidente. Puntaje 71.</t>
+          <t>Fotografía buena (nitidez 1,83; textil de 3136 px de lado); colores identificables (probabilidad 0,97; 2 colores claramente distintos, 3 tonos, colorido 34); formas visibles (probabilidad 0,98; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,80; compacidad 0,88, lagunas 0,3 %, el título dice «fragment»); estructura no evidente. Puntaje 89 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -5499,7 +5499,7 @@
         </is>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>68.8</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="AB46" s="4" t="inlineStr">
         <is>
@@ -5513,7 +5513,7 @@
       </c>
       <c r="AD46" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,98; textil de 2443 px de lado); colores identificables (probabilidad 0,96; 3 colores claramente distintos, 2 tonos, colorido 51); formas visibles (probabilidad 0,95; bordes cromáticos en el 25 % del textil); textil completo (probabilidad 0,85; compacidad 0,96, lagunas 0,0 %); estructura repetitiva. Puntaje 69.</t>
+          <t>Fotografía buena (nitidez 1,98; textil de 2443 px de lado); colores identificables (probabilidad 0,98; 3 colores claramente distintos, 2 tonos, colorido 51); formas visibles (probabilidad 0,98; bordes cromáticos en el 25 % del textil); textil completo (probabilidad 0,95; compacidad 0,96, lagunas 0,0 %); estructura repetitiva. Puntaje 96 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -5605,7 +5605,7 @@
         </is>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>75.5</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="AB47" s="4" t="inlineStr">
         <is>
@@ -5619,7 +5619,7 @@
       </c>
       <c r="AD47" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,56; textil de 2877 px de lado); colores identificables (probabilidad 0,97; 4 colores claramente distintos, 3 tonos, colorido 48); formas visibles (probabilidad 0,96; bordes cromáticos en el 44 % del textil); textil completo (probabilidad 0,85; compacidad 0,92, lagunas 0,0 %); estructura no evidente. Puntaje 75.</t>
+          <t>Fotografía buena (nitidez 1,56; textil de 2877 px de lado); colores identificables (probabilidad 0,99; 4 colores claramente distintos, 3 tonos, colorido 48); formas visibles (probabilidad 0,99; bordes cromáticos en el 44 % del textil); textil completo (probabilidad 0,95; compacidad 0,92, lagunas 0,0 %); estructura no evidente. Puntaje 96 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -5711,7 +5711,7 @@
         </is>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>63.1</v>
+        <v>71.3</v>
       </c>
       <c r="AB48" s="4" t="inlineStr">
         <is>
@@ -5725,7 +5725,7 @@
       </c>
       <c r="AD48" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,17; textil de 1495 px de lado); colores identificables (probabilidad 0,77; 2 colores claramente distintos, 3 tonos, colorido 32); formas visibles (probabilidad 0,72; bordes cromáticos en el 37 % del textil); completitud incierta (probabilidad 0,48; compacidad 0,50, lagunas 0,0 %); estructura repetitiva. Puntaje 63.</t>
+          <t>Fotografía regular (nitidez 1,17; textil de 1495 px de lado); colores identificables (probabilidad 0,81; 2 colores claramente distintos, 3 tonos, colorido 32); formas visibles (probabilidad 0,80; bordes cromáticos en el 37 % del textil); completitud incierta (probabilidad 0,58; compacidad 0,50, lagunas 0,0 %); estructura repetitiva. Puntaje 71.</t>
         </is>
       </c>
     </row>
@@ -5817,7 +5817,7 @@
         </is>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>68.7</v>
+        <v>85.2</v>
       </c>
       <c r="AB49" s="4" t="inlineStr">
         <is>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="AD49" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,76; textil de 3094 px de lado); colores identificables (probabilidad 0,93; 2 colores claramente distintos, 3 tonos, colorido 36); formas visibles (probabilidad 0,95; bordes cromáticos en el 47 % del textil); completitud incierta (probabilidad 0,67; compacidad 0,86, lagunas 0,1 %, el título dice «fragment»); estructura no evidente. Puntaje 69.</t>
+          <t>Fotografía buena (nitidez 1,76; textil de 3094 px de lado); colores identificables (probabilidad 0,97; 2 colores claramente distintos, 3 tonos, colorido 36); formas visibles (probabilidad 0,98; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,74; compacidad 0,86, lagunas 0,1 %, el título dice «fragment»); estructura no evidente. Puntaje 85 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -5923,7 +5923,7 @@
         </is>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>74.3</v>
+        <v>96.5</v>
       </c>
       <c r="AB50" s="4" t="inlineStr">
         <is>
@@ -5937,7 +5937,7 @@
       </c>
       <c r="AD50" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,87; textil de 3193 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 3 tonos, colorido 33); formas visibles (probabilidad 0,99; bordes cromáticos en el 36 % del textil); textil completo (probabilidad 0,93; compacidad 0,97, lagunas 0,0 %); estructura no evidente. Puntaje 74.</t>
+          <t>Fotografía buena (nitidez 1,87; textil de 3193 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 3 tonos, colorido 33); formas visibles (probabilidad 0,99; bordes cromáticos en el 36 % del textil); textil completo (probabilidad 0,96; compacidad 0,97, lagunas 0,0 %); estructura no evidente. Puntaje 97 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>75</v>
+        <v>97.2</v>
       </c>
       <c r="AB51" s="4" t="inlineStr">
         <is>
@@ -6043,7 +6043,7 @@
       </c>
       <c r="AD51" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,32; textil de 2721 px de lado); colores identificables (probabilidad 0,98; 3 colores claramente distintos, 3 tonos, colorido 43); formas visibles (probabilidad 0,98; bordes cromáticos en el 24 % del textil); textil completo (probabilidad 0,93; compacidad 0,95, lagunas 0,0 %); estructura repetitiva. Puntaje 75.</t>
+          <t>Fotografía regular (nitidez 1,32; textil de 2721 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 43); formas visibles (probabilidad 0,99; bordes cromáticos en el 24 % del textil); textil completo (probabilidad 0,97; compacidad 0,95, lagunas 0,0 %); estructura repetitiva. Puntaje 97 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6135,7 @@
         </is>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>71.8</v>
+        <v>86</v>
       </c>
       <c r="AB52" s="4" t="inlineStr">
         <is>
@@ -6149,7 +6149,7 @@
       </c>
       <c r="AD52" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,41; textil de 2116 px de lado); colores identificables (probabilidad 0,83; 2 colores claramente distintos, 3 tonos, colorido 30); formas visibles (probabilidad 0,90; bordes cromáticos en el 28 % del textil); completitud incierta (probabilidad 0,64; compacidad 0,83, lagunas 13,6 %); estructura no evidente. Puntaje 72.</t>
+          <t>Fotografía buena (nitidez 1,41; textil de 2116 px de lado); colores identificables (probabilidad 0,91; 2 colores claramente distintos, 3 tonos, colorido 30); formas visibles (probabilidad 0,95; bordes cromáticos en el 28 % del textil); textil completo (probabilidad 0,81; compacidad 0,83, lagunas 13,6 %); estructura no evidente. Puntaje 86 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6241,7 @@
         </is>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>74.2</v>
+        <v>97</v>
       </c>
       <c r="AB53" s="4" t="inlineStr">
         <is>
@@ -6255,7 +6255,7 @@
       </c>
       <c r="AD53" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,51; textil de 3149 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 42); formas visibles (probabilidad 0,98; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,92; compacidad 0,96, lagunas 0,0 %); estructura no evidente. Puntaje 74.</t>
+          <t>Fotografía buena (nitidez 1,51; textil de 3149 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 42); formas visibles (probabilidad 0,99; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,96; compacidad 0,96, lagunas 0,0 %); estructura no evidente. Puntaje 97 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6347,7 @@
         </is>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>73.59999999999999</v>
+        <v>96.2</v>
       </c>
       <c r="AB54" s="4" t="inlineStr">
         <is>
@@ -6361,7 +6361,7 @@
       </c>
       <c r="AD54" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,63; textil de 2925 px de lado); colores identificables (probabilidad 0,97; 1 color claramente distinto, 3 tonos, colorido 39); formas visibles (probabilidad 0,98; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,94; compacidad 0,93, lagunas 0,0 %); estructura repetitiva. Puntaje 74.</t>
+          <t>Fotografía buena (nitidez 1,63; textil de 2925 px de lado); colores identificables (probabilidad 0,98; 1 color claramente distinto, 3 tonos, colorido 39); formas visibles (probabilidad 0,99; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,95; compacidad 0,93, lagunas 0,0 %); estructura repetitiva. Puntaje 96 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -6453,7 +6453,7 @@
         </is>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46.9</v>
+        <v>59.6</v>
       </c>
       <c r="AB55" s="4" t="inlineStr">
         <is>
@@ -6467,7 +6467,7 @@
       </c>
       <c r="AD55" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 0,90; textil de 1874 px de lado); colores parcialmente identificables (probabilidad 0,57; 3 colores claramente distintos, 2 tonos, colorido 37); formas parcialmente visibles (probabilidad 0,59; bordes cromáticos en el 34 % del textil); textil incompleto (probabilidad 0,25; compacidad 0,66, lagunas 2,9 %, el título dice «fragment»); estructura no evidente. Puntaje 47.</t>
+          <t>Fotografía deficiente (nitidez 0,90; textil de 1874 px de lado); colores identificables (probabilidad 0,74; 3 colores claramente distintos, 2 tonos, colorido 37); formas visibles (probabilidad 0,80; bordes cromáticos en el 34 % del textil); textil incompleto (probabilidad 0,37; compacidad 0,66, lagunas 2,9 %, el título dice «fragment»); estructura no evidente. Puntaje 60.</t>
         </is>
       </c>
     </row>
@@ -6559,7 +6559,7 @@
         </is>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>80</v>
+        <v>89.2</v>
       </c>
       <c r="AB56" s="4" t="inlineStr">
         <is>
@@ -6573,7 +6573,7 @@
       </c>
       <c r="AD56" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,50; textil de 2790 px de lado); colores identificables (probabilidad 0,91; 2 colores claramente distintos, 3 tonos, colorido 39); formas visibles (probabilidad 0,96; bordes cromáticos en el 37 % del textil); completitud incierta (probabilidad 0,69; compacidad 0,92, lagunas 22,7 %); estructura no evidente. Puntaje 80 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 1,50; textil de 2790 px de lado); colores identificables (probabilidad 0,96; 2 colores claramente distintos, 3 tonos, colorido 39); formas visibles (probabilidad 0,98; bordes cromáticos en el 37 % del textil); textil completo (probabilidad 0,86; compacidad 0,92, lagunas 22,7 %); estructura no evidente. Puntaje 89 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -6665,7 +6665,7 @@
         </is>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>66.40000000000001</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="AB57" s="4" t="inlineStr">
         <is>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="AD57" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,91; textil de 2911 px de lado); colores identificables (probabilidad 0,91; 2 colores claramente distintos, 1 tono, colorido 18); formas visibles (probabilidad 0,94; bordes cromáticos en el 6 % del textil); textil completo (probabilidad 0,83; compacidad 0,90, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 66.</t>
+          <t>Fotografía buena (nitidez 1,91; textil de 2911 px de lado); colores identificables (probabilidad 0,93; 2 colores claramente distintos, 1 tono, colorido 18); formas visibles (probabilidad 0,95; bordes cromáticos en el 6 % del textil); textil completo (probabilidad 0,88; compacidad 0,90, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 91 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6771,7 @@
         </is>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>56.6</v>
+        <v>68.3</v>
       </c>
       <c r="AB58" s="4" t="inlineStr">
         <is>
@@ -6785,7 +6785,7 @@
       </c>
       <c r="AD58" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,87; textil de 2204 px de lado); colores identificables (probabilidad 0,74; 1 color claramente distinto, 3 tonos, colorido 25); formas visibles (probabilidad 0,82; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,48; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 57.</t>
+          <t>Fotografía buena (nitidez 1,87; textil de 2204 px de lado); colores identificables (probabilidad 0,82; 1 color claramente distinto, 3 tonos, colorido 25); formas visibles (probabilidad 0,88; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,44; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 68.</t>
         </is>
       </c>
     </row>
@@ -6877,7 +6877,7 @@
         </is>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>63.3</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="AB59" s="4" t="inlineStr">
         <is>
@@ -6891,7 +6891,7 @@
       </c>
       <c r="AD59" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,15; textil de 2409 px de lado); colores identificables (probabilidad 0,85; 1 color claramente distinto, 2 tonos, colorido 32); formas visibles (probabilidad 0,90; bordes cromáticos en el 19 % del textil); completitud incierta (probabilidad 0,67; compacidad 0,94, lagunas 0,3 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
+          <t>Fotografía regular (nitidez 1,15; textil de 2409 px de lado); colores identificables (probabilidad 0,90; 1 color claramente distinto, 2 tonos, colorido 32); formas visibles (probabilidad 0,94; bordes cromáticos en el 19 % del textil); completitud incierta (probabilidad 0,64; compacidad 0,94, lagunas 0,3 %, el título dice «fragment»); estructura no evidente. Puntaje 78.</t>
         </is>
       </c>
     </row>
@@ -6983,7 +6983,7 @@
         </is>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>77.5</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="AB60" s="4" t="inlineStr">
         <is>
@@ -6997,7 +6997,7 @@
       </c>
       <c r="AD60" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 1,00; textil de 1225 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 2 tonos, colorido 37); formas visibles (probabilidad 0,97; bordes cromáticos en el 31 % del textil); textil completo (probabilidad 0,86; compacidad 0,93, lagunas 0,0 %, el título dice «fragment»); estructura simétrica. Puntaje 77 (imagen de referencia sugerida).</t>
+          <t>Fotografía deficiente (nitidez 1,00; textil de 1225 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 2 tonos, colorido 37); formas visibles (probabilidad 0,94; bordes cromáticos en el 31 % del textil); textil completo (probabilidad 0,78; compacidad 0,93, lagunas 0,0 %, el título dice «fragment»); estructura simétrica. Puntaje 85 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -7089,7 +7089,7 @@
         </is>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>74.7</v>
+        <v>95.3</v>
       </c>
       <c r="AB61" s="4" t="inlineStr">
         <is>
@@ -7103,7 +7103,7 @@
       </c>
       <c r="AD61" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,51; textil de 2454 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 59); formas visibles (probabilidad 0,99; bordes cromáticos en el 60 % del textil); textil completo (probabilidad 0,91; compacidad 0,96, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 75.</t>
+          <t>Fotografía buena (nitidez 2,51; textil de 2454 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 59); formas visibles (probabilidad 0,99; bordes cromáticos en el 60 % del textil); textil completo (probabilidad 0,93; compacidad 0,96, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 95 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -7195,7 +7195,7 @@
         </is>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>68.2</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="AB62" s="4" t="inlineStr">
         <is>
@@ -7209,7 +7209,7 @@
       </c>
       <c r="AD62" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,35; textil de 2897 px de lado); colores identificables (probabilidad 0,93; 3 colores claramente distintos, 3 tonos, colorido 46); formas visibles (probabilidad 0,93; bordes cromáticos en el 21 % del textil); completitud incierta (probabilidad 0,63; compacidad 0,90, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 68.</t>
+          <t>Fotografía regular (nitidez 1,35; textil de 2897 px de lado); colores identificables (probabilidad 0,96; 3 colores claramente distintos, 3 tonos, colorido 46); formas visibles (probabilidad 0,96; bordes cromáticos en el 21 % del textil); textil completo (probabilidad 0,72; compacidad 0,90, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 84.</t>
         </is>
       </c>
     </row>
@@ -7301,7 +7301,7 @@
         </is>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>80.5</v>
+        <v>96.5</v>
       </c>
       <c r="AB63" s="4" t="inlineStr">
         <is>
@@ -7315,7 +7315,7 @@
       </c>
       <c r="AD63" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,63; textil de 2088 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 45); formas visibles (probabilidad 1,00; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,97; compacidad 0,97, lagunas 0,0 %, el título dice «fragment»); estructura simétrica. Puntaje 81 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 1,63; textil de 2088 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 45); formas visibles (probabilidad 1,00; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,96; compacidad 0,97, lagunas 0,0 %, el título dice «fragment»); estructura simétrica. Puntaje 97 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -7407,7 +7407,7 @@
         </is>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>67.09999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="AB64" s="4" t="inlineStr">
         <is>
@@ -7421,7 +7421,7 @@
       </c>
       <c r="AD64" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 0,87; textil de 2456 px de lado); colores identificables (probabilidad 0,92; 3 colores claramente distintos, 2 tonos, colorido 52); formas visibles (probabilidad 0,83; bordes cromáticos en el 35 % del textil); completitud incierta (probabilidad 0,62; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 67.</t>
+          <t>Fotografía deficiente (nitidez 0,87; textil de 2456 px de lado); colores identificables (probabilidad 0,95; 3 colores claramente distintos, 2 tonos, colorido 52); formas visibles (probabilidad 0,87; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,77; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 82.</t>
         </is>
       </c>
     </row>
@@ -7513,7 +7513,7 @@
         </is>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>78</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="AB65" s="4" t="inlineStr">
         <is>
@@ -7527,7 +7527,7 @@
       </c>
       <c r="AD65" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,96; textil de 814 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 3 tonos, colorido 38); formas visibles (probabilidad 0,96; bordes cromáticos en el 40 % del textil); textil completo (probabilidad 0,72; compacidad 0,82, lagunas 0,4 %); estructura no evidente. Puntaje 78 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 1,96; textil de 814 px de lado); colores identificables (probabilidad 0,96; 2 colores claramente distintos, 3 tonos, colorido 38); formas visibles (probabilidad 0,95; bordes cromáticos en el 40 % del textil); textil completo (probabilidad 0,71; compacidad 0,82, lagunas 0,4 %); estructura no evidente. Puntaje 82.</t>
         </is>
       </c>
     </row>
@@ -7619,7 +7619,7 @@
         </is>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>80.2</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="AB66" s="4" t="inlineStr">
         <is>
@@ -7633,7 +7633,7 @@
       </c>
       <c r="AD66" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,15; textil de 704 px de lado); colores identificables (probabilidad 0,97; 3 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,95; bordes cromáticos en el 40 % del textil); textil completo (probabilidad 0,80; compacidad 0,83, lagunas 0,0 %); estructura no evidente. Puntaje 80 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 2,15; textil de 704 px de lado); colores identificables (probabilidad 0,95; 3 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,92; bordes cromáticos en el 40 % del textil); textil completo (probabilidad 0,85; compacidad 0,83, lagunas 0,0 %); estructura no evidente. Puntaje 89 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -7725,7 +7725,7 @@
         </is>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>73.09999999999999</v>
+        <v>86</v>
       </c>
       <c r="AB67" s="4" t="inlineStr">
         <is>
@@ -7739,7 +7739,7 @@
       </c>
       <c r="AD67" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,89; textil de 1207 px de lado); colores identificables (probabilidad 0,93; 2 colores claramente distintos, 2 tonos, colorido 37); formas visibles (probabilidad 0,90; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,76; compacidad 0,62, lagunas 0,0 %); estructura no evidente. Puntaje 73.</t>
+          <t>Fotografía buena (nitidez 1,89; textil de 1207 px de lado); colores identificables (probabilidad 0,92; 2 colores claramente distintos, 2 tonos, colorido 37); formas visibles (probabilidad 0,90; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,81; compacidad 0,62, lagunas 0,0 %); estructura no evidente. Puntaje 86 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -7831,7 +7831,7 @@
         </is>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>78.40000000000001</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="AB68" s="4" t="inlineStr">
         <is>
@@ -7845,7 +7845,7 @@
       </c>
       <c r="AD68" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,13; textil de 1077 px de lado); colores identificables (probabilidad 0,97; 3 colores claramente distintos, 3 tonos, colorido 49); formas visibles (probabilidad 0,95; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,73; compacidad 0,64, lagunas 3,1 %); estructura repetitiva. Puntaje 78 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 2,13; textil de 1077 px de lado); colores identificables (probabilidad 0,97; 3 colores claramente distintos, 3 tonos, colorido 49); formas visibles (probabilidad 0,94; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,80; compacidad 0,64, lagunas 3,1 %); estructura repetitiva. Puntaje 87 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -7937,7 +7937,7 @@
         </is>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>67.09999999999999</v>
+        <v>73.5</v>
       </c>
       <c r="AB69" s="4" t="inlineStr">
         <is>
@@ -7951,7 +7951,7 @@
       </c>
       <c r="AD69" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,02; textil de 1558 px de lado); colores identificables (probabilidad 0,93; 2 colores claramente distintos, 3 tonos, colorido 24); formas visibles (probabilidad 0,92; bordes cromáticos en el 24 % del textil); completitud incierta (probabilidad 0,56; compacidad 0,90, lagunas 0,1 %, el título dice «fragment»); estructura no evidente. Puntaje 67.</t>
+          <t>Fotografía regular (nitidez 1,02; textil de 1558 px de lado); colores identificables (probabilidad 0,96; 2 colores claramente distintos, 3 tonos, colorido 24); formas visibles (probabilidad 0,95; bordes cromáticos en el 24 % del textil); completitud incierta (probabilidad 0,56; compacidad 0,90, lagunas 0,1 %, el título dice «fragment»); estructura no evidente. Puntaje 74.</t>
         </is>
       </c>
     </row>
@@ -8043,7 +8043,7 @@
         </is>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>66</v>
+        <v>72.2</v>
       </c>
       <c r="AB70" s="4" t="inlineStr">
         <is>
@@ -8057,7 +8057,7 @@
       </c>
       <c r="AD70" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,00; textil de 1666 px de lado); colores identificables (probabilidad 0,90; 2 colores claramente distintos, 3 tonos, colorido 23); formas visibles (probabilidad 0,91; bordes cromáticos en el 19 % del textil); completitud incierta (probabilidad 0,54; compacidad 0,90, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 66.</t>
+          <t>Fotografía regular (nitidez 1,00; textil de 1666 px de lado); colores identificables (probabilidad 0,95; 2 colores claramente distintos, 3 tonos, colorido 23); formas visibles (probabilidad 0,95; bordes cromáticos en el 19 % del textil); completitud incierta (probabilidad 0,55; compacidad 0,90, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 72.</t>
         </is>
       </c>
     </row>
@@ -8149,7 +8149,7 @@
         </is>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>69.59999999999999</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="AB71" s="4" t="inlineStr">
         <is>
@@ -8163,7 +8163,7 @@
       </c>
       <c r="AD71" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,61; textil de 2077 px de lado); colores identificables (probabilidad 0,94; 2 colores claramente distintos, 3 tonos, colorido 30); formas visibles (probabilidad 0,95; bordes cromáticos en el 29 % del textil); completitud incierta (probabilidad 0,61; compacidad 0,91, lagunas 2,4 %, el título dice «fragment»); estructura no evidente. Puntaje 70.</t>
+          <t>Fotografía buena (nitidez 1,61; textil de 2077 px de lado); colores identificables (probabilidad 0,97; 2 colores claramente distintos, 3 tonos, colorido 30); formas visibles (probabilidad 0,97; bordes cromáticos en el 29 % del textil); completitud incierta (probabilidad 0,65; compacidad 0,91, lagunas 2,4 %, el título dice «fragment»); estructura no evidente. Puntaje 80.</t>
         </is>
       </c>
     </row>
@@ -8255,7 +8255,7 @@
         </is>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>74.2</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="AB72" s="4" t="inlineStr">
         <is>
@@ -8269,7 +8269,7 @@
       </c>
       <c r="AD72" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,36; textil de 2716 px de lado); colores identificables (probabilidad 0,97; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,97; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,95; compacidad 0,95, lagunas 0,0 %); estructura simétrica. Puntaje 74.</t>
+          <t>Fotografía regular (nitidez 1,36; textil de 2716 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,98; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,97; compacidad 0,95, lagunas 0,0 %); estructura simétrica. Puntaje 97 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -8361,7 +8361,7 @@
         </is>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>69.3</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="AB73" s="4" t="inlineStr">
         <is>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="AD73" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 3,19; textil de 2988 px de lado); colores identificables (probabilidad 0,94; 1 color claramente distinto, 1 tono, colorido 35); formas visibles (probabilidad 0,96; bordes cromáticos en el 18 % del textil); textil completo (probabilidad 0,95; compacidad 0,95, lagunas 0,0 %); estructura no evidente. Puntaje 69.</t>
+          <t>Fotografía buena (nitidez 3,19; textil de 2988 px de lado); colores identificables (probabilidad 0,92; 1 color claramente distinto, 1 tono, colorido 35); formas visibles (probabilidad 0,95; bordes cromáticos en el 18 % del textil); textil completo (probabilidad 0,95; compacidad 0,95, lagunas 0,0 %); estructura no evidente. Puntaje 96 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -8467,7 +8467,7 @@
         </is>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>70.3</v>
+        <v>90.7</v>
       </c>
       <c r="AB74" s="4" t="inlineStr">
         <is>
@@ -8481,7 +8481,7 @@
       </c>
       <c r="AD74" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,17; textil de 2477 px de lado); colores identificables (probabilidad 0,93; 2 colores claramente distintos, 2 tonos, colorido 22); formas visibles (probabilidad 0,94; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,79; compacidad 0,92, lagunas 3,8 %); estructura no evidente. Puntaje 70.</t>
+          <t>Fotografía regular (nitidez 1,17; textil de 2477 px de lado); colores identificables (probabilidad 0,95; 2 colores claramente distintos, 2 tonos, colorido 22); formas visibles (probabilidad 0,96; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,88; compacidad 0,92, lagunas 3,8 %); estructura no evidente. Puntaje 91 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -8573,7 +8573,7 @@
         </is>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>60.9</v>
+        <v>70.5</v>
       </c>
       <c r="AB75" s="4" t="inlineStr">
         <is>
@@ -8587,7 +8587,7 @@
       </c>
       <c r="AD75" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,92; textil de 2430 px de lado); colores identificables (probabilidad 0,72; 2 colores claramente distintos, 2 tonos, colorido 31); formas visibles (probabilidad 0,85; bordes cromáticos en el 25 % del textil); textil incompleto (probabilidad 0,38; compacidad 0,86, lagunas 15,1 %, el título dice «fragment»); estructura no evidente. Puntaje 61.</t>
+          <t>Fotografía buena (nitidez 1,92; textil de 2430 px de lado); colores identificables (probabilidad 0,82; 2 colores claramente distintos, 2 tonos, colorido 31); formas visibles (probabilidad 0,92; bordes cromáticos en el 25 % del textil); completitud incierta (probabilidad 0,50; compacidad 0,86, lagunas 15,1 %, el título dice «fragment»); estructura no evidente. Puntaje 70.</t>
         </is>
       </c>
     </row>
@@ -8679,7 +8679,7 @@
         </is>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>70.7</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="AB76" s="4" t="inlineStr">
         <is>
@@ -8693,7 +8693,7 @@
       </c>
       <c r="AD76" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,39; textil de 2469 px de lado); colores identificables (probabilidad 0,96; 1 color claramente distinto, 2 tonos, colorido 18); formas visibles (probabilidad 0,97; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,91; compacidad 0,90, lagunas 0,0 %); estructura repetitiva. Puntaje 71.</t>
+          <t>Fotografía buena (nitidez 1,39; textil de 2469 px de lado); colores identificables (probabilidad 0,97; 1 color claramente distinto, 2 tonos, colorido 18); formas visibles (probabilidad 0,98; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,93; compacidad 0,90, lagunas 0,0 %); estructura repetitiva. Puntaje 94 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -8785,7 +8785,7 @@
         </is>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>67.59999999999999</v>
+        <v>89.8</v>
       </c>
       <c r="AB77" s="4" t="inlineStr">
         <is>
@@ -8799,7 +8799,7 @@
       </c>
       <c r="AD77" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 0,98; textil de 2858 px de lado); colores identificables (probabilidad 0,92; 1 color claramente distinto, 1 tono, colorido 15); formas visibles (probabilidad 0,94; bordes cromáticos en el 10 % del textil); textil completo (probabilidad 0,84; compacidad 0,91, lagunas 0,9 %); estructura repetitiva y simétrica. Puntaje 68.</t>
+          <t>Fotografía regular (nitidez 0,98; textil de 2858 px de lado); colores identificables (probabilidad 0,94; 1 color claramente distinto, 1 tono, colorido 15); formas visibles (probabilidad 0,95; bordes cromáticos en el 10 % del textil); textil completo (probabilidad 0,88; compacidad 0,91, lagunas 0,9 %); estructura repetitiva y simétrica. Puntaje 90 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -8891,7 +8891,7 @@
         </is>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>79.40000000000001</v>
+        <v>96.7</v>
       </c>
       <c r="AB78" s="4" t="inlineStr">
         <is>
@@ -8905,7 +8905,7 @@
       </c>
       <c r="AD78" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,05; textil de 2968 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 4 tonos, colorido 44); formas visibles (probabilidad 1,00; bordes cromáticos en el 56 % del textil); textil completo (probabilidad 0,96; compacidad 0,98, lagunas 1,0 %, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 79 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 2,05; textil de 2968 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 4 tonos, colorido 44); formas visibles (probabilidad 1,00; bordes cromáticos en el 56 % del textil); textil completo (probabilidad 0,96; compacidad 0,98, lagunas 1,0 %, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 97 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -8997,7 +8997,7 @@
         </is>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>78.8</v>
+        <v>98</v>
       </c>
       <c r="AB79" s="4" t="inlineStr">
         <is>
@@ -9011,7 +9011,7 @@
       </c>
       <c r="AD79" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,88; textil de 2489 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 45); formas visibles (probabilidad 0,99; bordes cromáticos en el 56 % del textil); textil completo (probabilidad 0,96; compacidad 0,95, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 79 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 1,88; textil de 2489 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 45); formas visibles (probabilidad 1,00; bordes cromáticos en el 56 % del textil); textil completo (probabilidad 0,98; compacidad 0,95, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 98 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -9103,7 +9103,7 @@
         </is>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>79.5</v>
+        <v>98.2</v>
       </c>
       <c r="AB80" s="4" t="inlineStr">
         <is>
@@ -9117,7 +9117,7 @@
       </c>
       <c r="AD80" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,87; textil de 2535 px de lado); colores identificables (probabilidad 1,00; 5 colores claramente distintos, 4 tonos, colorido 45); formas visibles (probabilidad 1,00; bordes cromáticos en el 54 % del textil); textil completo (probabilidad 0,94; compacidad 0,98, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 80 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 1,87; textil de 2535 px de lado); colores identificables (probabilidad 1,00; 5 colores claramente distintos, 4 tonos, colorido 45); formas visibles (probabilidad 1,00; bordes cromáticos en el 54 % del textil); textil completo (probabilidad 0,98; compacidad 0,98, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 98 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -9209,7 +9209,7 @@
         </is>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>79.40000000000001</v>
+        <v>98.8</v>
       </c>
       <c r="AB81" s="4" t="inlineStr">
         <is>
@@ -9223,7 +9223,7 @@
       </c>
       <c r="AD81" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,45; textil de 3178 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 57); formas visibles (probabilidad 1,00; bordes cromáticos en el 40 % del textil); textil completo (probabilidad 0,98; compacidad 0,93, lagunas 0,1 %); estructura repetitiva y simétrica. Puntaje 79 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 1,45; textil de 3178 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 57); formas visibles (probabilidad 1,00; bordes cromáticos en el 40 % del textil); textil completo (probabilidad 0,99; compacidad 0,93, lagunas 0,1 %); estructura repetitiva y simétrica. Puntaje 99 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -9315,7 +9315,7 @@
         </is>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>65.7</v>
+        <v>85.7</v>
       </c>
       <c r="AB82" s="4" t="inlineStr">
         <is>
@@ -9329,7 +9329,7 @@
       </c>
       <c r="AD82" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,18; textil de 2399 px de lado); colores identificables (probabilidad 0,88; 1 color claramente distinto, 2 tonos, colorido 29); formas visibles (probabilidad 0,92; bordes cromáticos en el 11 % del textil); textil completo (probabilidad 0,80; compacidad 0,85, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 66.</t>
+          <t>Fotografía buena (nitidez 2,18; textil de 2399 px de lado); colores identificables (probabilidad 0,90; 1 color claramente distinto, 2 tonos, colorido 29); formas visibles (probabilidad 0,93; bordes cromáticos en el 11 % del textil); textil completo (probabilidad 0,76; compacidad 0,85, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 86 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -9421,7 +9421,7 @@
         </is>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>65.7</v>
+        <v>85.7</v>
       </c>
       <c r="AB83" s="4" t="inlineStr">
         <is>
@@ -9435,7 +9435,7 @@
       </c>
       <c r="AD83" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,18; textil de 2399 px de lado); colores identificables (probabilidad 0,88; 1 color claramente distinto, 2 tonos, colorido 29); formas visibles (probabilidad 0,92; bordes cromáticos en el 11 % del textil); textil completo (probabilidad 0,80; compacidad 0,85, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 66.</t>
+          <t>Fotografía buena (nitidez 2,18; textil de 2399 px de lado); colores identificables (probabilidad 0,90; 1 color claramente distinto, 2 tonos, colorido 29); formas visibles (probabilidad 0,93; bordes cromáticos en el 11 % del textil); textil completo (probabilidad 0,76; compacidad 0,85, lagunas 1,0 %, el título dice «fragment»); estructura no evidente. Puntaje 86 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -9527,7 +9527,7 @@
         </is>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>62.9</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="AB84" s="4" t="inlineStr">
         <is>
@@ -9541,7 +9541,7 @@
       </c>
       <c r="AD84" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,29; textil de 2283 px de lado); colores identificables (probabilidad 0,84; 1 color claramente distinto, 2 tonos, colorido 28); formas visibles (probabilidad 0,90; bordes cromáticos en el 12 % del textil); completitud incierta (probabilidad 0,69; compacidad 0,80, lagunas 1,3 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
+          <t>Fotografía buena (nitidez 2,29; textil de 2283 px de lado); colores identificables (probabilidad 0,87; 1 color claramente distinto, 2 tonos, colorido 28); formas visibles (probabilidad 0,90; bordes cromáticos en el 12 % del textil); completitud incierta (probabilidad 0,63; compacidad 0,80, lagunas 1,3 %, el título dice «fragment»); estructura no evidente. Puntaje 79.</t>
         </is>
       </c>
     </row>
@@ -9633,7 +9633,7 @@
         </is>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>62.6</v>
+        <v>82.5</v>
       </c>
       <c r="AB85" s="4" t="inlineStr">
         <is>
@@ -9647,7 +9647,7 @@
       </c>
       <c r="AD85" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,23; textil de 2605 px de lado); colores identificables (probabilidad 0,82; 1 color claramente distinto, 2 tonos, colorido 30); formas visibles (probabilidad 0,89; bordes cromáticos en el 14 % del textil); textil completo (probabilidad 0,74; compacidad 0,82, lagunas 0,7 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
+          <t>Fotografía buena (nitidez 2,23; textil de 2605 px de lado); colores identificables (probabilidad 0,86; 1 color claramente distinto, 2 tonos, colorido 30); formas visibles (probabilidad 0,91; bordes cromáticos en el 14 % del textil); textil completo (probabilidad 0,70; compacidad 0,82, lagunas 0,7 %, el título dice «fragment»); estructura no evidente. Puntaje 82.</t>
         </is>
       </c>
     </row>
@@ -9739,7 +9739,7 @@
         </is>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>64</v>
+        <v>90.2</v>
       </c>
       <c r="AB86" s="4" t="inlineStr">
         <is>
@@ -9753,7 +9753,7 @@
       </c>
       <c r="AD86" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,12; textil de 2809 px de lado); colores identificables (probabilidad 0,86; 1 color claramente distinto, 2 tonos, colorido 18); formas visibles (probabilidad 0,89; bordes cromáticos en el 3 % del textil); textil completo (probabilidad 0,83; compacidad 0,85, lagunas 0,0 %); estructura no evidente. Puntaje 64.</t>
+          <t>Fotografía regular (nitidez 1,12; textil de 2809 px de lado); colores identificables (probabilidad 0,87; 1 color claramente distinto, 2 tonos, colorido 18); formas visibles (probabilidad 0,92; bordes cromáticos en el 3 % del textil); textil completo (probabilidad 0,89; compacidad 0,85, lagunas 0,0 %); estructura no evidente. Puntaje 90 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -9845,7 +9845,7 @@
         </is>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>65.59999999999999</v>
+        <v>84.2</v>
       </c>
       <c r="AB87" s="4" t="inlineStr">
         <is>
@@ -9859,7 +9859,7 @@
       </c>
       <c r="AD87" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,04; textil de 1679 px de lado); colores identificables (probabilidad 0,82; 1 color claramente distinto, 1 tono, colorido 22); formas visibles (probabilidad 0,82; bordes cromáticos en el 16 % del textil); textil completo (probabilidad 0,85; compacidad 0,70, lagunas 0,0 %); estructura repetitiva. Puntaje 66.</t>
+          <t>Fotografía regular (nitidez 1,04; textil de 1679 px de lado); colores identificables (probabilidad 0,80; 1 color claramente distinto, 1 tono, colorido 22); formas visibles (probabilidad 0,82; bordes cromáticos en el 16 % del textil); textil completo (probabilidad 0,85; compacidad 0,70, lagunas 0,0 %); estructura repetitiva. Puntaje 84.</t>
         </is>
       </c>
     </row>
@@ -9951,7 +9951,7 @@
         </is>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>69.40000000000001</v>
+        <v>91.2</v>
       </c>
       <c r="AB88" s="4" t="inlineStr">
         <is>
@@ -9965,7 +9965,7 @@
       </c>
       <c r="AD88" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,24; textil de 2757 px de lado); colores identificables (probabilidad 0,92; 4 colores claramente distintos, 2 tonos, colorido 48); formas visibles (probabilidad 0,86; bordes cromáticos en el 30 % del textil); textil completo (probabilidad 0,72; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 69.</t>
+          <t>Fotografía regular (nitidez 1,24; textil de 2757 px de lado); colores identificables (probabilidad 0,96; 4 colores claramente distintos, 2 tonos, colorido 48); formas visibles (probabilidad 0,94; bordes cromáticos en el 30 % del textil); textil completo (probabilidad 0,89; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 91 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -10057,7 +10057,7 @@
         </is>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>80.3</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="AB89" s="4" t="inlineStr">
         <is>
@@ -10071,7 +10071,7 @@
       </c>
       <c r="AD89" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,56; textil de 1657 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 3 tonos, colorido 45); formas visibles (probabilidad 0,98; bordes cromáticos en el 36 % del textil); textil completo (probabilidad 0,95; compacidad 0,85, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 80 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 1,56; textil de 1657 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 3 tonos, colorido 45); formas visibles (probabilidad 0,98; bordes cromáticos en el 36 % del textil); textil completo (probabilidad 0,95; compacidad 0,85, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 96 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -10179,21 +10179,21 @@
         </is>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>70.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="AB90" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC90" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD90" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,60; textil de 2088 px de lado); colores identificables (probabilidad 0,96; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,97; bordes cromáticos en el 27 % del textil); completitud incierta (probabilidad 0,59; compacidad 0,83, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 71.</t>
+          <t>Fotografía buena (nitidez 1,60; textil de 2088 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,97; bordes cromáticos en el 27 % del textil); completitud incierta (probabilidad 0,42; compacidad 0,83, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 65.</t>
         </is>
       </c>
     </row>
@@ -10301,21 +10301,21 @@
         </is>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>63.5</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="AB91" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC91" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD91" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,65; textil de 1378 px de lado); colores identificables (probabilidad 0,85; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,84; bordes cromáticos en el 27 % del textil); completitud incierta (probabilidad 0,57; compacidad 0,82, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
+          <t>Fotografía buena (nitidez 1,65; textil de 1378 px de lado); colores identificables (probabilidad 0,88; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,86; bordes cromáticos en el 27 % del textil); completitud incierta (probabilidad 0,47; compacidad 0,82, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 69.</t>
         </is>
       </c>
     </row>
@@ -10423,7 +10423,7 @@
         </is>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>63.6</v>
+        <v>71.5</v>
       </c>
       <c r="AB92" s="4" t="inlineStr">
         <is>
@@ -10437,7 +10437,7 @@
       </c>
       <c r="AD92" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,56; textil de 1445 px de lado); colores identificables (probabilidad 0,84; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,84; bordes cromáticos en el 24 % del textil); completitud incierta (probabilidad 0,60; compacidad 0,87, lagunas 0,2 %, el título dice «fragment»); estructura no evidente. Puntaje 64.</t>
+          <t>Fotografía buena (nitidez 1,56; textil de 1445 px de lado); colores identificables (probabilidad 0,87; 2 colores claramente distintos, 2 tonos, colorido 35); formas visibles (probabilidad 0,87; bordes cromáticos en el 24 % del textil); completitud incierta (probabilidad 0,52; compacidad 0,87, lagunas 0,2 %, el título dice «fragment»); estructura no evidente. Puntaje 72.</t>
         </is>
       </c>
     </row>
@@ -10545,7 +10545,7 @@
         </is>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>71.7</v>
+        <v>78.5</v>
       </c>
       <c r="AB93" s="4" t="inlineStr">
         <is>
@@ -10559,7 +10559,7 @@
       </c>
       <c r="AD93" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,76; textil de 1528 px de lado); colores identificables (probabilidad 0,93; 3 colores claramente distintos, 3 tonos, colorido 36); formas visibles (probabilidad 0,92; bordes cromáticos en el 30 % del textil); completitud incierta (probabilidad 0,64; compacidad 0,81, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 72.</t>
+          <t>Fotografía buena (nitidez 1,76; textil de 1528 px de lado); colores identificables (probabilidad 0,95; 3 colores claramente distintos, 3 tonos, colorido 36); formas visibles (probabilidad 0,94; bordes cromáticos en el 30 % del textil); completitud incierta (probabilidad 0,61; compacidad 0,81, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 78.</t>
         </is>
       </c>
     </row>
@@ -10667,7 +10667,7 @@
         </is>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>68.3</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="AB94" s="4" t="inlineStr">
         <is>
@@ -10681,7 +10681,7 @@
       </c>
       <c r="AD94" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 3,33; textil de 1348 px de lado); colores identificables (probabilidad 0,79; 2 colores claramente distintos, 1 tono, colorido 20); formas visibles (probabilidad 0,75; bordes cromáticos en el 38 % del textil); textil completo (probabilidad 0,70; compacidad 0,38, lagunas 5,4 %); estructura no evidente. Puntaje 68.</t>
+          <t>Fotografía buena (nitidez 3,33; textil de 1348 px de lado); colores parcialmente identificables (probabilidad 0,69; 2 colores claramente distintos, 1 tono, colorido 20); formas parcialmente visibles (probabilidad 0,64; bordes cromáticos en el 38 % del textil); textil completo (probabilidad 0,75; compacidad 0,38, lagunas 5,4 %); estructura no evidente. Puntaje 76.</t>
         </is>
       </c>
     </row>
@@ -10789,7 +10789,7 @@
         </is>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>69.2</v>
+        <v>93.3</v>
       </c>
       <c r="AB95" s="4" t="inlineStr">
         <is>
@@ -10803,7 +10803,7 @@
       </c>
       <c r="AD95" s="4" t="inlineStr">
         <is>
-          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía buena (nitidez 1,85; textil de 1849 px de lado); colores identificables (probabilidad 0,94; 1 color claramente distinto, 2 tonos, colorido 36); formas visibles (probabilidad 0,94; bordes cromáticos en el 9 % del textil); textil completo (probabilidad 0,93; compacidad 0,91, lagunas 0,4 %); estructura no evidente. Puntaje 69.</t>
+          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía buena (nitidez 1,85; textil de 1849 px de lado); colores identificables (probabilidad 0,93; 1 color claramente distinto, 2 tonos, colorido 36); formas visibles (probabilidad 0,93; bordes cromáticos en el 9 % del textil); textil completo (probabilidad 0,93; compacidad 0,91, lagunas 0,4 %); estructura no evidente. Puntaje 93.</t>
         </is>
       </c>
     </row>
@@ -10911,7 +10911,7 @@
         </is>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>71.2</v>
+        <v>82</v>
       </c>
       <c r="AB96" s="4" t="inlineStr">
         <is>
@@ -10925,7 +10925,7 @@
       </c>
       <c r="AD96" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,24; textil de 1536 px de lado); colores identificables (probabilidad 0,85; 2 colores claramente distintos, 1 tono, colorido 16); formas visibles (probabilidad 0,80; bordes cromáticos en el 49 % del textil); textil completo (probabilidad 0,77; compacidad 0,52, lagunas 0,0 %); estructura no evidente. Puntaje 71.</t>
+          <t>Fotografía buena (nitidez 2,24; textil de 1536 px de lado); colores identificables (probabilidad 0,81; 2 colores claramente distintos, 1 tono, colorido 16); formas visibles (probabilidad 0,78; bordes cromáticos en el 49 % del textil); textil completo (probabilidad 0,79; compacidad 0,52, lagunas 0,0 %); estructura no evidente. Puntaje 82.</t>
         </is>
       </c>
     </row>
@@ -11033,7 +11033,7 @@
         </is>
       </c>
       <c r="AA97" s="4" t="n">
-        <v>70.59999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="AB97" s="4" t="inlineStr">
         <is>
@@ -11047,7 +11047,7 @@
       </c>
       <c r="AD97" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,02; textil de 2238 px de lado); colores identificables (probabilidad 0,94; 5 colores claramente distintos, 4 tonos, colorido 61); formas visibles (probabilidad 0,84; bordes cromáticos en el 38 % del textil); completitud incierta (probabilidad 0,45; compacidad 0,69, lagunas 0,1 %); estructura no evidente. Puntaje 71.</t>
+          <t>Fotografía regular (nitidez 1,02; textil de 2238 px de lado); colores identificables (probabilidad 0,97; 5 colores claramente distintos, 4 tonos, colorido 61); formas visibles (probabilidad 0,94; bordes cromáticos en el 38 % del textil); textil completo (probabilidad 0,80; compacidad 0,69, lagunas 0,1 %); estructura no evidente. Puntaje 86 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -11155,7 +11155,7 @@
         </is>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>66.2</v>
+        <v>90.5</v>
       </c>
       <c r="AB98" s="4" t="inlineStr">
         <is>
@@ -11169,7 +11169,7 @@
       </c>
       <c r="AD98" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 0,69; textil de 3140 px de lado); colores identificables (probabilidad 0,89; 5 colores claramente distintos, 3 tonos, colorido 54); formas visibles (probabilidad 0,80; bordes cromáticos en el 22 % del textil); completitud incierta (probabilidad 0,59; toma cerrada, el contorno de la pieza no se ve); estructura simétrica. Puntaje 66.</t>
+          <t>Fotografía deficiente (nitidez 0,69; textil de 3140 px de lado); colores identificables (probabilidad 0,97; 5 colores claramente distintos, 3 tonos, colorido 54); formas visibles (probabilidad 0,94; bordes cromáticos en el 22 % del textil); textil completo (probabilidad 0,90; toma cerrada, el contorno de la pieza no se ve); estructura simétrica. Puntaje 91 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -11277,7 +11277,7 @@
         </is>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>68.5</v>
+        <v>82.3</v>
       </c>
       <c r="AB99" s="4" t="inlineStr">
         <is>
@@ -11291,7 +11291,7 @@
       </c>
       <c r="AD99" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,49; textil de 2055 px de lado); colores identificables (probabilidad 0,93; 3 colores claramente distintos, 3 tonos, colorido 59); formas visibles (probabilidad 0,90; bordes cromáticos en el 47 % del textil); completitud incierta (probabilidad 0,55; compacidad 0,81, lagunas 0,0 %); estructura no evidente. Puntaje 68.</t>
+          <t>Fotografía regular (nitidez 1,49; textil de 2055 px de lado); colores identificables (probabilidad 0,94; 3 colores claramente distintos, 3 tonos, colorido 59); formas visibles (probabilidad 0,92; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,72; compacidad 0,81, lagunas 0,0 %); estructura no evidente. Puntaje 82.</t>
         </is>
       </c>
     </row>
@@ -11399,7 +11399,7 @@
         </is>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>73.3</v>
+        <v>88.3</v>
       </c>
       <c r="AB100" s="4" t="inlineStr">
         <is>
@@ -11413,7 +11413,7 @@
       </c>
       <c r="AD100" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,50; textil de 2177 px de lado); colores identificables (probabilidad 0,96; 4 colores claramente distintos, 3 tonos, colorido 50); formas visibles (probabilidad 0,93; bordes cromáticos en el 42 % del textil); completitud incierta (probabilidad 0,62; compacidad 0,80, lagunas 0,0 %); estructura no evidente. Puntaje 73.</t>
+          <t>Fotografía buena (nitidez 1,50; textil de 2177 px de lado); colores identificables (probabilidad 0,97; 4 colores claramente distintos, 3 tonos, colorido 50); formas visibles (probabilidad 0,96; bordes cromáticos en el 42 % del textil); textil completo (probabilidad 0,83; compacidad 0,80, lagunas 0,0 %); estructura no evidente. Puntaje 88 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -11521,7 +11521,7 @@
         </is>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>73.40000000000001</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="AB101" s="4" t="inlineStr">
         <is>
@@ -11535,7 +11535,7 @@
       </c>
       <c r="AD101" s="4" t="inlineStr">
         <is>
-          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía buena (nitidez 1,58; textil de 3053 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 3 tonos, colorido 51); formas visibles (probabilidad 0,97; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,90; compacidad 0,86, lagunas 0,8 %); estructura repetitiva y simétrica. Puntaje 73.</t>
+          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía buena (nitidez 1,58; textil de 3053 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 3 tonos, colorido 51); formas visibles (probabilidad 0,98; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,92; compacidad 0,86, lagunas 0,8 %); estructura repetitiva y simétrica. Puntaje 94.</t>
         </is>
       </c>
     </row>
@@ -11643,21 +11643,21 @@
         </is>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>68.2</v>
+        <v>83.5</v>
       </c>
       <c r="AB102" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC102" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>posible_figurilla</t>
         </is>
       </c>
       <c r="AD102" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,37; textil de 1774 px de lado); colores identificables (probabilidad 0,90; 4 colores claramente distintos, 3 tonos, colorido 63); formas visibles (probabilidad 0,80; bordes cromáticos en el 35 % del textil); completitud incierta (probabilidad 0,57; compacidad 0,65, lagunas 0,4 %); estructura no evidente. Puntaje 68.</t>
+          <t>El título sugiere una figurilla («Figure»): confirmar si es un textil o un objeto tridimensional. Fotografía regular (nitidez 1,37; textil de 1774 px de lado); colores identificables (probabilidad 0,93; 4 colores claramente distintos, 3 tonos, colorido 63); formas visibles (probabilidad 0,87; bordes cromáticos en el 35 % del textil); textil completo (probabilidad 0,77; compacidad 0,65, lagunas 0,4 %); estructura no evidente. Puntaje 84.</t>
         </is>
       </c>
     </row>
@@ -11765,7 +11765,7 @@
         </is>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>82.09999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="AB103" s="4" t="inlineStr">
         <is>
@@ -11779,7 +11779,7 @@
       </c>
       <c r="AD103" s="4" t="inlineStr">
         <is>
-          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía deficiente (nitidez 0,71; textil de 2797 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 28); formas visibles (probabilidad 0,99; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,90; toma cerrada, el contorno de la pieza no se ve); estructura simétrica. Puntaje 82.</t>
+          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía deficiente (nitidez 0,71; textil de 2797 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 28); formas visibles (probabilidad 0,97; bordes cromáticos en el 23 % del textil); textil completo (probabilidad 0,93; toma cerrada, el contorno de la pieza no se ve); estructura simétrica. Puntaje 92.</t>
         </is>
       </c>
     </row>
@@ -11887,7 +11887,7 @@
         </is>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>78</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="AB104" s="4" t="inlineStr">
         <is>
@@ -11901,7 +11901,7 @@
       </c>
       <c r="AD104" s="4" t="inlineStr">
         <is>
-          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía regular (nitidez 1,09; textil de 2509 px de lado); colores identificables (probabilidad 0,99; 4 colores claramente distintos, 3 tonos, colorido 100); formas visibles (probabilidad 0,96; bordes cromáticos en el 45 % del textil); textil completo (probabilidad 0,89; toma cerrada, el contorno de la pieza no se ve); estructura repetitiva y simétrica. Puntaje 78.</t>
+          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía regular (nitidez 1,09; textil de 2509 px de lado); colores identificables (probabilidad 1,00; 4 colores claramente distintos, 3 tonos, colorido 100); formas visibles (probabilidad 0,97; bordes cromáticos en el 45 % del textil); textil completo (probabilidad 0,95; toma cerrada, el contorno de la pieza no se ve); estructura repetitiva y simétrica. Puntaje 95.</t>
         </is>
       </c>
     </row>
@@ -12009,21 +12009,21 @@
         </is>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>58.5</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="AB105" s="4" t="inlineStr">
         <is>
-          <t>revisar</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="AC105" s="4" t="inlineStr">
         <is>
-          <t>zona_intermedia</t>
+          <t>puntaje</t>
         </is>
       </c>
       <c r="AD105" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 0,73; textil de 3203 px de lado); colores identificables (probabilidad 0,80; 3 colores claramente distintos, 2 tonos, colorido 22); formas visibles (probabilidad 0,77; bordes cromáticos en el 11 % del textil); completitud incierta (probabilidad 0,53; toma cerrada, el contorno de la pieza no se ve); estructura simétrica. Puntaje 59.</t>
+          <t>Fotografía deficiente (nitidez 0,73; textil de 3203 px de lado); colores identificables (probabilidad 0,92; 3 colores claramente distintos, 2 tonos, colorido 22); formas visibles (probabilidad 0,91; bordes cromáticos en el 11 % del textil); textil completo (probabilidad 0,78; toma cerrada, el contorno de la pieza no se ve); estructura simétrica. Puntaje 83.</t>
         </is>
       </c>
     </row>
@@ -12131,7 +12131,7 @@
         </is>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>17.6</v>
+        <v>61.9</v>
       </c>
       <c r="AB106" s="4" t="inlineStr">
         <is>
@@ -12145,7 +12145,7 @@
       </c>
       <c r="AD106" s="4" t="inlineStr">
         <is>
-          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía deficiente (nitidez 0,77; textil de 2078 px de lado); colores no identificables (probabilidad 0,21; 4 colores claramente distintos, 4 tonos, colorido 127); formas no visibles (probabilidad 0,21; bordes cromáticos en el 20 % del textil); textil incompleto (probabilidad 0,10; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 18.</t>
+          <t>Los metadatos registran plumas: los textiles con plumaria quedan fuera del estudio. Fotografía deficiente (nitidez 0,77; textil de 2078 px de lado); colores parcialmente identificables (probabilidad 0,67; 4 colores claramente distintos, 4 tonos, colorido 127); formas visibles (probabilidad 0,73; bordes cromáticos en el 20 % del textil); completitud incierta (probabilidad 0,46; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 62.</t>
         </is>
       </c>
     </row>
@@ -12253,7 +12253,7 @@
         </is>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>64.5</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="AB107" s="4" t="inlineStr">
         <is>
@@ -12267,7 +12267,7 @@
       </c>
       <c r="AD107" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 0,99; textil de 1749 px de lado); colores identificables (probabilidad 0,86; 3 colores claramente distintos, 1 tono, colorido 15); formas visibles (probabilidad 0,81; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,66; compacidad 0,77, lagunas 1,3 %); estructura simétrica. Puntaje 65.</t>
+          <t>Fotografía regular (nitidez 0,99; textil de 1749 px de lado); colores identificables (probabilidad 0,90; 3 colores claramente distintos, 1 tono, colorido 15); formas visibles (probabilidad 0,85; bordes cromáticos en el 13 % del textil); textil completo (probabilidad 0,80; compacidad 0,77, lagunas 1,3 %); estructura simétrica. Puntaje 83.</t>
         </is>
       </c>
     </row>
@@ -12375,7 +12375,7 @@
         </is>
       </c>
       <c r="AA108" s="4" t="n">
-        <v>21.5</v>
+        <v>24.1</v>
       </c>
       <c r="AB108" s="4" t="inlineStr">
         <is>
@@ -12389,7 +12389,7 @@
       </c>
       <c r="AD108" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 0,60; textil de 1139 px de lado); colores no identificables (probabilidad 0,29; 3 colores claramente distintos, 1 tono, colorido 21); formas no visibles (probabilidad 0,20; bordes cromáticos en el 15 % del textil); textil incompleto (probabilidad 0,09; compacidad 0,44, lagunas 0,1 %); estructura no evidente. Puntaje 21.</t>
+          <t>Fotografía deficiente (nitidez 0,60; textil de 1139 px de lado); colores no identificables (probabilidad 0,31; 3 colores claramente distintos, 1 tono, colorido 21); formas no visibles (probabilidad 0,20; bordes cromáticos en el 15 % del textil); textil incompleto (probabilidad 0,18; compacidad 0,44, lagunas 0,1 %); estructura no evidente. Puntaje 24.</t>
         </is>
       </c>
     </row>
@@ -12497,7 +12497,7 @@
         </is>
       </c>
       <c r="AA109" s="4" t="n">
-        <v>73.2</v>
+        <v>98.7</v>
       </c>
       <c r="AB109" s="4" t="inlineStr">
         <is>
@@ -12511,7 +12511,7 @@
       </c>
       <c r="AD109" s="4" t="inlineStr">
         <is>
-          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,06; textil de 3273 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 2 tonos, colorido 63); formas visibles (probabilidad 0,99; bordes cromáticos en el 30 % del textil); textil completo (probabilidad 0,98; compacidad 0,97, lagunas 0,0 %); estructura repetitiva. Puntaje 73.</t>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,06; textil de 3273 px de lado); colores identificables (probabilidad 0,99; 2 colores claramente distintos, 2 tonos, colorido 63); formas visibles (probabilidad 0,99; bordes cromáticos en el 30 % del textil); textil completo (probabilidad 0,99; compacidad 0,97, lagunas 0,0 %); estructura repetitiva. Puntaje 99.</t>
         </is>
       </c>
     </row>
@@ -12603,7 +12603,7 @@
         </is>
       </c>
       <c r="AA110" s="4" t="n">
-        <v>73.8</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="AB110" s="4" t="inlineStr">
         <is>
@@ -12617,7 +12617,7 @@
       </c>
       <c r="AD110" s="4" t="inlineStr">
         <is>
-          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,92; textil de 2142 px de lado); colores identificables (probabilidad 0,97; 2 colores claramente distintos, 1 tono, colorido 30); formas visibles (probabilidad 0,97; bordes cromáticos en el 31 % del textil); textil completo (probabilidad 0,95; compacidad 0,96, lagunas 0,0 %); estructura no evidente. Puntaje 74.</t>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,92; textil de 2142 px de lado); colores identificables (probabilidad 0,95; 2 colores claramente distintos, 1 tono, colorido 30); formas visibles (probabilidad 0,96; bordes cromáticos en el 31 % del textil); textil completo (probabilidad 0,96; compacidad 0,96, lagunas 0,0 %); estructura no evidente. Puntaje 96.</t>
         </is>
       </c>
     </row>
@@ -12709,7 +12709,7 @@
         </is>
       </c>
       <c r="AA111" s="4" t="n">
-        <v>75.90000000000001</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="AB111" s="4" t="inlineStr">
         <is>
@@ -12723,7 +12723,7 @@
       </c>
       <c r="AD111" s="4" t="inlineStr">
         <is>
-          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,73; textil de 1410 px de lado); colores identificables (probabilidad 0,96; 2 colores claramente distintos, 0 tonos, colorido 11); formas visibles (probabilidad 0,95; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,93; compacidad 0,88, lagunas 0,0 %); estructura no evidente. Puntaje 76.</t>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,73; textil de 1410 px de lado); colores identificables (probabilidad 0,93; 2 colores claramente distintos, 0 tonos, colorido 11); formas visibles (probabilidad 0,94; bordes cromáticos en el 43 % del textil); textil completo (probabilidad 0,93; compacidad 0,88, lagunas 0,0 %); estructura no evidente. Puntaje 93.</t>
         </is>
       </c>
     </row>
@@ -12831,7 +12831,7 @@
         </is>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>76.40000000000001</v>
+        <v>57.4</v>
       </c>
       <c r="AB112" s="4" t="inlineStr">
         <is>
@@ -12845,7 +12845,7 @@
       </c>
       <c r="AD112" s="4" t="inlineStr">
         <is>
-          <t>El textil mide 288 px de lado en la imagen institucional (mínimo 300). Fotografía buena (nitidez 2,99; textil de 288 px de lado); colores identificables (probabilidad 0,98; 1 color claramente distinto, 2 tonos, colorido 17); formas visibles (probabilidad 0,97; bordes cromáticos en el 3 % del textil); textil completo (probabilidad 0,89; compacidad 0,51, lagunas 0,0 %); estructura no evidente. Puntaje 76.</t>
+          <t>El textil mide 288 px de lado en la imagen institucional (mínimo 300). Fotografía buena (nitidez 2,99; textil de 288 px de lado); colores parcialmente identificables (probabilidad 0,69; 1 color claramente distinto, 2 tonos, colorido 17); formas visibles (probabilidad 0,70; bordes cromáticos en el 3 % del textil); textil incompleto (probabilidad 0,39; compacidad 0,51, lagunas 0,0 %); estructura no evidente. Puntaje 57.</t>
         </is>
       </c>
     </row>
@@ -12953,7 +12953,7 @@
         </is>
       </c>
       <c r="AA113" s="4" t="n">
-        <v>74.5</v>
+        <v>75.2</v>
       </c>
       <c r="AB113" s="4" t="inlineStr">
         <is>
@@ -12967,7 +12967,7 @@
       </c>
       <c r="AD113" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 0,64; textil de 1599 px de lado); colores identificables (probabilidad 0,94; 4 colores claramente distintos, 5 tonos, colorido 38); formas visibles (probabilidad 0,92; bordes cromáticos en el 17 % del textil); completitud incierta (probabilidad 0,42; compacidad 0,76, lagunas 0,2 %); estructura no evidente. Puntaje 75.</t>
+          <t>Fotografía deficiente (nitidez 0,64; textil de 1599 px de lado); colores identificables (probabilidad 0,98; 4 colores claramente distintos, 5 tonos, colorido 38); formas visibles (probabilidad 0,97; bordes cromáticos en el 17 % del textil); completitud incierta (probabilidad 0,66; compacidad 0,76, lagunas 0,2 %); estructura no evidente. Puntaje 75.</t>
         </is>
       </c>
     </row>
@@ -13075,21 +13075,21 @@
         </is>
       </c>
       <c r="AA114" s="4" t="n">
-        <v>41</v>
+        <v>46.7</v>
       </c>
       <c r="AB114" s="4" t="inlineStr">
         <is>
-          <t>descartar</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC114" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD114" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,08; textil de 2550 px de lado); colores parcialmente identificables (probabilidad 0,52; 2 colores claramente distintos, 1 tono, colorido 18); formas parcialmente visibles (probabilidad 0,61; bordes cromáticos en el 19 % del textil); textil incompleto (probabilidad 0,18; compacidad 0,79, lagunas 0,3 %, el título dice «fragment»); estructura no evidente. Puntaje 41.</t>
+          <t>Fotografía regular (nitidez 1,08; textil de 2550 px de lado); colores parcialmente identificables (probabilidad 0,58; 2 colores claramente distintos, 1 tono, colorido 18); formas visibles (probabilidad 0,72; bordes cromáticos en el 19 % del textil); textil incompleto (probabilidad 0,19; compacidad 0,79, lagunas 0,3 %, el título dice «fragment»); estructura no evidente. Puntaje 47.</t>
         </is>
       </c>
     </row>
@@ -13197,21 +13197,21 @@
         </is>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>70.40000000000001</v>
+        <v>59.5</v>
       </c>
       <c r="AB115" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC115" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD115" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,28; textil de 920 px de lado); colores identificables (probabilidad 0,90; 3 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,80; bordes cromáticos en el 57 % del textil); textil incompleto (probabilidad 0,39; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 70.</t>
+          <t>Fotografía regular (nitidez 1,28; textil de 920 px de lado); colores identificables (probabilidad 0,92; 3 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,85; bordes cromáticos en el 57 % del textil); textil incompleto (probabilidad 0,32; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 60.</t>
         </is>
       </c>
     </row>
@@ -13319,21 +13319,21 @@
         </is>
       </c>
       <c r="AA116" s="4" t="n">
-        <v>72.5</v>
+        <v>63.5</v>
       </c>
       <c r="AB116" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC116" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD116" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,26; textil de 922 px de lado); colores identificables (probabilidad 0,91; 3 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,81; bordes cromáticos en el 57 % del textil); completitud incierta (probabilidad 0,45; compacidad 0,68, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 72.</t>
+          <t>Fotografía regular (nitidez 1,26; textil de 922 px de lado); colores identificables (probabilidad 0,93; 3 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,87; bordes cromáticos en el 57 % del textil); textil incompleto (probabilidad 0,38; compacidad 0,68, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
         </is>
       </c>
     </row>
@@ -13441,21 +13441,21 @@
         </is>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>72.2</v>
+        <v>61.4</v>
       </c>
       <c r="AB117" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC117" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD117" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,28; textil de 918 px de lado); colores identificables (probabilidad 0,91; 3 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,82; bordes cromáticos en el 57 % del textil); completitud incierta (probabilidad 0,43; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 72.</t>
+          <t>Fotografía regular (nitidez 1,28; textil de 918 px de lado); colores identificables (probabilidad 0,93; 3 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,86; bordes cromáticos en el 57 % del textil); textil incompleto (probabilidad 0,35; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 61.</t>
         </is>
       </c>
     </row>
@@ -13563,21 +13563,21 @@
         </is>
       </c>
       <c r="AA118" s="4" t="n">
-        <v>69.59999999999999</v>
+        <v>58.1</v>
       </c>
       <c r="AB118" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC118" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD118" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,28; textil de 925 px de lado); colores identificables (probabilidad 0,88; 2 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,80; bordes cromáticos en el 57 % del textil); completitud incierta (probabilidad 0,43; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 70.</t>
+          <t>Fotografía regular (nitidez 1,28; textil de 925 px de lado); colores identificables (probabilidad 0,91; 2 colores claramente distintos, 3 tonos, colorido 47); formas visibles (probabilidad 0,84; bordes cromáticos en el 57 % del textil); textil incompleto (probabilidad 0,30; compacidad 0,67, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 58.</t>
         </is>
       </c>
     </row>
@@ -13669,21 +13669,21 @@
         </is>
       </c>
       <c r="AA119" s="4" t="n">
-        <v>52.8</v>
+        <v>80.2</v>
       </c>
       <c r="AB119" s="4" t="inlineStr">
         <is>
-          <t>revisar</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="AC119" s="4" t="inlineStr">
         <is>
-          <t>zona_intermedia</t>
+          <t>puntaje</t>
         </is>
       </c>
       <c r="AD119" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,54; textil de 2608 px de lado); colores identificables (probabilidad 0,72; 1 color claramente distinto, 2 tonos, colorido 22); formas visibles (probabilidad 0,75; bordes cromáticos en el 11 % del textil); completitud incierta (probabilidad 0,56; compacidad 0,73, lagunas 0,5 %); estructura no evidente. Puntaje 53.</t>
+          <t>Fotografía buena (nitidez 1,54; textil de 2608 px de lado); colores identificables (probabilidad 0,82; 1 color claramente distinto, 2 tonos, colorido 22); formas visibles (probabilidad 0,84; bordes cromáticos en el 11 % del textil); textil completo (probabilidad 0,74; compacidad 0,73, lagunas 0,5 %); estructura no evidente. Puntaje 80.</t>
         </is>
       </c>
     </row>
@@ -13791,7 +13791,7 @@
         </is>
       </c>
       <c r="AA120" s="4" t="n">
-        <v>85.8</v>
+        <v>92.3</v>
       </c>
       <c r="AB120" s="4" t="inlineStr">
         <is>
@@ -13805,7 +13805,7 @@
       </c>
       <c r="AD120" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,18; textil de 1118 px de lado); colores identificables (probabilidad 0,99; 4 colores claramente distintos, 3 tonos, colorido 46); formas visibles (probabilidad 0,97; bordes cromáticos en el 68 % del textil); textil completo (probabilidad 0,87; compacidad 0,89, lagunas 0,0 %); estructura no evidente. Puntaje 86 (imagen de referencia sugerida).</t>
+          <t>Fotografía regular (nitidez 1,18; textil de 1118 px de lado); colores identificables (probabilidad 0,99; 4 colores claramente distintos, 3 tonos, colorido 46); formas visibles (probabilidad 0,98; bordes cromáticos en el 68 % del textil); textil completo (probabilidad 0,90; compacidad 0,89, lagunas 0,0 %); estructura no evidente. Puntaje 92 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -13913,7 +13913,7 @@
         </is>
       </c>
       <c r="AA121" s="4" t="n">
-        <v>82.40000000000001</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="AB121" s="4" t="inlineStr">
         <is>
@@ -13927,7 +13927,7 @@
       </c>
       <c r="AD121" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,30; textil de 842 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 2 tonos, colorido 37); formas visibles (probabilidad 0,96; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,95; compacidad 0,79, lagunas 0,0 %); estructura no evidente. Puntaje 82 (imagen de referencia sugerida).</t>
+          <t>Fotografía buena (nitidez 2,30; textil de 842 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 2 tonos, colorido 37); formas visibles (probabilidad 0,94; bordes cromáticos en el 47 % del textil); textil completo (probabilidad 0,93; compacidad 0,79, lagunas 0,0 %); estructura no evidente. Puntaje 94 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -14035,7 +14035,7 @@
         </is>
       </c>
       <c r="AA122" s="4" t="n">
-        <v>72.5</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="AB122" s="4" t="inlineStr">
         <is>
@@ -14049,7 +14049,7 @@
       </c>
       <c r="AD122" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,23; textil de 1167 px de lado); colores identificables (probabilidad 0,91; 3 colores claramente distintos, 3 tonos, colorido 40); formas visibles (probabilidad 0,84; bordes cromáticos en el 42 % del textil); completitud incierta (probabilidad 0,49; compacidad 0,71, lagunas 0,0 %); estructura no evidente. Puntaje 72.</t>
+          <t>Fotografía regular (nitidez 1,23; textil de 1167 px de lado); colores identificables (probabilidad 0,90; 3 colores claramente distintos, 3 tonos, colorido 40); formas visibles (probabilidad 0,86; bordes cromáticos en el 42 % del textil); completitud incierta (probabilidad 0,55; compacidad 0,71, lagunas 0,0 %); estructura no evidente. Puntaje 72.</t>
         </is>
       </c>
     </row>
@@ -14157,7 +14157,7 @@
         </is>
       </c>
       <c r="AA123" s="4" t="n">
-        <v>48.4</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="AB123" s="4" t="inlineStr">
         <is>
@@ -14171,7 +14171,7 @@
       </c>
       <c r="AD123" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,84; textil de 1632 px de lado); colores parcialmente identificables (probabilidad 0,64; 2 colores claramente distintos, 1 tono, colorido 20); formas parcialmente visibles (probabilidad 0,61; bordes cromáticos en el 16 % del textil); completitud incierta (probabilidad 0,53; compacidad 0,61, lagunas 0,0 %); estructura no evidente. Puntaje 48.</t>
+          <t>Fotografía buena (nitidez 1,84; textil de 1632 px de lado); colores parcialmente identificables (probabilidad 0,63; 2 colores claramente distintos, 1 tono, colorido 20); formas parcialmente visibles (probabilidad 0,61; bordes cromáticos en el 16 % del textil); completitud incierta (probabilidad 0,60; compacidad 0,61, lagunas 0,0 %); estructura no evidente. Puntaje 67.</t>
         </is>
       </c>
     </row>
@@ -14279,21 +14279,21 @@
         </is>
       </c>
       <c r="AA124" s="4" t="n">
-        <v>66.8</v>
+        <v>64.7</v>
       </c>
       <c r="AB124" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC124" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD124" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 0,27; textil de 1975 px de lado); colores identificables (probabilidad 0,87; 2 colores claramente distintos, 2 tonos, colorido 16); formas visibles (probabilidad 0,85; bordes cromáticos en el 8 % del textil); completitud incierta (probabilidad 0,49; toma cerrada, el contorno de la pieza no se ve, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 67.</t>
+          <t>Fotografía deficiente (nitidez 0,27; textil de 1975 px de lado); colores identificables (probabilidad 0,94; 2 colores claramente distintos, 2 tonos, colorido 16); formas visibles (probabilidad 0,90; bordes cromáticos en el 8 % del textil); completitud incierta (probabilidad 0,51; toma cerrada, el contorno de la pieza no se ve, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 65.</t>
         </is>
       </c>
     </row>
@@ -14401,21 +14401,21 @@
         </is>
       </c>
       <c r="AA125" s="4" t="n">
-        <v>71.59999999999999</v>
+        <v>66.8</v>
       </c>
       <c r="AB125" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC125" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD125" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 1,00; textil de 737 px de lado); colores identificables (probabilidad 0,89; 2 colores claramente distintos, 2 tonos, colorido 27); formas visibles (probabilidad 0,89; bordes cromáticos en el 33 % del textil); completitud incierta (probabilidad 0,64; compacidad 0,87, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 72.</t>
+          <t>Fotografía deficiente (nitidez 1,00; textil de 737 px de lado); colores identificables (probabilidad 0,92; 2 colores claramente distintos, 2 tonos, colorido 27); formas visibles (probabilidad 0,94; bordes cromáticos en el 33 % del textil); completitud incierta (probabilidad 0,51; compacidad 0,87, lagunas 0,0 %, el título dice «fragment»); estructura repetitiva y simétrica. Puntaje 67.</t>
         </is>
       </c>
     </row>
@@ -14523,7 +14523,7 @@
         </is>
       </c>
       <c r="AA126" s="4" t="n">
-        <v>78.8</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="AB126" s="4" t="inlineStr">
         <is>
@@ -14537,7 +14537,7 @@
       </c>
       <c r="AD126" s="4" t="inlineStr">
         <is>
-          <t>Fotografía deficiente (nitidez 0,96; textil de 815 px de lado); colores identificables (probabilidad 0,98; 2 colores claramente distintos, 2 tonos, colorido 27); formas visibles (probabilidad 0,95; bordes cromáticos en el 25 % del textil); textil completo (probabilidad 0,82; compacidad 0,88, lagunas 0,0 %, el título dice «fragment»); estructura simétrica. Puntaje 79 (imagen de referencia sugerida).</t>
+          <t>Fotografía deficiente (nitidez 0,96; textil de 815 px de lado); colores identificables (probabilidad 0,97; 2 colores claramente distintos, 2 tonos, colorido 27); formas visibles (probabilidad 0,91; bordes cromáticos en el 25 % del textil); completitud incierta (probabilidad 0,65; compacidad 0,88, lagunas 0,0 %, el título dice «fragment»); estructura simétrica. Puntaje 76.</t>
         </is>
       </c>
     </row>
@@ -14629,7 +14629,7 @@
         </is>
       </c>
       <c r="AA127" s="4" t="n">
-        <v>70.7</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="AB127" s="4" t="inlineStr">
         <is>
@@ -14643,7 +14643,7 @@
       </c>
       <c r="AD127" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,39; textil de 2469 px de lado); colores identificables (probabilidad 0,96; 1 color claramente distinto, 2 tonos, colorido 18); formas visibles (probabilidad 0,97; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,91; compacidad 0,90, lagunas 0,0 %); estructura repetitiva. Puntaje 71.</t>
+          <t>Fotografía buena (nitidez 1,39; textil de 2469 px de lado); colores identificables (probabilidad 0,97; 1 color claramente distinto, 2 tonos, colorido 18); formas visibles (probabilidad 0,98; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,93; compacidad 0,90, lagunas 0,0 %); estructura repetitiva. Puntaje 94 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -14751,21 +14751,21 @@
         </is>
       </c>
       <c r="AA128" s="4" t="n">
-        <v>30.8</v>
+        <v>40.2</v>
       </c>
       <c r="AB128" s="4" t="inlineStr">
         <is>
-          <t>descartar</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC128" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD128" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,20; textil de 1289 px de lado); colores no identificables (probabilidad 0,27; 2 colores claramente distintos, 1 tono, colorido 16); formas no visibles (probabilidad 0,27; bordes cromáticos en el 19 % del textil); textil incompleto (probabilidad 0,20; compacidad 0,37, lagunas 7,2 %); estructura no evidente. Puntaje 31.</t>
+          <t>Fotografía regular (nitidez 1,20; textil de 1289 px de lado); colores no identificables (probabilidad 0,32; 2 colores claramente distintos, 1 tono, colorido 16); formas no visibles (probabilidad 0,31; bordes cromáticos en el 19 % del textil); textil incompleto (probabilidad 0,32; compacidad 0,37, lagunas 7,2 %); estructura no evidente. Puntaje 40.</t>
         </is>
       </c>
     </row>
@@ -14873,7 +14873,7 @@
         </is>
       </c>
       <c r="AA129" s="4" t="n">
-        <v>47.8</v>
+        <v>56.9</v>
       </c>
       <c r="AB129" s="4" t="inlineStr">
         <is>
@@ -14887,7 +14887,7 @@
       </c>
       <c r="AD129" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,56; textil de 2124 px de lado); colores parcialmente identificables (probabilidad 0,56; 1 color claramente distinto, 2 tonos, colorido 27); formas parcialmente visibles (probabilidad 0,69; bordes cromáticos en el 13 % del textil); textil incompleto (probabilidad 0,37; compacidad 0,55, lagunas 8,1 %, el título dice «fragment»); estructura no evidente. Puntaje 48.</t>
+          <t>Fotografía buena (nitidez 2,56; textil de 2124 px de lado); colores parcialmente identificables (probabilidad 0,62; 1 color claramente distinto, 2 tonos, colorido 27); formas visibles (probabilidad 0,70; bordes cromáticos en el 13 % del textil); textil incompleto (probabilidad 0,32; compacidad 0,55, lagunas 8,1 %, el título dice «fragment»); estructura no evidente. Puntaje 57.</t>
         </is>
       </c>
     </row>
@@ -14995,21 +14995,21 @@
         </is>
       </c>
       <c r="AA130" s="4" t="n">
-        <v>58.9</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="AB130" s="4" t="inlineStr">
         <is>
-          <t>revisar</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="AC130" s="4" t="inlineStr">
         <is>
-          <t>zona_intermedia</t>
+          <t>puntaje</t>
         </is>
       </c>
       <c r="AD130" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,43; textil de 2361 px de lado); colores identificables (probabilidad 0,74; 1 color claramente distinto, 2 tonos, colorido 29); formas visibles (probabilidad 0,85; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,62; compacidad 0,76, lagunas 4,3 %, el título dice «fragment»); estructura no evidente. Puntaje 59.</t>
+          <t>Fotografía buena (nitidez 2,43; textil de 2361 px de lado); colores identificables (probabilidad 0,80; 1 color claramente distinto, 2 tonos, colorido 29); formas visibles (probabilidad 0,88; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,59; compacidad 0,76, lagunas 4,3 %, el título dice «fragment»); estructura no evidente. Puntaje 76.</t>
         </is>
       </c>
     </row>
@@ -15117,7 +15117,7 @@
         </is>
       </c>
       <c r="AA131" s="4" t="n">
-        <v>53.5</v>
+        <v>63.4</v>
       </c>
       <c r="AB131" s="4" t="inlineStr">
         <is>
@@ -15131,7 +15131,7 @@
       </c>
       <c r="AD131" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,91; textil de 2166 px de lado); colores parcialmente identificables (probabilidad 0,64; 1 color claramente distinto, 2 tonos, colorido 30); formas visibles (probabilidad 0,76; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,43; compacidad 0,66, lagunas 8,9 %, el título dice «fragment»); estructura no evidente. Puntaje 54.</t>
+          <t>Fotografía buena (nitidez 1,91; textil de 2166 px de lado); colores identificables (probabilidad 0,74; 1 color claramente distinto, 2 tonos, colorido 30); formas visibles (probabilidad 0,79; bordes cromáticos en el 13 % del textil); completitud incierta (probabilidad 0,41; compacidad 0,66, lagunas 8,9 %, el título dice «fragment»); estructura no evidente. Puntaje 63.</t>
         </is>
       </c>
     </row>
@@ -15239,7 +15239,7 @@
         </is>
       </c>
       <c r="AA132" s="4" t="n">
-        <v>14.1</v>
+        <v>15.8</v>
       </c>
       <c r="AB132" s="4" t="inlineStr">
         <is>
@@ -15253,7 +15253,7 @@
       </c>
       <c r="AD132" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,20; textil de 2285 px de lado); colores no identificables (probabilidad 0,18; 2 colores claramente distintos, 2 tonos, colorido 42); formas no visibles (probabilidad 0,15; bordes cromáticos en el 31 % del textil); textil incompleto (probabilidad 0,01; compacidad 0,07, lagunas 2,0 %, el título dice «fragment»); estructura no evidente. Puntaje 14.</t>
+          <t>Fotografía regular (nitidez 1,20; textil de 2285 px de lado); colores parcialmente identificables (probabilidad 0,50; 2 colores claramente distintos, 2 tonos, colorido 42); formas no visibles (probabilidad 0,31; bordes cromáticos en el 31 % del textil); textil incompleto (probabilidad 0,01; compacidad 0,07, lagunas 2,0 %, el título dice «fragment»); estructura no evidente. Puntaje 16.</t>
         </is>
       </c>
     </row>
@@ -15345,7 +15345,7 @@
         </is>
       </c>
       <c r="AA133" s="4" t="n">
-        <v>61.5</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="AB133" s="4" t="inlineStr">
         <is>
@@ -15359,7 +15359,7 @@
       </c>
       <c r="AD133" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,04; textil de 1825 px de lado); colores identificables (probabilidad 0,78; 2 colores claramente distintos, 1 tono, colorido 23); formas visibles (probabilidad 0,79; bordes cromáticos en el 17 % del textil); completitud incierta (probabilidad 0,62; compacidad 0,70, lagunas 0,0 %); estructura repetitiva. Puntaje 61.</t>
+          <t>Fotografía regular (nitidez 1,04; textil de 1825 px de lado); colores identificables (probabilidad 0,80; 2 colores claramente distintos, 1 tono, colorido 23); formas visibles (probabilidad 0,83; bordes cromáticos en el 17 % del textil); textil completo (probabilidad 0,73; compacidad 0,70, lagunas 0,0 %); estructura repetitiva. Puntaje 78.</t>
         </is>
       </c>
     </row>
@@ -15467,21 +15467,21 @@
         </is>
       </c>
       <c r="AA134" s="4" t="n">
-        <v>28.6</v>
+        <v>40.5</v>
       </c>
       <c r="AB134" s="4" t="inlineStr">
         <is>
-          <t>descartar</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC134" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD134" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,22; textil de 1284 px de lado); colores no identificables (probabilidad 0,28; 2 colores claramente distintos, 1 tono, colorido 16); formas no visibles (probabilidad 0,27; bordes cromáticos en el 17 % del textil); textil incompleto (probabilidad 0,21; compacidad 0,35, lagunas 3,9 %); estructura repetitiva. Puntaje 29.</t>
+          <t>Fotografía regular (nitidez 1,22; textil de 1284 px de lado); colores no identificables (probabilidad 0,33; 2 colores claramente distintos, 1 tono, colorido 16); formas no visibles (probabilidad 0,32; bordes cromáticos en el 17 % del textil); textil incompleto (probabilidad 0,31; compacidad 0,35, lagunas 3,9 %); estructura repetitiva. Puntaje 40.</t>
         </is>
       </c>
     </row>
@@ -15589,21 +15589,21 @@
         </is>
       </c>
       <c r="AA135" s="4" t="n">
-        <v>64.8</v>
+        <v>65</v>
       </c>
       <c r="AB135" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC135" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD135" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 1,77; textil de 1155 px de lado); colores identificables (probabilidad 0,81; 2 colores claramente distintos, 3 tonos, colorido 43); formas parcialmente visibles (probabilidad 0,67; bordes cromáticos en el 50 % del textil); completitud incierta (probabilidad 0,49; compacidad 0,35, lagunas 0,0 %); estructura no evidente. Puntaje 65.</t>
+          <t>Fotografía buena (nitidez 1,77; textil de 1155 px de lado); colores identificables (probabilidad 0,80; 2 colores claramente distintos, 3 tonos, colorido 43); formas parcialmente visibles (probabilidad 0,66; bordes cromáticos en el 50 % del textil); completitud incierta (probabilidad 0,50; compacidad 0,35, lagunas 0,0 %); estructura no evidente. Puntaje 65.</t>
         </is>
       </c>
     </row>
@@ -15711,21 +15711,21 @@
         </is>
       </c>
       <c r="AA136" s="4" t="n">
-        <v>59.5</v>
+        <v>84.3</v>
       </c>
       <c r="AB136" s="4" t="inlineStr">
         <is>
-          <t>revisar</t>
+          <t>principal</t>
         </is>
       </c>
       <c r="AC136" s="4" t="inlineStr">
         <is>
-          <t>zona_intermedia</t>
+          <t>puntaje</t>
         </is>
       </c>
       <c r="AD136" s="4" t="inlineStr">
         <is>
-          <t>Fotografía buena (nitidez 2,03; textil de 2930 px de lado); colores identificables (probabilidad 0,78; 1 color claramente distinto, 1 tono, colorido 30); formas visibles (probabilidad 0,87; bordes cromáticos en el 4 % del textil); textil completo (probabilidad 0,78; compacidad 0,88, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 59.</t>
+          <t>Fotografía buena (nitidez 2,03; textil de 2930 px de lado); colores identificables (probabilidad 0,79; 1 color claramente distinto, 1 tono, colorido 30); formas visibles (probabilidad 0,89; bordes cromáticos en el 4 % del textil); textil completo (probabilidad 0,77; compacidad 0,88, lagunas 0,0 %, el título dice «fragment»); estructura no evidente. Puntaje 84.</t>
         </is>
       </c>
     </row>
@@ -15833,7 +15833,7 @@
         </is>
       </c>
       <c r="AA137" s="4" t="n">
-        <v>60.2</v>
+        <v>85.7</v>
       </c>
       <c r="AB137" s="4" t="inlineStr">
         <is>
@@ -15847,7 +15847,7 @@
       </c>
       <c r="AD137" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,28; textil de 2912 px de lado); colores identificables (probabilidad 0,79; 2 colores claramente distintos, 2 tonos, colorido 48); formas visibles (probabilidad 0,83; bordes cromáticos en el 12 % del textil); completitud incierta (probabilidad 0,69; compacidad 0,84, lagunas 0,0 %); estructura repetitiva. Puntaje 60.</t>
+          <t>Fotografía regular (nitidez 1,28; textil de 2912 px de lado); colores identificables (probabilidad 0,84; 2 colores claramente distintos, 2 tonos, colorido 48); formas visibles (probabilidad 0,89; bordes cromáticos en el 12 % del textil); textil completo (probabilidad 0,80; compacidad 0,84, lagunas 0,0 %); estructura repetitiva. Puntaje 86 (imagen de referencia sugerida).</t>
         </is>
       </c>
     </row>
@@ -15939,7 +15939,7 @@
         </is>
       </c>
       <c r="AA138" s="4" t="n">
-        <v>78</v>
+        <v>97.7</v>
       </c>
       <c r="AB138" s="4" t="inlineStr">
         <is>
@@ -15953,7 +15953,7 @@
       </c>
       <c r="AD138" s="4" t="inlineStr">
         <is>
-          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,01; textil de 2470 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 3 tonos, colorido 33); formas visibles (probabilidad 0,99; bordes cromáticos en el 36 % del textil); textil completo (probabilidad 0,95; compacidad 0,97, lagunas 0,0 %); estructura no evidente. Puntaje 78.</t>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 2,01; textil de 2470 px de lado); colores identificables (probabilidad 1,00; 3 colores claramente distintos, 3 tonos, colorido 33); formas visibles (probabilidad 0,99; bordes cromáticos en el 36 % del textil); textil completo (probabilidad 0,97; compacidad 0,97, lagunas 0,0 %); estructura no evidente. Puntaje 98.</t>
         </is>
       </c>
     </row>
@@ -16045,7 +16045,7 @@
         </is>
       </c>
       <c r="AA139" s="4" t="n">
-        <v>78.09999999999999</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="AB139" s="4" t="inlineStr">
         <is>
@@ -16059,7 +16059,7 @@
       </c>
       <c r="AD139" s="4" t="inlineStr">
         <is>
-          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 1,86; textil de 2462 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 2 tonos, colorido 33); formas visibles (probabilidad 0,99; bordes cromáticos en el 33 % del textil); textil completo (probabilidad 0,96; compacidad 0,98, lagunas 0,0 %); estructura no evidente. Puntaje 78.</t>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 1,86; textil de 2462 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 2 tonos, colorido 33); formas visibles (probabilidad 0,99; bordes cromáticos en el 33 % del textil); textil completo (probabilidad 0,98; compacidad 0,98, lagunas 0,0 %); estructura no evidente. Puntaje 98.</t>
         </is>
       </c>
     </row>
@@ -16167,21 +16167,21 @@
         </is>
       </c>
       <c r="AA140" s="4" t="n">
-        <v>62.7</v>
+        <v>62.2</v>
       </c>
       <c r="AB140" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC140" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD140" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,55; textil de 530 px de lado); colores identificables (probabilidad 0,76; 2 colores claramente distintos, 1 tono, colorido 24); formas parcialmente visibles (probabilidad 0,52; bordes cromáticos en el 44 % del textil); textil completo (probabilidad 0,70; compacidad 0,44, lagunas 0,0 %); estructura no evidente. Puntaje 63.</t>
+          <t>Fotografía regular (nitidez 1,55; textil de 530 px de lado); colores parcialmente identificables (probabilidad 0,69; 2 colores claramente distintos, 1 tono, colorido 24); formas parcialmente visibles (probabilidad 0,42; bordes cromáticos en el 44 % del textil); completitud incierta (probabilidad 0,63; compacidad 0,44, lagunas 0,0 %); estructura no evidente. Puntaje 62.</t>
         </is>
       </c>
     </row>
@@ -16289,21 +16289,21 @@
         </is>
       </c>
       <c r="AA141" s="4" t="n">
-        <v>64.8</v>
+        <v>58.6</v>
       </c>
       <c r="AB141" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC141" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD141" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,54; textil de 500 px de lado); colores identificables (probabilidad 0,77; 2 colores claramente distintos, 0 tonos, colorido 12); formas parcialmente visibles (probabilidad 0,54; bordes cromáticos en el 60 % del textil); completitud incierta (probabilidad 0,65; compacidad 0,52, lagunas 0,0 %); estructura no evidente. Puntaje 65.</t>
+          <t>Fotografía regular (nitidez 1,54; textil de 500 px de lado); colores parcialmente identificables (probabilidad 0,68; 2 colores claramente distintos, 0 tonos, colorido 12); formas parcialmente visibles (probabilidad 0,45; bordes cromáticos en el 60 % del textil); completitud incierta (probabilidad 0,55; compacidad 0,52, lagunas 0,0 %); estructura no evidente. Puntaje 59.</t>
         </is>
       </c>
     </row>
@@ -16411,21 +16411,21 @@
         </is>
       </c>
       <c r="AA142" s="4" t="n">
-        <v>68.7</v>
+        <v>48.7</v>
       </c>
       <c r="AB142" s="4" t="inlineStr">
         <is>
-          <t>principal</t>
+          <t>revisar</t>
         </is>
       </c>
       <c r="AC142" s="4" t="inlineStr">
         <is>
-          <t>puntaje</t>
+          <t>zona_intermedia</t>
         </is>
       </c>
       <c r="AD142" s="4" t="inlineStr">
         <is>
-          <t>Fotografía regular (nitidez 1,17; textil de 706 px de lado); colores identificables (probabilidad 0,84; 1 color claramente distinto, 2 tonos, colorido 20); formas parcialmente visibles (probabilidad 0,66; bordes cromáticos en el 27 % del textil); completitud incierta (probabilidad 0,48; compacidad 0,35, lagunas 6,9 %); estructura simétrica. Puntaje 69.</t>
+          <t>Fotografía regular (nitidez 1,17; textil de 706 px de lado); colores identificables (probabilidad 0,78; 1 color claramente distinto, 2 tonos, colorido 20); formas parcialmente visibles (probabilidad 0,42; bordes cromáticos en el 27 % del textil); textil incompleto (probabilidad 0,37; compacidad 0,35, lagunas 6,9 %); estructura simétrica. Puntaje 49.</t>
         </is>
       </c>
     </row>
@@ -16533,7 +16533,7 @@
         </is>
       </c>
       <c r="AA143" s="4" t="n">
-        <v>81.5</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="AB143" s="4" t="inlineStr">
         <is>
@@ -16547,7 +16547,7 @@
       </c>
       <c r="AD143" s="4" t="inlineStr">
         <is>
-          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 1,84; textil de 2602 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 2 tonos, colorido 48); formas visibles (probabilidad 0,98; bordes cromáticos en el 39 % del textil); textil completo (probabilidad 0,97; compacidad 0,83, lagunas 0,0 %); estructura simétrica. Puntaje 81.</t>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía buena (nitidez 1,84; textil de 2602 px de lado); colores identificables (probabilidad 0,99; 3 colores claramente distintos, 2 tonos, colorido 48); formas visibles (probabilidad 0,98; bordes cromáticos en el 39 % del textil); textil completo (probabilidad 0,99; compacidad 0,83, lagunas 0,0 %); estructura simétrica. Puntaje 98.</t>
         </is>
       </c>
     </row>
@@ -16655,7 +16655,7 @@
         </is>
       </c>
       <c r="AA144" s="4" t="n">
-        <v>86.59999999999999</v>
+        <v>97.5</v>
       </c>
       <c r="AB144" s="4" t="inlineStr">
         <is>
@@ -16669,7 +16669,7 @@
       </c>
       <c r="AD144" s="4" t="inlineStr">
         <is>
-          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía regular (nitidez 0,92; textil de 3022 px de lado); colores identificables (probabilidad 1,00; 4 colores claramente distintos, 3 tonos, colorido 64); formas visibles (probabilidad 1,00; bordes cromáticos en el 64 % del textil); textil completo (probabilidad 0,99; compacidad 0,95, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 87.</t>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía regular (nitidez 0,92; textil de 3022 px de lado); colores identificables (probabilidad 1,00; 4 colores claramente distintos, 3 tonos, colorido 64); formas visibles (probabilidad 1,00; bordes cromáticos en el 64 % del textil); textil completo (probabilidad 0,99; compacidad 0,95, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 98.</t>
         </is>
       </c>
     </row>
@@ -16777,7 +16777,7 @@
         </is>
       </c>
       <c r="AA145" s="4" t="n">
-        <v>84.2</v>
+        <v>98.2</v>
       </c>
       <c r="AB145" s="4" t="inlineStr">
         <is>
@@ -16791,7 +16791,7 @@
       </c>
       <c r="AD145" s="4" t="inlineStr">
         <is>
-          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía regular (nitidez 0,92; textil de 2405 px de lado); colores identificables (probabilidad 1,00; 4 colores claramente distintos, 3 tonos, colorido 63); formas visibles (probabilidad 1,00; bordes cromáticos en el 60 % del textil); textil completo (probabilidad 0,98; compacidad 0,94, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 84.</t>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía regular (nitidez 0,92; textil de 2405 px de lado); colores identificables (probabilidad 1,00; 4 colores claramente distintos, 3 tonos, colorido 63); formas visibles (probabilidad 1,00; bordes cromáticos en el 60 % del textil); textil completo (probabilidad 0,99; compacidad 0,94, lagunas 0,0 %); estructura repetitiva y simétrica. Puntaje 98.</t>
         </is>
       </c>
     </row>
@@ -16899,7 +16899,7 @@
         </is>
       </c>
       <c r="AA146" s="4" t="n">
-        <v>79.3</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="AB146" s="4" t="inlineStr">
         <is>
@@ -16913,7 +16913,7 @@
       </c>
       <c r="AD146" s="4" t="inlineStr">
         <is>
-          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía deficiente (nitidez 0,89; textil de 2270 px de lado); colores identificables (probabilidad 1,00; 4 colores claramente distintos, 3 tonos, colorido 65); formas visibles (probabilidad 0,99; bordes cromáticos en el 62 % del textil); textil completo (probabilidad 0,92; compacidad 0,96, lagunas 0,1 %); estructura repetitiva y simétrica. Puntaje 79.</t>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía deficiente (nitidez 0,89; textil de 2270 px de lado); colores identificables (probabilidad 1,00; 4 colores claramente distintos, 3 tonos, colorido 65); formas visibles (probabilidad 0,99; bordes cromáticos en el 62 % del textil); textil completo (probabilidad 0,96; compacidad 0,96, lagunas 0,1 %); estructura repetitiva y simétrica. Puntaje 96.</t>
         </is>
       </c>
     </row>
@@ -17021,7 +17021,7 @@
         </is>
       </c>
       <c r="AA147" s="4" t="n">
-        <v>52.6</v>
+        <v>82.8</v>
       </c>
       <c r="AB147" s="4" t="inlineStr">
         <is>
@@ -17035,7 +17035,7 @@
       </c>
       <c r="AD147" s="4" t="inlineStr">
         <is>
-          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía deficiente (nitidez 0,89; textil de 3181 px de lado); colores identificables (probabilidad 0,77; 5 colores claramente distintos, 2 tonos, colorido 39); formas parcialmente visibles (probabilidad 0,65; bordes cromáticos en el 21 % del textil); textil incompleto (probabilidad 0,37; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 53.</t>
+          <t>Fecha de inicio posterior a 1532: el estudio abarca textiles incas y anteriores. Fotografía deficiente (nitidez 0,89; textil de 3181 px de lado); colores identificables (probabilidad 0,91; 5 colores claramente distintos, 2 tonos, colorido 39); formas visibles (probabilidad 0,89; bordes cromáticos en el 21 % del textil); textil completo (probabilidad 0,77; toma cerrada, el contorno de la pieza no se ve); estructura no evidente. Puntaje 83.</t>
         </is>
       </c>
     </row>

</xml_diff>